<commit_message>
SmartDoc 2.0 tracker + checkpoint: P0 done, P1 verified (tokens, primitives, sign-in screens, shell)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/SMARTDOC_2_0_MASTER_TRACKER.xlsx
+++ b/docs/SMARTDOC_2_0_MASTER_TRACKER.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\speed\Desktop\Claude - ПРОЕКТ\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5B0B8E3-4634-4433-A6B2-E2007B42E1E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBCD3504-1791-4710-8804-3282960E9414}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,12 +22,12 @@
     <sheet name="Release Readiness" sheetId="7" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Bugs!$A$1:$H$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Bugs!$A$1:$H$5</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Decisions!$A$1:$F$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Release Readiness'!$A$1:$E$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Roadmap!$A$1:$F$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Tasks!$A$1:$P$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Tests!$A$1:$G$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Tests!$A$1:$G$9</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="440" uniqueCount="272">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="318">
   <si>
     <t>SmartDoc 2.0 -- master tracker</t>
   </si>
@@ -310,6 +310,18 @@
     <t>Branch on origin; a READY preview of it</t>
   </si>
   <si>
+    <t>937d11a</t>
+  </si>
+  <si>
+    <t>dpl_Bb5PUC2q963bMZmhGaz3bfb44Rb6 (READY); branch alias smartdoc-git-feature-smartdoc-20-drajeto.vercel.app</t>
+  </si>
+  <si>
+    <t>Preview READY</t>
+  </si>
+  <si>
+    <t>Branch alias always serves the newest preview of feature/smartdoc-2.0 (behind Vercel Authentication)</t>
+  </si>
+  <si>
     <t>S2-003</t>
   </si>
   <si>
@@ -322,6 +334,9 @@
     <t>Files committed; next session can resume from them</t>
   </si>
   <si>
+    <t>n/a (docs)</t>
+  </si>
+  <si>
     <t>S2-004</t>
   </si>
   <si>
@@ -334,6 +349,12 @@
     <t>xlsx builds and recalculates with 0 formula errors</t>
   </si>
   <si>
+    <t>Builder + Excel recalc: 19 formulas, 0 errors; summary values checked</t>
+  </si>
+  <si>
+    <t>tools/tracker/excel_recalc.py now recalculates any workbook; 1.x value checks only on the 1.x tracker</t>
+  </si>
+  <si>
     <t>S2-010</t>
   </si>
   <si>
@@ -349,6 +370,15 @@
     <t>Tokens used by the new primitives; build passes; Cyrillic renders in Inter</t>
   </si>
   <si>
+    <t>eb69d40</t>
+  </si>
+  <si>
+    <t>dpl_4KbNxArvRLBNuJARviMwh5Mj8bys (READY)</t>
+  </si>
+  <si>
+    <t>tsc, eslint, next build; Playwright visual spec unchanged (editor fonts untouched); Cyrillic seen in Inter locally</t>
+  </si>
+  <si>
     <t>S2-011</t>
   </si>
   <si>
@@ -361,6 +391,9 @@
     <t>Unit tests for states and accessibility (labels, aria-invalid, focus)</t>
   </si>
   <si>
+    <t>ui.test.tsx 7 passed; Vitest 374</t>
+  </si>
+  <si>
     <t>S2-012</t>
   </si>
   <si>
@@ -376,6 +409,12 @@
     <t>Existing AuthForm tests and Playwright auth specs pass; seen in the browser on a throwaway local server; preview builds</t>
   </si>
   <si>
+    <t>Playwright auth/visual/CSP/documents 17 passed; local browser: sign in, create account, wrong-password message, 375 px</t>
+  </si>
+  <si>
+    <t>Also forgot/reset password and address confirmation pages on the same layout. Owner's look at the preview pending.</t>
+  </si>
+  <si>
     <t>S2-013</t>
   </si>
   <si>
@@ -388,6 +427,18 @@
     <t>All signed-in pages render inside it; keyboard navigation; 375 px works</t>
   </si>
   <si>
+    <t>1003d53</t>
+  </si>
+  <si>
+    <t>pending build</t>
+  </si>
+  <si>
+    <t>AppShell.test.tsx 4; Vitest 378; Playwright full 57 + accessibility/auth 11 after fixes; local browser 1280 px and 375 px (drawer, Escape, no horizontal overflow)</t>
+  </si>
+  <si>
+    <t>Editor, compare, create wizard and public page keep AppHeader (restyled) until their own milestones</t>
+  </si>
+  <si>
     <t>S2-014</t>
   </si>
   <si>
@@ -553,6 +604,45 @@
     <t>Not fixable retroactively; owner decided to keep the data (REL-020)</t>
   </si>
   <si>
+    <t>B-003</t>
+  </si>
+  <si>
+    <t>Phone width, open the menu drawer</t>
+  </si>
+  <si>
+    <t>Logo mark in its blue-purple gradient</t>
+  </si>
+  <si>
+    <t>Mark colourless: every logo copy used the same SVG gradient id; the first copy (hidden sidebar) defined it</t>
+  </si>
+  <si>
+    <t>1003d53 (gradient in CSS)</t>
+  </si>
+  <si>
+    <t>Seen in the local browser after reload</t>
+  </si>
+  <si>
+    <t>B-004</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>Open Projects, Templates or Plan and billing inside the new shell; run axe</t>
+  </si>
+  <si>
+    <t>No serious violations</t>
+  </si>
+  <si>
+    <t>Grey zinc-500 text under 4.5:1 on the shell background</t>
+  </si>
+  <si>
+    <t>1003d53 (text-muted token)</t>
+  </si>
+  <si>
+    <t>Playwright accessibility spec passes</t>
+  </si>
+  <si>
     <t>Test ID</t>
   </si>
   <si>
@@ -640,6 +730,54 @@
     <t>Owner's browser test + Supabase storage logs</t>
   </si>
   <si>
+    <t>T-005</t>
+  </si>
+  <si>
+    <t>Vitest full</t>
+  </si>
+  <si>
+    <t>PASS 378</t>
+  </si>
+  <si>
+    <t>T-006</t>
+  </si>
+  <si>
+    <t>Playwright full (Chromium, production build)</t>
+  </si>
+  <si>
+    <t>57 passed, 2 failed -&gt; fixed; accessibility + auth 11 passed</t>
+  </si>
+  <si>
+    <t>T-007</t>
+  </si>
+  <si>
+    <t>Sign in / create account / error / 375 px; shell 1280 + 375 px, drawer</t>
+  </si>
+  <si>
+    <t>Local throwaway servers</t>
+  </si>
+  <si>
+    <t>Browser pane screenshots</t>
+  </si>
+  <si>
+    <t>T-008</t>
+  </si>
+  <si>
+    <t>Deploy</t>
+  </si>
+  <si>
+    <t>2.0 preview builds</t>
+  </si>
+  <si>
+    <t>Vercel Preview</t>
+  </si>
+  <si>
+    <t>READY: 937d11a, eb69d40</t>
+  </si>
+  <si>
+    <t>dpl_Bb5P..., dpl_4KbN...</t>
+  </si>
+  <si>
     <t>Decision ID</t>
   </si>
   <si>
@@ -856,7 +994,7 @@
     <t>SmartDoc 2.0 release</t>
   </si>
   <si>
-    <t>Phase 0</t>
+    <t>P1 done (design system, sign-in screens, shell); P2 in progress</t>
   </si>
   <si>
     <t>Not started</t>
@@ -1493,11 +1631,11 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIF(Tasks!$G$2:$G$16,A5)</f>
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C5" s="5">
         <f>COUNTIF(Roadmap!$D$2:$D$10,A5)</f>
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -1506,11 +1644,11 @@
       </c>
       <c r="B6" s="5">
         <f>COUNTIF(Tasks!$G$2:$G$16,A6)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C6" s="5">
         <f>COUNTIF(Roadmap!$D$2:$D$10,A6)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -1519,7 +1657,7 @@
       </c>
       <c r="B7" s="5">
         <f>COUNTIF(Tasks!$G$2:$G$16,A7)</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C7" s="5">
         <f>COUNTIF(Roadmap!$D$2:$D$10,A7)</f>
@@ -1558,11 +1696,11 @@
       </c>
       <c r="B10" s="5">
         <f>COUNTIF(Tasks!$G$2:$G$16,A10)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="C10" s="5">
         <f>COUNTIF(Roadmap!$D$2:$D$10,A10)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -1571,11 +1709,11 @@
       </c>
       <c r="B11" s="5">
         <f>COUNTIF(Tasks!$G$2:$G$16,A11)</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C11" s="5">
         <f>COUNTIF(Roadmap!$D$2:$D$10,A11)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -1597,7 +1735,7 @@
       </c>
       <c r="B13" s="14">
         <f>IFERROR((B11+B10)/B12,0)</f>
-        <v>6.6666666666666666E-2</v>
+        <v>0.53333333333333333</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -1606,7 +1744,7 @@
       </c>
       <c r="B14">
         <f>COUNTIFS(Tasks!$F$2:$F$16,"P0",Tasks!$G$2:$G$16,"&lt;&gt;DONE",Tasks!$G$2:$G$16,"&lt;&gt;VERIFIED")</f>
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -1614,7 +1752,7 @@
         <v>15</v>
       </c>
       <c r="B15">
-        <f>COUNTA(Bugs!$A$2:$A$3)-COUNTIF(Bugs!$F$2:$F$3,"DONE")-COUNTIF(Bugs!$F$2:$F$3,"VERIFIED")</f>
+        <f>COUNTA(Bugs!$A$2:$A$5)-COUNTIF(Bugs!$F$2:$F$5,"DONE")-COUNTIF(Bugs!$F$2:$F$5,"VERIFIED")</f>
         <v>2</v>
       </c>
     </row>
@@ -1660,7 +1798,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
         <v>22</v>
       </c>
@@ -1671,7 +1809,7 @@
         <v>24</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="E2" s="17"/>
       <c r="F2" s="17" t="s">
@@ -1689,7 +1827,7 @@
         <v>28</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E3" s="17" t="s">
         <v>22</v>
@@ -1698,7 +1836,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
         <v>30</v>
       </c>
@@ -1709,7 +1847,7 @@
         <v>32</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E4" s="17" t="s">
         <v>26</v>
@@ -1983,7 +2121,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
         <v>83</v>
       </c>
@@ -2003,7 +2141,7 @@
         <v>22</v>
       </c>
       <c r="G3" s="17" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="H3" s="17" t="s">
         <v>73</v>
@@ -2017,17 +2155,25 @@
       <c r="K3" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="L3" s="17"/>
-      <c r="M3" s="17"/>
-      <c r="N3" s="17"/>
+      <c r="L3" s="17" t="s">
+        <v>87</v>
+      </c>
+      <c r="M3" s="17" t="s">
+        <v>88</v>
+      </c>
+      <c r="N3" s="17" t="s">
+        <v>89</v>
+      </c>
       <c r="O3" s="17" t="s">
         <v>81</v>
       </c>
-      <c r="P3" s="17"/>
+      <c r="P3" s="17" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="4" spans="1:16" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B4" s="17" t="s">
         <v>22</v>
@@ -2036,22 +2182,22 @@
         <v>74</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="F4" s="17" t="s">
         <v>22</v>
       </c>
       <c r="G4" s="17" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="H4" s="17" t="s">
         <v>73</v>
       </c>
       <c r="I4" s="17" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="J4" s="17" t="s">
         <v>78</v>
@@ -2059,17 +2205,21 @@
       <c r="K4" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="L4" s="17"/>
+      <c r="L4" s="17" t="s">
+        <v>87</v>
+      </c>
       <c r="M4" s="17"/>
-      <c r="N4" s="17"/>
+      <c r="N4" s="17" t="s">
+        <v>95</v>
+      </c>
       <c r="O4" s="17" t="s">
         <v>81</v>
       </c>
       <c r="P4" s="17"/>
     </row>
-    <row r="5" spans="1:16" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="B5" s="17" t="s">
         <v>22</v>
@@ -2078,20 +2228,20 @@
         <v>74</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="F5" s="17" t="s">
         <v>22</v>
       </c>
       <c r="G5" s="17" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="H5" s="17"/>
       <c r="I5" s="17" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="J5" s="17" t="s">
         <v>78</v>
@@ -2099,41 +2249,47 @@
       <c r="K5" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="L5" s="17"/>
+      <c r="L5" s="17" t="s">
+        <v>87</v>
+      </c>
       <c r="M5" s="17"/>
-      <c r="N5" s="17"/>
+      <c r="N5" s="17" t="s">
+        <v>100</v>
+      </c>
       <c r="O5" s="17" t="s">
         <v>81</v>
       </c>
-      <c r="P5" s="17"/>
-    </row>
-    <row r="6" spans="1:16" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="P5" s="17" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="B6" s="17" t="s">
         <v>26</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="F6" s="17" t="s">
         <v>22</v>
       </c>
       <c r="G6" s="17" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="H6" s="17" t="s">
         <v>83</v>
       </c>
       <c r="I6" s="17" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="J6" s="17" t="s">
         <v>78</v>
@@ -2141,9 +2297,15 @@
       <c r="K6" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="L6" s="17"/>
-      <c r="M6" s="17"/>
-      <c r="N6" s="17"/>
+      <c r="L6" s="17" t="s">
+        <v>107</v>
+      </c>
+      <c r="M6" s="17" t="s">
+        <v>108</v>
+      </c>
+      <c r="N6" s="17" t="s">
+        <v>109</v>
+      </c>
       <c r="O6" s="17" t="s">
         <v>81</v>
       </c>
@@ -2151,31 +2313,31 @@
     </row>
     <row r="7" spans="1:16" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="B7" s="17" t="s">
         <v>26</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="F7" s="17" t="s">
         <v>22</v>
       </c>
       <c r="G7" s="17" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="H7" s="17" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="I7" s="17" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="J7" s="17" t="s">
         <v>78</v>
@@ -2183,41 +2345,47 @@
       <c r="K7" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="L7" s="17"/>
-      <c r="M7" s="17"/>
-      <c r="N7" s="17"/>
+      <c r="L7" s="17" t="s">
+        <v>107</v>
+      </c>
+      <c r="M7" s="17" t="s">
+        <v>108</v>
+      </c>
+      <c r="N7" s="17" t="s">
+        <v>114</v>
+      </c>
       <c r="O7" s="17" t="s">
         <v>81</v>
       </c>
       <c r="P7" s="17"/>
     </row>
-    <row r="8" spans="1:16" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
-        <v>104</v>
+        <v>115</v>
       </c>
       <c r="B8" s="17" t="s">
         <v>30</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>105</v>
+        <v>116</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>107</v>
+        <v>118</v>
       </c>
       <c r="F8" s="17" t="s">
         <v>22</v>
       </c>
       <c r="G8" s="17" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="H8" s="17" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="I8" s="17" t="s">
-        <v>108</v>
+        <v>119</v>
       </c>
       <c r="J8" s="17" t="s">
         <v>78</v>
@@ -2225,41 +2393,49 @@
       <c r="K8" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="L8" s="17"/>
-      <c r="M8" s="17"/>
-      <c r="N8" s="17"/>
+      <c r="L8" s="17" t="s">
+        <v>107</v>
+      </c>
+      <c r="M8" s="17" t="s">
+        <v>108</v>
+      </c>
+      <c r="N8" s="17" t="s">
+        <v>120</v>
+      </c>
       <c r="O8" s="17" t="s">
         <v>81</v>
       </c>
-      <c r="P8" s="17"/>
-    </row>
-    <row r="9" spans="1:16" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="P8" s="17" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
       <c r="B9" s="17" t="s">
         <v>26</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>110</v>
+        <v>123</v>
       </c>
       <c r="E9" s="17" t="s">
-        <v>111</v>
+        <v>124</v>
       </c>
       <c r="F9" s="17" t="s">
         <v>26</v>
       </c>
       <c r="G9" s="17" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H9" s="17" t="s">
-        <v>100</v>
+        <v>110</v>
       </c>
       <c r="I9" s="17" t="s">
-        <v>112</v>
+        <v>125</v>
       </c>
       <c r="J9" s="17" t="s">
         <v>78</v>
@@ -2267,41 +2443,49 @@
       <c r="K9" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="L9" s="17"/>
-      <c r="M9" s="17"/>
-      <c r="N9" s="17"/>
+      <c r="L9" s="17" t="s">
+        <v>126</v>
+      </c>
+      <c r="M9" s="17" t="s">
+        <v>127</v>
+      </c>
+      <c r="N9" s="17" t="s">
+        <v>128</v>
+      </c>
       <c r="O9" s="17" t="s">
         <v>81</v>
       </c>
-      <c r="P9" s="17"/>
+      <c r="P9" s="17" t="s">
+        <v>129</v>
+      </c>
     </row>
     <row r="10" spans="1:16" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A10" s="17" t="s">
-        <v>113</v>
+        <v>130</v>
       </c>
       <c r="B10" s="17" t="s">
         <v>30</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>105</v>
+        <v>116</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>114</v>
+        <v>131</v>
       </c>
       <c r="E10" s="17" t="s">
-        <v>115</v>
+        <v>132</v>
       </c>
       <c r="F10" s="17" t="s">
         <v>26</v>
       </c>
       <c r="G10" s="17" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H10" s="17" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
       <c r="I10" s="17" t="s">
-        <v>116</v>
+        <v>133</v>
       </c>
       <c r="J10" s="17" t="s">
         <v>78</v>
@@ -2319,31 +2503,31 @@
     </row>
     <row r="11" spans="1:16" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A11" s="17" t="s">
-        <v>117</v>
+        <v>134</v>
       </c>
       <c r="B11" s="17" t="s">
         <v>30</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>105</v>
+        <v>116</v>
       </c>
       <c r="D11" s="17" t="s">
-        <v>118</v>
+        <v>135</v>
       </c>
       <c r="E11" s="17" t="s">
-        <v>119</v>
+        <v>136</v>
       </c>
       <c r="F11" s="17" t="s">
         <v>26</v>
       </c>
       <c r="G11" s="17" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H11" s="17" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
       <c r="I11" s="17" t="s">
-        <v>120</v>
+        <v>137</v>
       </c>
       <c r="J11" s="17" t="s">
         <v>78</v>
@@ -2361,19 +2545,19 @@
     </row>
     <row r="12" spans="1:16" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
-        <v>121</v>
+        <v>138</v>
       </c>
       <c r="B12" s="17" t="s">
         <v>34</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>105</v>
+        <v>116</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>122</v>
+        <v>139</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>123</v>
+        <v>140</v>
       </c>
       <c r="F12" s="17" t="s">
         <v>26</v>
@@ -2382,10 +2566,10 @@
         <v>5</v>
       </c>
       <c r="H12" s="17" t="s">
-        <v>117</v>
+        <v>134</v>
       </c>
       <c r="I12" s="17" t="s">
-        <v>124</v>
+        <v>141</v>
       </c>
       <c r="J12" s="17" t="s">
         <v>78</v>
@@ -2400,24 +2584,24 @@
         <v>81</v>
       </c>
       <c r="P12" s="17" t="s">
-        <v>125</v>
+        <v>142</v>
       </c>
     </row>
     <row r="13" spans="1:16" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A13" s="17" t="s">
-        <v>126</v>
+        <v>143</v>
       </c>
       <c r="B13" s="17" t="s">
         <v>38</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>127</v>
+        <v>144</v>
       </c>
       <c r="D13" s="17" t="s">
-        <v>128</v>
+        <v>145</v>
       </c>
       <c r="E13" s="17" t="s">
-        <v>129</v>
+        <v>146</v>
       </c>
       <c r="F13" s="17" t="s">
         <v>26</v>
@@ -2426,10 +2610,10 @@
         <v>5</v>
       </c>
       <c r="H13" s="17" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
       <c r="I13" s="17" t="s">
-        <v>130</v>
+        <v>147</v>
       </c>
       <c r="J13" s="17" t="s">
         <v>78</v>
@@ -2447,19 +2631,19 @@
     </row>
     <row r="14" spans="1:16" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
-        <v>131</v>
+        <v>148</v>
       </c>
       <c r="B14" s="17" t="s">
         <v>42</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>127</v>
+        <v>144</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>132</v>
+        <v>149</v>
       </c>
       <c r="E14" s="17" t="s">
-        <v>133</v>
+        <v>150</v>
       </c>
       <c r="F14" s="17" t="s">
         <v>26</v>
@@ -2468,10 +2652,10 @@
         <v>5</v>
       </c>
       <c r="H14" s="17" t="s">
-        <v>126</v>
+        <v>143</v>
       </c>
       <c r="I14" s="17" t="s">
-        <v>134</v>
+        <v>151</v>
       </c>
       <c r="J14" s="17" t="s">
         <v>78</v>
@@ -2486,24 +2670,24 @@
         <v>81</v>
       </c>
       <c r="P14" s="17" t="s">
-        <v>135</v>
+        <v>152</v>
       </c>
     </row>
     <row r="15" spans="1:16" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A15" s="17" t="s">
-        <v>136</v>
+        <v>153</v>
       </c>
       <c r="B15" s="17" t="s">
         <v>46</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>137</v>
+        <v>154</v>
       </c>
       <c r="D15" s="17" t="s">
-        <v>138</v>
+        <v>155</v>
       </c>
       <c r="E15" s="17" t="s">
-        <v>139</v>
+        <v>156</v>
       </c>
       <c r="F15" s="17" t="s">
         <v>26</v>
@@ -2512,10 +2696,10 @@
         <v>5</v>
       </c>
       <c r="H15" s="17" t="s">
-        <v>126</v>
+        <v>143</v>
       </c>
       <c r="I15" s="17" t="s">
-        <v>140</v>
+        <v>157</v>
       </c>
       <c r="J15" s="17" t="s">
         <v>78</v>
@@ -2530,24 +2714,24 @@
         <v>81</v>
       </c>
       <c r="P15" s="17" t="s">
-        <v>141</v>
+        <v>158</v>
       </c>
     </row>
     <row r="16" spans="1:16" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A16" s="17" t="s">
-        <v>142</v>
+        <v>159</v>
       </c>
       <c r="B16" s="17" t="s">
         <v>51</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>143</v>
+        <v>160</v>
       </c>
       <c r="D16" s="17" t="s">
-        <v>144</v>
+        <v>161</v>
       </c>
       <c r="E16" s="17" t="s">
-        <v>145</v>
+        <v>162</v>
       </c>
       <c r="F16" s="17" t="s">
         <v>26</v>
@@ -2556,10 +2740,10 @@
         <v>5</v>
       </c>
       <c r="H16" s="17" t="s">
-        <v>126</v>
+        <v>143</v>
       </c>
       <c r="I16" s="17" t="s">
-        <v>146</v>
+        <v>163</v>
       </c>
       <c r="J16" s="17" t="s">
         <v>78</v>
@@ -2574,7 +2758,7 @@
         <v>81</v>
       </c>
       <c r="P16" s="17" t="s">
-        <v>147</v>
+        <v>164</v>
       </c>
     </row>
   </sheetData>
@@ -2608,7 +2792,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -2623,83 +2807,135 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>148</v>
+        <v>165</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>149</v>
+        <v>166</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>150</v>
+        <v>167</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>151</v>
+        <v>168</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>152</v>
+        <v>169</v>
       </c>
       <c r="F1" s="16" t="s">
         <v>2</v>
       </c>
       <c r="G1" s="16" t="s">
-        <v>153</v>
+        <v>170</v>
       </c>
       <c r="H1" s="16" t="s">
-        <v>154</v>
+        <v>171</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
-        <v>155</v>
+        <v>172</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>156</v>
+        <v>173</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>157</v>
+        <v>174</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>158</v>
+        <v>175</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>159</v>
+        <v>176</v>
       </c>
       <c r="F2" s="17" t="s">
         <v>8</v>
       </c>
       <c r="G2" s="17" t="s">
-        <v>160</v>
+        <v>177</v>
       </c>
       <c r="H2" s="17" t="s">
-        <v>161</v>
+        <v>178</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
-        <v>162</v>
+        <v>179</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>163</v>
+        <v>180</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>164</v>
+        <v>181</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>165</v>
+        <v>182</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>166</v>
+        <v>183</v>
       </c>
       <c r="F3" s="17" t="s">
         <v>5</v>
       </c>
       <c r="G3" s="17"/>
       <c r="H3" s="17" t="s">
-        <v>167</v>
+        <v>184</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A4" s="17" t="s">
+        <v>185</v>
+      </c>
+      <c r="B4" s="17" t="s">
+        <v>180</v>
+      </c>
+      <c r="C4" s="17" t="s">
+        <v>186</v>
+      </c>
+      <c r="D4" s="17" t="s">
+        <v>187</v>
+      </c>
+      <c r="E4" s="17" t="s">
+        <v>188</v>
+      </c>
+      <c r="F4" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="G4" s="17" t="s">
+        <v>189</v>
+      </c>
+      <c r="H4" s="17" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A5" s="17" t="s">
+        <v>191</v>
+      </c>
+      <c r="B5" s="17" t="s">
+        <v>192</v>
+      </c>
+      <c r="C5" s="17" t="s">
+        <v>193</v>
+      </c>
+      <c r="D5" s="17" t="s">
+        <v>194</v>
+      </c>
+      <c r="E5" s="17" t="s">
+        <v>195</v>
+      </c>
+      <c r="F5" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="G5" s="17" t="s">
+        <v>196</v>
+      </c>
+      <c r="H5" s="17" t="s">
+        <v>197</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H3" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
-  <conditionalFormatting sqref="F2:F3">
+  <autoFilter ref="A1:H5" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
+  <conditionalFormatting sqref="F2:F5">
     <cfRule type="expression" dxfId="6" priority="1">
       <formula>$F2="BACKLOG"</formula>
     </cfRule>
@@ -2728,7 +2964,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -2742,45 +2978,45 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>168</v>
+        <v>198</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>169</v>
+        <v>199</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>170</v>
+        <v>200</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>171</v>
+        <v>201</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>172</v>
+        <v>202</v>
       </c>
       <c r="F1" s="16" t="s">
-        <v>173</v>
+        <v>203</v>
       </c>
       <c r="G1" s="16" t="s">
-        <v>174</v>
+        <v>204</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
-        <v>175</v>
+        <v>205</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>176</v>
+        <v>206</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>177</v>
+        <v>207</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>178</v>
+        <v>208</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>179</v>
+        <v>209</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>180</v>
+        <v>210</v>
       </c>
       <c r="G2" s="17" t="s">
         <v>81</v>
@@ -2788,22 +3024,22 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
-        <v>181</v>
+        <v>211</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>182</v>
+        <v>212</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>183</v>
+        <v>213</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>178</v>
+        <v>208</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>184</v>
+        <v>214</v>
       </c>
       <c r="F3" s="17" t="s">
-        <v>185</v>
+        <v>215</v>
       </c>
       <c r="G3" s="17" t="s">
         <v>81</v>
@@ -2811,22 +3047,22 @@
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>186</v>
+        <v>216</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>187</v>
+        <v>217</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>188</v>
+        <v>218</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>178</v>
+        <v>208</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>189</v>
+        <v>219</v>
       </c>
       <c r="F4" s="17" t="s">
-        <v>190</v>
+        <v>220</v>
       </c>
       <c r="G4" s="17" t="s">
         <v>81</v>
@@ -2834,29 +3070,121 @@
     </row>
     <row r="5" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>191</v>
+        <v>221</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>192</v>
+        <v>222</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>193</v>
+        <v>223</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>194</v>
+        <v>224</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>195</v>
+        <v>225</v>
       </c>
       <c r="F5" s="17" t="s">
-        <v>196</v>
+        <v>226</v>
       </c>
       <c r="G5" s="17" t="s">
         <v>81</v>
       </c>
     </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="17" t="s">
+        <v>227</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>212</v>
+      </c>
+      <c r="C6" s="17" t="s">
+        <v>228</v>
+      </c>
+      <c r="D6" s="17" t="s">
+        <v>208</v>
+      </c>
+      <c r="E6" s="17" t="s">
+        <v>229</v>
+      </c>
+      <c r="F6" s="17" t="s">
+        <v>126</v>
+      </c>
+      <c r="G6" s="17" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A7" s="17" t="s">
+        <v>230</v>
+      </c>
+      <c r="B7" s="17" t="s">
+        <v>217</v>
+      </c>
+      <c r="C7" s="17" t="s">
+        <v>231</v>
+      </c>
+      <c r="D7" s="17" t="s">
+        <v>208</v>
+      </c>
+      <c r="E7" s="17" t="s">
+        <v>232</v>
+      </c>
+      <c r="F7" s="17" t="s">
+        <v>126</v>
+      </c>
+      <c r="G7" s="17" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A8" s="17" t="s">
+        <v>233</v>
+      </c>
+      <c r="B8" s="17" t="s">
+        <v>116</v>
+      </c>
+      <c r="C8" s="17" t="s">
+        <v>234</v>
+      </c>
+      <c r="D8" s="17" t="s">
+        <v>235</v>
+      </c>
+      <c r="E8" s="17" t="s">
+        <v>225</v>
+      </c>
+      <c r="F8" s="17" t="s">
+        <v>236</v>
+      </c>
+      <c r="G8" s="17" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A9" s="17" t="s">
+        <v>237</v>
+      </c>
+      <c r="B9" s="17" t="s">
+        <v>238</v>
+      </c>
+      <c r="C9" s="17" t="s">
+        <v>239</v>
+      </c>
+      <c r="D9" s="17" t="s">
+        <v>240</v>
+      </c>
+      <c r="E9" s="17" t="s">
+        <v>241</v>
+      </c>
+      <c r="F9" s="17" t="s">
+        <v>242</v>
+      </c>
+      <c r="G9" s="17" t="s">
+        <v>81</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G5" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
+  <autoFilter ref="A1:G9" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2875,39 +3203,39 @@
   <sheetData>
     <row r="1" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>197</v>
+        <v>243</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>198</v>
+        <v>244</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>199</v>
+        <v>245</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>174</v>
+        <v>204</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>200</v>
+        <v>246</v>
       </c>
       <c r="F1" s="16" t="s">
-        <v>201</v>
+        <v>247</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
-        <v>202</v>
+        <v>248</v>
       </c>
       <c r="B2" s="17" t="s">
         <v>67</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>203</v>
+        <v>249</v>
       </c>
       <c r="D2" s="17" t="s">
         <v>81</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>204</v>
+        <v>250</v>
       </c>
       <c r="F2" s="17" t="s">
         <v>83</v>
@@ -2915,19 +3243,19 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
-        <v>205</v>
+        <v>251</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>206</v>
+        <v>252</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>207</v>
+        <v>253</v>
       </c>
       <c r="D3" s="17" t="s">
         <v>81</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>208</v>
+        <v>254</v>
       </c>
       <c r="F3" s="17" t="s">
         <v>83</v>
@@ -2935,53 +3263,53 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>209</v>
+        <v>255</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>210</v>
+        <v>256</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>211</v>
+        <v>257</v>
       </c>
       <c r="D4" s="17" t="s">
         <v>81</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>212</v>
+        <v>258</v>
       </c>
       <c r="F4" s="17" t="s">
-        <v>213</v>
+        <v>259</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>214</v>
+        <v>260</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>215</v>
+        <v>261</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>216</v>
+        <v>262</v>
       </c>
       <c r="D5" s="17" t="s">
         <v>81</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>217</v>
+        <v>263</v>
       </c>
       <c r="F5" s="17" t="s">
-        <v>131</v>
+        <v>148</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
-        <v>218</v>
+        <v>264</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>219</v>
+        <v>265</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>220</v>
+        <v>266</v>
       </c>
       <c r="D6" s="17" t="s">
         <v>81</v>
@@ -2990,78 +3318,78 @@
         <v>26</v>
       </c>
       <c r="F6" s="17" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
-        <v>221</v>
+        <v>267</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>222</v>
+        <v>268</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>223</v>
+        <v>269</v>
       </c>
       <c r="D7" s="17" t="s">
         <v>81</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>224</v>
+        <v>270</v>
       </c>
       <c r="F7" s="17" t="s">
-        <v>131</v>
+        <v>148</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
-        <v>225</v>
+        <v>271</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>226</v>
+        <v>272</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>227</v>
+        <v>273</v>
       </c>
       <c r="D8" s="17" t="s">
         <v>81</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>228</v>
+        <v>274</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>229</v>
+        <v>275</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
-        <v>141</v>
+        <v>158</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>230</v>
+        <v>276</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>231</v>
+        <v>277</v>
       </c>
       <c r="D9" s="17" t="s">
         <v>81</v>
       </c>
       <c r="E9" s="17" t="s">
-        <v>228</v>
+        <v>274</v>
       </c>
       <c r="F9" s="17" t="s">
-        <v>136</v>
+        <v>153</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="17" t="s">
-        <v>232</v>
+        <v>278</v>
       </c>
       <c r="B10" s="17" t="s">
         <v>52</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>233</v>
+        <v>279</v>
       </c>
       <c r="D10" s="17" t="s">
         <v>81</v>
@@ -3070,45 +3398,45 @@
         <v>51</v>
       </c>
       <c r="F10" s="17" t="s">
-        <v>142</v>
+        <v>159</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="17" t="s">
-        <v>234</v>
+        <v>280</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>235</v>
+        <v>281</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>236</v>
+        <v>282</v>
       </c>
       <c r="D11" s="17" t="s">
         <v>81</v>
       </c>
       <c r="E11" s="17" t="s">
-        <v>237</v>
+        <v>283</v>
       </c>
       <c r="F11" s="17"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
-        <v>238</v>
+        <v>284</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>239</v>
+        <v>285</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>240</v>
+        <v>286</v>
       </c>
       <c r="D12" s="17" t="s">
         <v>81</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>241</v>
+        <v>287</v>
       </c>
       <c r="F12" s="17" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -3131,121 +3459,121 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>242</v>
+        <v>288</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>243</v>
+        <v>289</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>244</v>
+        <v>290</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>245</v>
+        <v>291</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>246</v>
+        <v>292</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
-        <v>247</v>
+        <v>293</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>248</v>
+        <v>294</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>249</v>
+        <v>295</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>250</v>
+        <v>296</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>251</v>
+        <v>297</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
-        <v>252</v>
+        <v>298</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>253</v>
+        <v>299</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>254</v>
+        <v>300</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>255</v>
+        <v>301</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>256</v>
+        <v>302</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>257</v>
+        <v>303</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>258</v>
+        <v>304</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>258</v>
+        <v>304</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>259</v>
+        <v>305</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>260</v>
+        <v>306</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>261</v>
+        <v>307</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>262</v>
+        <v>308</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>263</v>
+        <v>309</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>264</v>
+        <v>310</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>256</v>
+        <v>302</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
-        <v>265</v>
+        <v>311</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>266</v>
+        <v>312</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>266</v>
+        <v>312</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>267</v>
+        <v>313</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
-        <v>268</v>
+        <v>314</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>269</v>
+        <v>315</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>270</v>
+        <v>316</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>271</v>
+        <v>317</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>251</v>
+        <v>297</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
SmartDoc 2.0 tracker + checkpoint: P2 verified (dashboard, new project, BG/EN); D-010 decided
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/SMARTDOC_2_0_MASTER_TRACKER.xlsx
+++ b/docs/SMARTDOC_2_0_MASTER_TRACKER.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\speed\Desktop\Claude - ПРОЕКТ\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBCD3504-1791-4710-8804-3282960E9414}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C9552D2-8908-442D-B2E5-90878C50EAA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,12 +22,12 @@
     <sheet name="Release Readiness" sheetId="7" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Bugs!$A$1:$H$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Bugs!$A$1:$H$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Decisions!$A$1:$F$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Release Readiness'!$A$1:$E$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Roadmap!$A$1:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Tasks!$A$1:$P$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Tests!$A$1:$G$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Tasks!$A$1:$P$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Tests!$A$1:$G$13</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -47,12 +47,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="507" uniqueCount="318">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="361">
   <si>
     <t>SmartDoc 2.0 -- master tracker</t>
   </si>
   <si>
-    <t>Branch feature/smartdoc-2.0 · source docs/SMARTDOC_2_0_TRACKER.json · updated 2026-10-13</t>
+    <t>Branch feature/smartdoc-2.0 · source docs/SMARTDOC_2_0_TRACKER.json · updated 2026-10-14</t>
   </si>
   <si>
     <t>Status</t>
@@ -292,396 +292,486 @@
     <t>n/a (audit)</t>
   </si>
   <si>
+    <t>2026-10-14</t>
+  </si>
+  <si>
+    <t>HEAD 327e22e; production dpl_HxSobnp5... (4c8fdca); candidate dpl_322ED... (f644146) awaiting promote approval</t>
+  </si>
+  <si>
+    <t>S2-002</t>
+  </si>
+  <si>
+    <t>Create the SmartDoc 2.0 branch</t>
+  </si>
+  <si>
+    <t>feature/smartdoc-2.0 from 327e22e, pushed; Preview builds from it.</t>
+  </si>
+  <si>
+    <t>Branch on origin; a READY preview of it</t>
+  </si>
+  <si>
+    <t>937d11a</t>
+  </si>
+  <si>
+    <t>dpl_Bb5PUC2q963bMZmhGaz3bfb44Rb6 (READY); branch alias smartdoc-git-feature-smartdoc-20-drajeto.vercel.app</t>
+  </si>
+  <si>
+    <t>Preview READY</t>
+  </si>
+  <si>
+    <t>Branch alias always serves the newest preview of feature/smartdoc-2.0 (behind Vercel Authentication)</t>
+  </si>
+  <si>
+    <t>S2-003</t>
+  </si>
+  <si>
+    <t>Specification, decisions, roadmap, session state</t>
+  </si>
+  <si>
+    <t>SMARTDOC_2_0_SPEC/DECISIONS/ROADMAP/PROGRESS/SESSION_STATE.md</t>
+  </si>
+  <si>
+    <t>Files committed; next session can resume from them</t>
+  </si>
+  <si>
+    <t>n/a (docs)</t>
+  </si>
+  <si>
+    <t>S2-004</t>
+  </si>
+  <si>
+    <t>Excel master tracker and its builder</t>
+  </si>
+  <si>
+    <t>JSON source + tools/smartdoc2/build_tracker.py -&gt; formatted xlsx (filters, frozen headers, conditional formatting, summary formulas).</t>
+  </si>
+  <si>
+    <t>xlsx builds and recalculates with 0 formula errors</t>
+  </si>
+  <si>
+    <t>Builder + Excel recalc: 19 formulas, 0 errors; summary values checked</t>
+  </si>
+  <si>
+    <t>tools/tracker/excel_recalc.py now recalculates any workbook; 1.x value checks only on the 1.x tracker</t>
+  </si>
+  <si>
+    <t>S2-010</t>
+  </si>
+  <si>
+    <t>DESIGN</t>
+  </si>
+  <si>
+    <t>Design tokens and Inter font</t>
+  </si>
+  <si>
+    <t>Colour, radius, shadow, spacing tokens in globals.css @theme; Inter (Latin + Cyrillic) via next/font; light theme first.</t>
+  </si>
+  <si>
+    <t>Tokens used by the new primitives; build passes; Cyrillic renders in Inter</t>
+  </si>
+  <si>
+    <t>eb69d40</t>
+  </si>
+  <si>
+    <t>dpl_4KbNxArvRLBNuJARviMwh5Mj8bys (READY)</t>
+  </si>
+  <si>
+    <t>tsc, eslint, next build; Playwright visual spec unchanged (editor fonts untouched); Cyrillic seen in Inter locally</t>
+  </si>
+  <si>
+    <t>S2-011</t>
+  </si>
+  <si>
+    <t>UI primitives</t>
+  </si>
+  <si>
+    <t>components/ui: Button (primary/secondary/ghost/danger, sizes, loading), TextField (label, hint, error), Card, Logo, Spinner, EmptyState, ErrorState.</t>
+  </si>
+  <si>
+    <t>Unit tests for states and accessibility (labels, aria-invalid, focus)</t>
+  </si>
+  <si>
+    <t>ui.test.tsx 7 passed; Vitest 374</t>
+  </si>
+  <si>
+    <t>S2-012</t>
+  </si>
+  <si>
+    <t>UI</t>
+  </si>
+  <si>
+    <t>Login / Registration screen (screen 1)</t>
+  </si>
+  <si>
+    <t>Split layout: brand panel + form card; sign in / create account; validation and server errors; no social login, no reset promise while e-mail is off; existing auth API and session cookie unchanged.</t>
+  </si>
+  <si>
+    <t>Existing AuthForm tests and Playwright auth specs pass; seen in the browser on a throwaway local server; preview builds</t>
+  </si>
+  <si>
+    <t>Playwright auth/visual/CSP/documents 17 passed; local browser: sign in, create account, wrong-password message, 375 px</t>
+  </si>
+  <si>
+    <t>Also forgot/reset password and address confirmation pages on the same layout. Owner's look at the preview pending.</t>
+  </si>
+  <si>
+    <t>S2-013</t>
+  </si>
+  <si>
+    <t>Application shell</t>
+  </si>
+  <si>
+    <t>Top bar + left navigation (Home, Projects, Templates, Settings) + content area, responsive (drawer under md).</t>
+  </si>
+  <si>
+    <t>All signed-in pages render inside it; keyboard navigation; 375 px works</t>
+  </si>
+  <si>
+    <t>1003d53</t>
+  </si>
+  <si>
+    <t>dpl_47bxa2UQMU5Q52ceD4T2uDAWUVrn (READY, 1003d53)</t>
+  </si>
+  <si>
+    <t>AppShell.test.tsx 4; Vitest 378; Playwright full 57 + accessibility/auth 11 after fixes; local browser 1280 px and 375 px (drawer, Escape, no horizontal overflow)</t>
+  </si>
+  <si>
+    <t>Editor, compare, create wizard and public page keep AppHeader (restyled) until their own milestones</t>
+  </si>
+  <si>
+    <t>S2-014</t>
+  </si>
+  <si>
+    <t>Dashboard (screen 2)</t>
+  </si>
+  <si>
+    <t>Create Project, recent projects gallery with thumbnails, search, type/last-edited, templates and AI entry, empty/loading/error states.</t>
+  </si>
+  <si>
+    <t>Existing documents listed; search works; states tested</t>
+  </si>
+  <si>
+    <t>9ed36a6</t>
+  </si>
+  <si>
+    <t>dpl_2rXqkcjNs6Ev8c5ngf3BcFXfornz (READY, 9ed36a6)</t>
+  </si>
+  <si>
+    <t>Dashboard.test.tsx 7 (gallery, search debounce, empty/no-match/error/loading, describe -&gt; New Project, Bulgarian); e2e: empty dashboard -&gt; New Project, search by title; local browser EN/BG 1280 px</t>
+  </si>
+  <si>
+    <t>Thumbnails are a drawn page (real first-page previews: S2-018). Search uses the existing /documents?q=.</t>
+  </si>
+  <si>
+    <t>S2-015</t>
+  </si>
+  <si>
+    <t>New Project (screen 3)</t>
+  </si>
+  <si>
+    <t>Project-type chooser + 'Describe what you want to create...' input; routes Document types to Add Content, Free Design types to canvas size choice.</t>
+  </si>
+  <si>
+    <t>Each type leads somewhere real; nothing pretends to work</t>
+  </si>
+  <si>
+    <t>NewProject.test.tsx 18 (keyword suggestions EN/BG, whole-word short keys, real hrefs, canvas types disabled, description from the dashboard, Bulgarian); e2e: suggestion + Document -&gt; /new; signed-out redirect</t>
+  </si>
+  <si>
+    <t>/projects/new; types without a flow are labelled Coming soon (canvas: P5). Suggestion is a keyword match and says so (not AI).</t>
+  </si>
+  <si>
+    <t>S2-020</t>
+  </si>
+  <si>
+    <t>Add Content / Structure Review / Style screens (4-6)</t>
+  </si>
+  <si>
+    <t>Rebuild the create wizard as the approved 3-step flow on the existing import + structure + format APIs; structure review edits (rename, level, reorder, reclassify).</t>
+  </si>
+  <si>
+    <t>TXT/DOCX/PDF/paste reach the editor through review; original content preserved</t>
+  </si>
+  <si>
+    <t>Structure review editing may need a backend endpoint (additive)</t>
+  </si>
+  <si>
+    <t>S2-030</t>
+  </si>
+  <si>
+    <t>EDITOR</t>
+  </si>
+  <si>
+    <t>Editor layout v2 (screen 7, Document Mode)</t>
+  </si>
+  <si>
+    <t>Left (outline/pages/elements), center canvas, top contextual toolbar, right properties, collapsible AI panel; reuses the existing Tiptap editor modules.</t>
+  </si>
+  <si>
+    <t>Existing editor tests and Playwright editor specs pass</t>
+  </si>
+  <si>
+    <t>S2-040</t>
+  </si>
+  <si>
+    <t>Canvas document kind and model</t>
+  </si>
+  <si>
+    <t>kind=canvas in documents.data with schema_version; adapter: old documents = flow; validation on the backend.</t>
+  </si>
+  <si>
+    <t>Round-trip tests; old documents unaffected; no schema migration</t>
+  </si>
+  <si>
+    <t>D-004, D-006</t>
+  </si>
+  <si>
+    <t>S2-060</t>
+  </si>
+  <si>
+    <t>AI</t>
+  </si>
+  <si>
+    <t>AI proposal framework</t>
+  </si>
+  <si>
+    <t>Proposal = patch against a revision; preview/diff; accept -&gt; revision; reject -&gt; nothing.</t>
+  </si>
+  <si>
+    <t>Rejecting leaves the saved document byte-identical (test)</t>
+  </si>
+  <si>
+    <t>D-008</t>
+  </si>
+  <si>
+    <t>S2-070</t>
+  </si>
+  <si>
+    <t>TRANSLATION</t>
+  </si>
+  <si>
+    <t>Translate panel and review</t>
+  </si>
+  <si>
+    <t>Scope (selection/element/page/document), languages (auto-detect, BG/EN first), preview, side-by-side compare, save as new.</t>
+  </si>
+  <si>
+    <t>DOCX fidelity tests on representative documents; overflow warnings</t>
+  </si>
+  <si>
+    <t>Provider: D-007</t>
+  </si>
+  <si>
+    <t>S2-016</t>
+  </si>
+  <si>
+    <t>I18N</t>
+  </si>
+  <si>
+    <t>Bulgarian / English interface (D-010)</t>
+  </si>
+  <si>
+    <t>Typed dictionaries (en source, bg checked), cookie smartdoc_locale (1 year), first visit from Accept-Language (bg -&gt; BG, else EN), switch in Settings and on sign-in pages, &lt;html lang&gt;, Intl relative times; independent of document language and Translate.</t>
+  </si>
+  <si>
+    <t>Both languages render; choice persists across reloads; parity of keys and placeholders tested</t>
+  </si>
+  <si>
+    <t>i18n.test.tsx 19 (negotiation, cookie precedence, key/placeholder parity, switch + cookie + refresh, fallback); e2e: bg-BG browser starts in BG, switch to EN survives reload, Settings switch survives reload</t>
+  </si>
+  <si>
+    <t>Preference per browser (cookie), not per account: an account-level setting would need a schema change (D-004).</t>
+  </si>
+  <si>
+    <t>S2-017</t>
+  </si>
+  <si>
+    <t>Move the remaining 1.x screens onto the dictionaries</t>
+  </si>
+  <si>
+    <t>Editor, create wizard, templates, documents list, billing, account settings content, compare, password reset forms: their English strings into en/bg.</t>
+  </si>
+  <si>
+    <t>No hard-coded interface English left in those screens (a grep test); both languages rendered in their tests</t>
+  </si>
+  <si>
+    <t>Until then those screens show English in Bulgarian mode.</t>
+  </si>
+  <si>
+    <t>S2-018</t>
+  </si>
+  <si>
+    <t>Real project thumbnails</t>
+  </si>
+  <si>
+    <t>A small rendering of a project's first page for the gallery (generated on save or on demand, stored as an asset).</t>
+  </si>
+  <si>
+    <t>Cards show the real first page; no cost on every list request</t>
+  </si>
+  <si>
+    <t>Needs a storage decision (assets) -- additive, no schema change if kept as an asset of the document.</t>
+  </si>
+  <si>
+    <t>Bug ID</t>
+  </si>
+  <si>
+    <t>Severity</t>
+  </si>
+  <si>
+    <t>Reproduction steps</t>
+  </si>
+  <si>
+    <t>Expected result</t>
+  </si>
+  <si>
+    <t>Actual result</t>
+  </si>
+  <si>
+    <t>Fix commit</t>
+  </si>
+  <si>
+    <t>Verification</t>
+  </si>
+  <si>
+    <t>B-001</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Production (4c8fdca): upload a DOCX with a picture; wait &gt; 5 min idle; reopen</t>
+  </si>
+  <si>
+    <t>Picture shown</t>
+  </si>
+  <si>
+    <t>Production stores files on the container's disk until the promote with STORAGE_BACKEND=s3 (settings added 2026-10-13, not yet deployed)</t>
+  </si>
+  <si>
+    <t>a07ebd3 / promote of f644146</t>
+  </si>
+  <si>
+    <t>Verified on Preview (REL-005); production needs the approved promote</t>
+  </si>
+  <si>
+    <t>B-002</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Open a document created on Production before the S3 settings, with pictures</t>
+  </si>
+  <si>
+    <t>Pictures shown</t>
+  </si>
+  <si>
+    <t>Pictures were on a replaced instance's disk: missing</t>
+  </si>
+  <si>
+    <t>Not fixable retroactively; owner decided to keep the data (REL-020)</t>
+  </si>
+  <si>
+    <t>B-003</t>
+  </si>
+  <si>
+    <t>Phone width, open the menu drawer</t>
+  </si>
+  <si>
+    <t>Logo mark in its blue-purple gradient</t>
+  </si>
+  <si>
+    <t>Mark colourless: every logo copy used the same SVG gradient id; the first copy (hidden sidebar) defined it</t>
+  </si>
+  <si>
+    <t>1003d53 (gradient in CSS)</t>
+  </si>
+  <si>
+    <t>Seen in the local browser after reload</t>
+  </si>
+  <si>
+    <t>B-004</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>Open Projects, Templates or Plan and billing inside the new shell; run axe</t>
+  </si>
+  <si>
+    <t>No serious violations</t>
+  </si>
+  <si>
+    <t>Grey zinc-500 text under 4.5:1 on the shell background</t>
+  </si>
+  <si>
+    <t>1003d53 (text-muted token)</t>
+  </si>
+  <si>
+    <t>Playwright accessibility spec passes</t>
+  </si>
+  <si>
+    <t>B-005</t>
+  </si>
+  <si>
+    <t>Local (SQLite) API: create a project, look at the dashboard from Sofia (UTC+3)</t>
+  </si>
+  <si>
+    <t>Edited just now</t>
+  </si>
+  <si>
+    <t>Edited 3 hours ago: a time without a zone was read as local time</t>
+  </si>
+  <si>
+    <t>9ed36a6 (parseServerTime: no zone = UTC; also lib/format.ts)</t>
+  </si>
+  <si>
+    <t>i18n.test.tsx case; seen in the local browser</t>
+  </si>
+  <si>
+    <t>Test ID</t>
+  </si>
+  <si>
+    <t>Area</t>
+  </si>
+  <si>
+    <t>Scenario</t>
+  </si>
+  <si>
+    <t>Environment</t>
+  </si>
+  <si>
+    <t>Result</t>
+  </si>
+  <si>
+    <t>Evidence</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>T-001</t>
+  </si>
+  <si>
+    <t>Backend</t>
+  </si>
+  <si>
+    <t>Full pytest suite</t>
+  </si>
+  <si>
+    <t>Local</t>
+  </si>
+  <si>
+    <t>PASS 2599 / 11 skipped</t>
+  </si>
+  <si>
+    <t>1.x tracker RUN-0309 (b5f8142)</t>
+  </si>
+  <si>
     <t>2026-10-13</t>
   </si>
   <si>
-    <t>HEAD 327e22e; production dpl_HxSobnp5... (4c8fdca); candidate dpl_322ED... (f644146) awaiting promote approval</t>
-  </si>
-  <si>
-    <t>S2-002</t>
-  </si>
-  <si>
-    <t>Create the SmartDoc 2.0 branch</t>
-  </si>
-  <si>
-    <t>feature/smartdoc-2.0 from 327e22e, pushed; Preview builds from it.</t>
-  </si>
-  <si>
-    <t>Branch on origin; a READY preview of it</t>
-  </si>
-  <si>
-    <t>937d11a</t>
-  </si>
-  <si>
-    <t>dpl_Bb5PUC2q963bMZmhGaz3bfb44Rb6 (READY); branch alias smartdoc-git-feature-smartdoc-20-drajeto.vercel.app</t>
-  </si>
-  <si>
-    <t>Preview READY</t>
-  </si>
-  <si>
-    <t>Branch alias always serves the newest preview of feature/smartdoc-2.0 (behind Vercel Authentication)</t>
-  </si>
-  <si>
-    <t>S2-003</t>
-  </si>
-  <si>
-    <t>Specification, decisions, roadmap, session state</t>
-  </si>
-  <si>
-    <t>SMARTDOC_2_0_SPEC/DECISIONS/ROADMAP/PROGRESS/SESSION_STATE.md</t>
-  </si>
-  <si>
-    <t>Files committed; next session can resume from them</t>
-  </si>
-  <si>
-    <t>n/a (docs)</t>
-  </si>
-  <si>
-    <t>S2-004</t>
-  </si>
-  <si>
-    <t>Excel master tracker and its builder</t>
-  </si>
-  <si>
-    <t>JSON source + tools/smartdoc2/build_tracker.py -&gt; formatted xlsx (filters, frozen headers, conditional formatting, summary formulas).</t>
-  </si>
-  <si>
-    <t>xlsx builds and recalculates with 0 formula errors</t>
-  </si>
-  <si>
-    <t>Builder + Excel recalc: 19 formulas, 0 errors; summary values checked</t>
-  </si>
-  <si>
-    <t>tools/tracker/excel_recalc.py now recalculates any workbook; 1.x value checks only on the 1.x tracker</t>
-  </si>
-  <si>
-    <t>S2-010</t>
-  </si>
-  <si>
-    <t>DESIGN</t>
-  </si>
-  <si>
-    <t>Design tokens and Inter font</t>
-  </si>
-  <si>
-    <t>Colour, radius, shadow, spacing tokens in globals.css @theme; Inter (Latin + Cyrillic) via next/font; light theme first.</t>
-  </si>
-  <si>
-    <t>Tokens used by the new primitives; build passes; Cyrillic renders in Inter</t>
-  </si>
-  <si>
-    <t>eb69d40</t>
-  </si>
-  <si>
-    <t>dpl_4KbNxArvRLBNuJARviMwh5Mj8bys (READY)</t>
-  </si>
-  <si>
-    <t>tsc, eslint, next build; Playwright visual spec unchanged (editor fonts untouched); Cyrillic seen in Inter locally</t>
-  </si>
-  <si>
-    <t>S2-011</t>
-  </si>
-  <si>
-    <t>UI primitives</t>
-  </si>
-  <si>
-    <t>components/ui: Button (primary/secondary/ghost/danger, sizes, loading), TextField (label, hint, error), Card, Logo, Spinner, EmptyState, ErrorState.</t>
-  </si>
-  <si>
-    <t>Unit tests for states and accessibility (labels, aria-invalid, focus)</t>
-  </si>
-  <si>
-    <t>ui.test.tsx 7 passed; Vitest 374</t>
-  </si>
-  <si>
-    <t>S2-012</t>
-  </si>
-  <si>
-    <t>UI</t>
-  </si>
-  <si>
-    <t>Login / Registration screen (screen 1)</t>
-  </si>
-  <si>
-    <t>Split layout: brand panel + form card; sign in / create account; validation and server errors; no social login, no reset promise while e-mail is off; existing auth API and session cookie unchanged.</t>
-  </si>
-  <si>
-    <t>Existing AuthForm tests and Playwright auth specs pass; seen in the browser on a throwaway local server; preview builds</t>
-  </si>
-  <si>
-    <t>Playwright auth/visual/CSP/documents 17 passed; local browser: sign in, create account, wrong-password message, 375 px</t>
-  </si>
-  <si>
-    <t>Also forgot/reset password and address confirmation pages on the same layout. Owner's look at the preview pending.</t>
-  </si>
-  <si>
-    <t>S2-013</t>
-  </si>
-  <si>
-    <t>Application shell</t>
-  </si>
-  <si>
-    <t>Top bar + left navigation (Home, Projects, Templates, Settings) + content area, responsive (drawer under md).</t>
-  </si>
-  <si>
-    <t>All signed-in pages render inside it; keyboard navigation; 375 px works</t>
-  </si>
-  <si>
-    <t>1003d53</t>
-  </si>
-  <si>
-    <t>pending build</t>
-  </si>
-  <si>
-    <t>AppShell.test.tsx 4; Vitest 378; Playwright full 57 + accessibility/auth 11 after fixes; local browser 1280 px and 375 px (drawer, Escape, no horizontal overflow)</t>
-  </si>
-  <si>
-    <t>Editor, compare, create wizard and public page keep AppHeader (restyled) until their own milestones</t>
-  </si>
-  <si>
-    <t>S2-014</t>
-  </si>
-  <si>
-    <t>Dashboard (screen 2)</t>
-  </si>
-  <si>
-    <t>Create Project, recent projects gallery with thumbnails, search, type/last-edited, templates and AI entry, empty/loading/error states.</t>
-  </si>
-  <si>
-    <t>Existing documents listed; search works; states tested</t>
-  </si>
-  <si>
-    <t>S2-015</t>
-  </si>
-  <si>
-    <t>New Project (screen 3)</t>
-  </si>
-  <si>
-    <t>Project-type chooser + 'Describe what you want to create...' input; routes Document types to Add Content, Free Design types to canvas size choice.</t>
-  </si>
-  <si>
-    <t>Each type leads somewhere real; nothing pretends to work</t>
-  </si>
-  <si>
-    <t>S2-020</t>
-  </si>
-  <si>
-    <t>Add Content / Structure Review / Style screens (4-6)</t>
-  </si>
-  <si>
-    <t>Rebuild the create wizard as the approved 3-step flow on the existing import + structure + format APIs; structure review edits (rename, level, reorder, reclassify).</t>
-  </si>
-  <si>
-    <t>TXT/DOCX/PDF/paste reach the editor through review; original content preserved</t>
-  </si>
-  <si>
-    <t>Structure review editing may need a backend endpoint (additive)</t>
-  </si>
-  <si>
-    <t>S2-030</t>
-  </si>
-  <si>
-    <t>EDITOR</t>
-  </si>
-  <si>
-    <t>Editor layout v2 (screen 7, Document Mode)</t>
-  </si>
-  <si>
-    <t>Left (outline/pages/elements), center canvas, top contextual toolbar, right properties, collapsible AI panel; reuses the existing Tiptap editor modules.</t>
-  </si>
-  <si>
-    <t>Existing editor tests and Playwright editor specs pass</t>
-  </si>
-  <si>
-    <t>S2-040</t>
-  </si>
-  <si>
-    <t>Canvas document kind and model</t>
-  </si>
-  <si>
-    <t>kind=canvas in documents.data with schema_version; adapter: old documents = flow; validation on the backend.</t>
-  </si>
-  <si>
-    <t>Round-trip tests; old documents unaffected; no schema migration</t>
-  </si>
-  <si>
-    <t>D-004, D-006</t>
-  </si>
-  <si>
-    <t>S2-060</t>
-  </si>
-  <si>
-    <t>AI</t>
-  </si>
-  <si>
-    <t>AI proposal framework</t>
-  </si>
-  <si>
-    <t>Proposal = patch against a revision; preview/diff; accept -&gt; revision; reject -&gt; nothing.</t>
-  </si>
-  <si>
-    <t>Rejecting leaves the saved document byte-identical (test)</t>
-  </si>
-  <si>
-    <t>D-008</t>
-  </si>
-  <si>
-    <t>S2-070</t>
-  </si>
-  <si>
-    <t>TRANSLATION</t>
-  </si>
-  <si>
-    <t>Translate panel and review</t>
-  </si>
-  <si>
-    <t>Scope (selection/element/page/document), languages (auto-detect, BG/EN first), preview, side-by-side compare, save as new.</t>
-  </si>
-  <si>
-    <t>DOCX fidelity tests on representative documents; overflow warnings</t>
-  </si>
-  <si>
-    <t>Provider: D-007</t>
-  </si>
-  <si>
-    <t>Bug ID</t>
-  </si>
-  <si>
-    <t>Severity</t>
-  </si>
-  <si>
-    <t>Reproduction steps</t>
-  </si>
-  <si>
-    <t>Expected result</t>
-  </si>
-  <si>
-    <t>Actual result</t>
-  </si>
-  <si>
-    <t>Fix commit</t>
-  </si>
-  <si>
-    <t>Verification</t>
-  </si>
-  <si>
-    <t>B-001</t>
-  </si>
-  <si>
-    <t>High</t>
-  </si>
-  <si>
-    <t>Production (4c8fdca): upload a DOCX with a picture; wait &gt; 5 min idle; reopen</t>
-  </si>
-  <si>
-    <t>Picture shown</t>
-  </si>
-  <si>
-    <t>Production stores files on the container's disk until the promote with STORAGE_BACKEND=s3 (settings added 2026-10-13, not yet deployed)</t>
-  </si>
-  <si>
-    <t>a07ebd3 / promote of f644146</t>
-  </si>
-  <si>
-    <t>Verified on Preview (REL-005); production needs the approved promote</t>
-  </si>
-  <si>
-    <t>B-002</t>
-  </si>
-  <si>
-    <t>Low</t>
-  </si>
-  <si>
-    <t>Open a document created on Production before the S3 settings, with pictures</t>
-  </si>
-  <si>
-    <t>Pictures shown</t>
-  </si>
-  <si>
-    <t>Pictures were on a replaced instance's disk: missing</t>
-  </si>
-  <si>
-    <t>Not fixable retroactively; owner decided to keep the data (REL-020)</t>
-  </si>
-  <si>
-    <t>B-003</t>
-  </si>
-  <si>
-    <t>Phone width, open the menu drawer</t>
-  </si>
-  <si>
-    <t>Logo mark in its blue-purple gradient</t>
-  </si>
-  <si>
-    <t>Mark colourless: every logo copy used the same SVG gradient id; the first copy (hidden sidebar) defined it</t>
-  </si>
-  <si>
-    <t>1003d53 (gradient in CSS)</t>
-  </si>
-  <si>
-    <t>Seen in the local browser after reload</t>
-  </si>
-  <si>
-    <t>B-004</t>
-  </si>
-  <si>
-    <t>Medium</t>
-  </si>
-  <si>
-    <t>Open Projects, Templates or Plan and billing inside the new shell; run axe</t>
-  </si>
-  <si>
-    <t>No serious violations</t>
-  </si>
-  <si>
-    <t>Grey zinc-500 text under 4.5:1 on the shell background</t>
-  </si>
-  <si>
-    <t>1003d53 (text-muted token)</t>
-  </si>
-  <si>
-    <t>Playwright accessibility spec passes</t>
-  </si>
-  <si>
-    <t>Test ID</t>
-  </si>
-  <si>
-    <t>Area</t>
-  </si>
-  <si>
-    <t>Scenario</t>
-  </si>
-  <si>
-    <t>Environment</t>
-  </si>
-  <si>
-    <t>Result</t>
-  </si>
-  <si>
-    <t>Evidence</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>T-001</t>
-  </si>
-  <si>
-    <t>Backend</t>
-  </si>
-  <si>
-    <t>Full pytest suite</t>
-  </si>
-  <si>
-    <t>Local</t>
-  </si>
-  <si>
-    <t>PASS 2599 / 11 skipped</t>
-  </si>
-  <si>
-    <t>1.x tracker RUN-0309 (b5f8142)</t>
-  </si>
-  <si>
     <t>T-002</t>
   </si>
   <si>
@@ -778,6 +868,42 @@
     <t>dpl_Bb5P..., dpl_4KbN...</t>
   </si>
   <si>
+    <t>T-009</t>
+  </si>
+  <si>
+    <t>PASS 422</t>
+  </si>
+  <si>
+    <t>T-010</t>
+  </si>
+  <si>
+    <t>Playwright full incl. smartdoc2.spec.ts (5 new)</t>
+  </si>
+  <si>
+    <t>Local (production build)</t>
+  </si>
+  <si>
+    <t>PASS 64 / 1 skipped</t>
+  </si>
+  <si>
+    <t>T-011</t>
+  </si>
+  <si>
+    <t>Dashboard + New Project in English and Bulgarian, 1280 px; language switch from Settings</t>
+  </si>
+  <si>
+    <t>PASS (2 layout issues + time-zone bug found and fixed)</t>
+  </si>
+  <si>
+    <t>T-012</t>
+  </si>
+  <si>
+    <t>READY: 1003d53, 9ed36a6</t>
+  </si>
+  <si>
+    <t>dpl_47bx..., dpl_2rXq...</t>
+  </si>
+  <si>
     <t>Decision ID</t>
   </si>
   <si>
@@ -895,12 +1021,15 @@
     <t>UI language</t>
   </si>
   <si>
-    <t>OPEN: interface language (EN today) -- owner to decide</t>
+    <t>Interface in Bulgarian and English: first visit from the browser language (bg -&gt; BG, else EN); manual switch in Settings (and sign-in pages); remembered per browser (cookie, 1 year); independent of document language and Translate; centralised dictionaries; tests for both languages and persistence</t>
   </si>
   <si>
     <t>All screens</t>
   </si>
   <si>
+    <t>S2-016, S2-017</t>
+  </si>
+  <si>
     <t>D-011</t>
   </si>
   <si>
@@ -994,7 +1123,7 @@
     <t>SmartDoc 2.0 release</t>
   </si>
   <si>
-    <t>P1 done (design system, sign-in screens, shell); P2 in progress</t>
+    <t>P1 + P2 done (design system, shell, sign-in, dashboard, new project, BG/EN)</t>
   </si>
   <si>
     <t>Not started</t>
@@ -1630,12 +1759,12 @@
         <v>5</v>
       </c>
       <c r="B5" s="5">
-        <f>COUNTIF(Tasks!$G$2:$G$16,A5)</f>
-        <v>5</v>
+        <f>COUNTIF(Tasks!$G$2:$G$19,A5)</f>
+        <v>7</v>
       </c>
       <c r="C5" s="5">
         <f>COUNTIF(Roadmap!$D$2:$D$10,A5)</f>
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -1643,12 +1772,12 @@
         <v>6</v>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF(Tasks!$G$2:$G$16,A6)</f>
-        <v>2</v>
+        <f>COUNTIF(Tasks!$G$2:$G$19,A6)</f>
+        <v>0</v>
       </c>
       <c r="C6" s="5">
         <f>COUNTIF(Roadmap!$D$2:$D$10,A6)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -1656,12 +1785,12 @@
         <v>7</v>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF(Tasks!$G$2:$G$16,A7)</f>
+        <f>COUNTIF(Tasks!$G$2:$G$19,A7)</f>
         <v>0</v>
       </c>
       <c r="C7" s="5">
         <f>COUNTIF(Roadmap!$D$2:$D$10,A7)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -1669,7 +1798,7 @@
         <v>8</v>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF(Tasks!$G$2:$G$16,A8)</f>
+        <f>COUNTIF(Tasks!$G$2:$G$19,A8)</f>
         <v>0</v>
       </c>
       <c r="C8" s="5">
@@ -1682,7 +1811,7 @@
         <v>9</v>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIF(Tasks!$G$2:$G$16,A9)</f>
+        <f>COUNTIF(Tasks!$G$2:$G$19,A9)</f>
         <v>0</v>
       </c>
       <c r="C9" s="5">
@@ -1695,12 +1824,12 @@
         <v>10</v>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIF(Tasks!$G$2:$G$16,A10)</f>
-        <v>4</v>
+        <f>COUNTIF(Tasks!$G$2:$G$19,A10)</f>
+        <v>7</v>
       </c>
       <c r="C10" s="5">
         <f>COUNTIF(Roadmap!$D$2:$D$10,A10)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -1708,7 +1837,7 @@
         <v>11</v>
       </c>
       <c r="B11" s="5">
-        <f>COUNTIF(Tasks!$G$2:$G$16,A11)</f>
+        <f>COUNTIF(Tasks!$G$2:$G$19,A11)</f>
         <v>4</v>
       </c>
       <c r="C11" s="5">
@@ -1722,7 +1851,7 @@
       </c>
       <c r="B12" s="12">
         <f>SUM(B5:B11)</f>
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C12" s="12">
         <f>SUM(C5:C11)</f>
@@ -1735,7 +1864,7 @@
       </c>
       <c r="B13" s="14">
         <f>IFERROR((B11+B10)/B12,0)</f>
-        <v>0.53333333333333333</v>
+        <v>0.61111111111111116</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -1743,7 +1872,7 @@
         <v>14</v>
       </c>
       <c r="B14">
-        <f>COUNTIFS(Tasks!$F$2:$F$16,"P0",Tasks!$G$2:$G$16,"&lt;&gt;DONE",Tasks!$G$2:$G$16,"&lt;&gt;VERIFIED")</f>
+        <f>COUNTIFS(Tasks!$F$2:$F$19,"P0",Tasks!$G$2:$G$19,"&lt;&gt;DONE",Tasks!$G$2:$G$19,"&lt;&gt;VERIFIED")</f>
         <v>0</v>
       </c>
     </row>
@@ -1752,7 +1881,7 @@
         <v>15</v>
       </c>
       <c r="B15">
-        <f>COUNTA(Bugs!$A$2:$A$5)-COUNTIF(Bugs!$F$2:$F$5,"DONE")-COUNTIF(Bugs!$F$2:$F$5,"VERIFIED")</f>
+        <f>COUNTA(Bugs!$A$2:$A$6)-COUNTIF(Bugs!$F$2:$F$6,"DONE")-COUNTIF(Bugs!$F$2:$F$6,"VERIFIED")</f>
         <v>2</v>
       </c>
     </row>
@@ -1836,7 +1965,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
         <v>30</v>
       </c>
@@ -1847,7 +1976,7 @@
         <v>32</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E4" s="17" t="s">
         <v>26</v>
@@ -1867,7 +1996,7 @@
         <v>36</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E5" s="17" t="s">
         <v>30</v>
@@ -2007,7 +2136,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:P16"/>
+  <dimension ref="A1:P19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
@@ -2459,7 +2588,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="25.5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" ht="114.75" x14ac:dyDescent="0.25">
       <c r="A10" s="17" t="s">
         <v>130</v>
       </c>
@@ -2479,7 +2608,7 @@
         <v>26</v>
       </c>
       <c r="G10" s="17" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="H10" s="17" t="s">
         <v>122</v>
@@ -2493,17 +2622,25 @@
       <c r="K10" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="L10" s="17"/>
-      <c r="M10" s="17"/>
-      <c r="N10" s="17"/>
+      <c r="L10" s="17" t="s">
+        <v>134</v>
+      </c>
+      <c r="M10" s="17" t="s">
+        <v>135</v>
+      </c>
+      <c r="N10" s="17" t="s">
+        <v>136</v>
+      </c>
       <c r="O10" s="17" t="s">
         <v>81</v>
       </c>
-      <c r="P10" s="17"/>
-    </row>
-    <row r="11" spans="1:16" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="P10" s="17" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" ht="114.75" x14ac:dyDescent="0.25">
       <c r="A11" s="17" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B11" s="17" t="s">
         <v>30</v>
@@ -2512,22 +2649,22 @@
         <v>116</v>
       </c>
       <c r="D11" s="17" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="E11" s="17" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="F11" s="17" t="s">
         <v>26</v>
       </c>
       <c r="G11" s="17" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="H11" s="17" t="s">
         <v>122</v>
       </c>
       <c r="I11" s="17" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="J11" s="17" t="s">
         <v>78</v>
@@ -2535,17 +2672,25 @@
       <c r="K11" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="L11" s="17"/>
-      <c r="M11" s="17"/>
-      <c r="N11" s="17"/>
+      <c r="L11" s="17" t="s">
+        <v>134</v>
+      </c>
+      <c r="M11" s="17" t="s">
+        <v>135</v>
+      </c>
+      <c r="N11" s="17" t="s">
+        <v>142</v>
+      </c>
       <c r="O11" s="17" t="s">
         <v>81</v>
       </c>
-      <c r="P11" s="17"/>
+      <c r="P11" s="17" t="s">
+        <v>143</v>
+      </c>
     </row>
     <row r="12" spans="1:16" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="B12" s="17" t="s">
         <v>34</v>
@@ -2554,10 +2699,10 @@
         <v>116</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="F12" s="17" t="s">
         <v>26</v>
@@ -2566,10 +2711,10 @@
         <v>5</v>
       </c>
       <c r="H12" s="17" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="I12" s="17" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="J12" s="17" t="s">
         <v>78</v>
@@ -2584,24 +2729,24 @@
         <v>81</v>
       </c>
       <c r="P12" s="17" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
     </row>
     <row r="13" spans="1:16" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A13" s="17" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="B13" s="17" t="s">
         <v>38</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="D13" s="17" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="E13" s="17" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="F13" s="17" t="s">
         <v>26</v>
@@ -2613,7 +2758,7 @@
         <v>122</v>
       </c>
       <c r="I13" s="17" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="J13" s="17" t="s">
         <v>78</v>
@@ -2631,19 +2776,19 @@
     </row>
     <row r="14" spans="1:16" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="B14" s="17" t="s">
         <v>42</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="E14" s="17" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="F14" s="17" t="s">
         <v>26</v>
@@ -2652,10 +2797,10 @@
         <v>5</v>
       </c>
       <c r="H14" s="17" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="I14" s="17" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="J14" s="17" t="s">
         <v>78</v>
@@ -2670,24 +2815,24 @@
         <v>81</v>
       </c>
       <c r="P14" s="17" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
     </row>
     <row r="15" spans="1:16" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A15" s="17" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="B15" s="17" t="s">
         <v>46</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="D15" s="17" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="E15" s="17" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="F15" s="17" t="s">
         <v>26</v>
@@ -2696,10 +2841,10 @@
         <v>5</v>
       </c>
       <c r="H15" s="17" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="I15" s="17" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="J15" s="17" t="s">
         <v>78</v>
@@ -2714,24 +2859,24 @@
         <v>81</v>
       </c>
       <c r="P15" s="17" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
     </row>
     <row r="16" spans="1:16" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A16" s="17" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="B16" s="17" t="s">
         <v>51</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="D16" s="17" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="E16" s="17" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="F16" s="17" t="s">
         <v>26</v>
@@ -2740,10 +2885,10 @@
         <v>5</v>
       </c>
       <c r="H16" s="17" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="I16" s="17" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="J16" s="17" t="s">
         <v>78</v>
@@ -2758,12 +2903,150 @@
         <v>81</v>
       </c>
       <c r="P16" s="17" t="s">
-        <v>164</v>
+        <v>170</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" ht="127.5" x14ac:dyDescent="0.25">
+      <c r="A17" s="17" t="s">
+        <v>171</v>
+      </c>
+      <c r="B17" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C17" s="17" t="s">
+        <v>172</v>
+      </c>
+      <c r="D17" s="17" t="s">
+        <v>173</v>
+      </c>
+      <c r="E17" s="17" t="s">
+        <v>174</v>
+      </c>
+      <c r="F17" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="G17" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="H17" s="17" t="s">
+        <v>110</v>
+      </c>
+      <c r="I17" s="17" t="s">
+        <v>175</v>
+      </c>
+      <c r="J17" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="K17" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="L17" s="17" t="s">
+        <v>134</v>
+      </c>
+      <c r="M17" s="17" t="s">
+        <v>135</v>
+      </c>
+      <c r="N17" s="17" t="s">
+        <v>176</v>
+      </c>
+      <c r="O17" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="P17" s="17" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A18" s="17" t="s">
+        <v>178</v>
+      </c>
+      <c r="B18" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C18" s="17" t="s">
+        <v>172</v>
+      </c>
+      <c r="D18" s="17" t="s">
+        <v>179</v>
+      </c>
+      <c r="E18" s="17" t="s">
+        <v>180</v>
+      </c>
+      <c r="F18" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="G18" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="H18" s="17" t="s">
+        <v>171</v>
+      </c>
+      <c r="I18" s="17" t="s">
+        <v>181</v>
+      </c>
+      <c r="J18" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="K18" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="L18" s="17"/>
+      <c r="M18" s="17"/>
+      <c r="N18" s="17"/>
+      <c r="O18" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="P18" s="17" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A19" s="17" t="s">
+        <v>183</v>
+      </c>
+      <c r="B19" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C19" s="17" t="s">
+        <v>116</v>
+      </c>
+      <c r="D19" s="17" t="s">
+        <v>184</v>
+      </c>
+      <c r="E19" s="17" t="s">
+        <v>185</v>
+      </c>
+      <c r="F19" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="G19" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="H19" s="17" t="s">
+        <v>130</v>
+      </c>
+      <c r="I19" s="17" t="s">
+        <v>186</v>
+      </c>
+      <c r="J19" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="K19" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="L19" s="17"/>
+      <c r="M19" s="17"/>
+      <c r="N19" s="17"/>
+      <c r="O19" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="P19" s="17" t="s">
+        <v>187</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P16" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
-  <conditionalFormatting sqref="G2:G16">
+  <autoFilter ref="A1:P19" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
+  <conditionalFormatting sqref="G2:G19">
     <cfRule type="expression" dxfId="13" priority="1">
       <formula>$G2="BACKLOG"</formula>
     </cfRule>
@@ -2792,7 +3075,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -2807,135 +3090,161 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>165</v>
+        <v>188</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>166</v>
+        <v>189</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>167</v>
+        <v>190</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>168</v>
+        <v>191</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>169</v>
+        <v>192</v>
       </c>
       <c r="F1" s="16" t="s">
         <v>2</v>
       </c>
       <c r="G1" s="16" t="s">
-        <v>170</v>
+        <v>193</v>
       </c>
       <c r="H1" s="16" t="s">
-        <v>171</v>
+        <v>194</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
-        <v>172</v>
+        <v>195</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>173</v>
+        <v>196</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>174</v>
+        <v>197</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>175</v>
+        <v>198</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>176</v>
+        <v>199</v>
       </c>
       <c r="F2" s="17" t="s">
         <v>8</v>
       </c>
       <c r="G2" s="17" t="s">
-        <v>177</v>
+        <v>200</v>
       </c>
       <c r="H2" s="17" t="s">
-        <v>178</v>
+        <v>201</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
-        <v>179</v>
+        <v>202</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>180</v>
+        <v>203</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>181</v>
+        <v>204</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>182</v>
+        <v>205</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>183</v>
+        <v>206</v>
       </c>
       <c r="F3" s="17" t="s">
         <v>5</v>
       </c>
       <c r="G3" s="17"/>
       <c r="H3" s="17" t="s">
-        <v>184</v>
+        <v>207</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>185</v>
+        <v>208</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>180</v>
+        <v>203</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>186</v>
+        <v>209</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>187</v>
+        <v>210</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>188</v>
+        <v>211</v>
       </c>
       <c r="F4" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G4" s="17" t="s">
-        <v>189</v>
+        <v>212</v>
       </c>
       <c r="H4" s="17" t="s">
-        <v>190</v>
+        <v>213</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>191</v>
+        <v>214</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>192</v>
+        <v>215</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>193</v>
+        <v>216</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>194</v>
+        <v>217</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>195</v>
+        <v>218</v>
       </c>
       <c r="F5" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G5" s="17" t="s">
-        <v>196</v>
+        <v>219</v>
       </c>
       <c r="H5" s="17" t="s">
-        <v>197</v>
+        <v>220</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="51" x14ac:dyDescent="0.25">
+      <c r="A6" s="17" t="s">
+        <v>221</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>215</v>
+      </c>
+      <c r="C6" s="17" t="s">
+        <v>222</v>
+      </c>
+      <c r="D6" s="17" t="s">
+        <v>223</v>
+      </c>
+      <c r="E6" s="17" t="s">
+        <v>224</v>
+      </c>
+      <c r="F6" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="G6" s="17" t="s">
+        <v>225</v>
+      </c>
+      <c r="H6" s="17" t="s">
+        <v>226</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H5" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
-  <conditionalFormatting sqref="F2:F5">
+  <autoFilter ref="A1:H6" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
+  <conditionalFormatting sqref="F2:F6">
     <cfRule type="expression" dxfId="6" priority="1">
       <formula>$F2="BACKLOG"</formula>
     </cfRule>
@@ -2964,7 +3273,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -2978,213 +3287,305 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>198</v>
+        <v>227</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>199</v>
+        <v>228</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>200</v>
+        <v>229</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>201</v>
+        <v>230</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>202</v>
+        <v>231</v>
       </c>
       <c r="F1" s="16" t="s">
-        <v>203</v>
+        <v>232</v>
       </c>
       <c r="G1" s="16" t="s">
-        <v>204</v>
+        <v>233</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
-        <v>205</v>
+        <v>234</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>206</v>
+        <v>235</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>207</v>
+        <v>236</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>208</v>
+        <v>237</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>209</v>
+        <v>238</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>210</v>
+        <v>239</v>
       </c>
       <c r="G2" s="17" t="s">
-        <v>81</v>
+        <v>240</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
-        <v>211</v>
+        <v>241</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>212</v>
+        <v>242</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>213</v>
+        <v>243</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>208</v>
+        <v>237</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>214</v>
+        <v>244</v>
       </c>
       <c r="F3" s="17" t="s">
-        <v>215</v>
+        <v>245</v>
       </c>
       <c r="G3" s="17" t="s">
-        <v>81</v>
+        <v>240</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>216</v>
+        <v>246</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>217</v>
+        <v>247</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>218</v>
+        <v>248</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>208</v>
+        <v>237</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>219</v>
+        <v>249</v>
       </c>
       <c r="F4" s="17" t="s">
-        <v>220</v>
+        <v>250</v>
       </c>
       <c r="G4" s="17" t="s">
-        <v>81</v>
+        <v>240</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>221</v>
+        <v>251</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>222</v>
+        <v>252</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>223</v>
+        <v>253</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>224</v>
+        <v>254</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>225</v>
+        <v>255</v>
       </c>
       <c r="F5" s="17" t="s">
-        <v>226</v>
+        <v>256</v>
       </c>
       <c r="G5" s="17" t="s">
-        <v>81</v>
+        <v>240</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
-        <v>227</v>
+        <v>257</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>212</v>
+        <v>242</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>228</v>
+        <v>258</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>208</v>
+        <v>237</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>229</v>
+        <v>259</v>
       </c>
       <c r="F6" s="17" t="s">
         <v>126</v>
       </c>
       <c r="G6" s="17" t="s">
-        <v>81</v>
+        <v>240</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
-        <v>230</v>
+        <v>260</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>217</v>
+        <v>247</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>231</v>
+        <v>261</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>208</v>
+        <v>237</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>232</v>
+        <v>262</v>
       </c>
       <c r="F7" s="17" t="s">
         <v>126</v>
       </c>
       <c r="G7" s="17" t="s">
-        <v>81</v>
+        <v>240</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
-        <v>233</v>
+        <v>263</v>
       </c>
       <c r="B8" s="17" t="s">
         <v>116</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>234</v>
+        <v>264</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>235</v>
+        <v>265</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>225</v>
+        <v>255</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>236</v>
+        <v>266</v>
       </c>
       <c r="G8" s="17" t="s">
-        <v>81</v>
+        <v>240</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
+        <v>267</v>
+      </c>
+      <c r="B9" s="17" t="s">
+        <v>268</v>
+      </c>
+      <c r="C9" s="17" t="s">
+        <v>269</v>
+      </c>
+      <c r="D9" s="17" t="s">
+        <v>270</v>
+      </c>
+      <c r="E9" s="17" t="s">
+        <v>271</v>
+      </c>
+      <c r="F9" s="17" t="s">
+        <v>272</v>
+      </c>
+      <c r="G9" s="17" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="17" t="s">
+        <v>273</v>
+      </c>
+      <c r="B10" s="17" t="s">
+        <v>242</v>
+      </c>
+      <c r="C10" s="17" t="s">
+        <v>258</v>
+      </c>
+      <c r="D10" s="17" t="s">
         <v>237</v>
       </c>
-      <c r="B9" s="17" t="s">
-        <v>238</v>
-      </c>
-      <c r="C9" s="17" t="s">
-        <v>239</v>
-      </c>
-      <c r="D9" s="17" t="s">
-        <v>240</v>
-      </c>
-      <c r="E9" s="17" t="s">
-        <v>241</v>
-      </c>
-      <c r="F9" s="17" t="s">
-        <v>242</v>
-      </c>
-      <c r="G9" s="17" t="s">
+      <c r="E10" s="17" t="s">
+        <v>274</v>
+      </c>
+      <c r="F10" s="17" t="s">
+        <v>134</v>
+      </c>
+      <c r="G10" s="17" t="s">
         <v>81</v>
       </c>
     </row>
+    <row r="11" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A11" s="17" t="s">
+        <v>275</v>
+      </c>
+      <c r="B11" s="17" t="s">
+        <v>247</v>
+      </c>
+      <c r="C11" s="17" t="s">
+        <v>276</v>
+      </c>
+      <c r="D11" s="17" t="s">
+        <v>277</v>
+      </c>
+      <c r="E11" s="17" t="s">
+        <v>278</v>
+      </c>
+      <c r="F11" s="17" t="s">
+        <v>134</v>
+      </c>
+      <c r="G11" s="17" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A12" s="17" t="s">
+        <v>279</v>
+      </c>
+      <c r="B12" s="17" t="s">
+        <v>116</v>
+      </c>
+      <c r="C12" s="17" t="s">
+        <v>280</v>
+      </c>
+      <c r="D12" s="17" t="s">
+        <v>265</v>
+      </c>
+      <c r="E12" s="17" t="s">
+        <v>281</v>
+      </c>
+      <c r="F12" s="17" t="s">
+        <v>266</v>
+      </c>
+      <c r="G12" s="17" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A13" s="17" t="s">
+        <v>282</v>
+      </c>
+      <c r="B13" s="17" t="s">
+        <v>268</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>269</v>
+      </c>
+      <c r="D13" s="17" t="s">
+        <v>270</v>
+      </c>
+      <c r="E13" s="17" t="s">
+        <v>283</v>
+      </c>
+      <c r="F13" s="17" t="s">
+        <v>284</v>
+      </c>
+      <c r="G13" s="17" t="s">
+        <v>81</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G9" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
+  <autoFilter ref="A1:G13" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3203,39 +3604,39 @@
   <sheetData>
     <row r="1" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>243</v>
+        <v>285</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>244</v>
+        <v>286</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>245</v>
+        <v>287</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>204</v>
+        <v>233</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>246</v>
+        <v>288</v>
       </c>
       <c r="F1" s="16" t="s">
-        <v>247</v>
+        <v>289</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
-        <v>248</v>
+        <v>290</v>
       </c>
       <c r="B2" s="17" t="s">
         <v>67</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>249</v>
+        <v>291</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>81</v>
+        <v>240</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>250</v>
+        <v>292</v>
       </c>
       <c r="F2" s="17" t="s">
         <v>83</v>
@@ -3243,19 +3644,19 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
-        <v>251</v>
+        <v>293</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>252</v>
+        <v>294</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>253</v>
+        <v>295</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>81</v>
+        <v>240</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>254</v>
+        <v>296</v>
       </c>
       <c r="F3" s="17" t="s">
         <v>83</v>
@@ -3263,56 +3664,56 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>255</v>
+        <v>297</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>256</v>
+        <v>298</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>257</v>
+        <v>299</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>81</v>
+        <v>240</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>258</v>
+        <v>300</v>
       </c>
       <c r="F4" s="17" t="s">
-        <v>259</v>
+        <v>301</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>260</v>
+        <v>302</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>261</v>
+        <v>303</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>262</v>
+        <v>304</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>81</v>
+        <v>240</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>263</v>
+        <v>305</v>
       </c>
       <c r="F5" s="17" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
-        <v>264</v>
+        <v>306</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>265</v>
+        <v>307</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>266</v>
+        <v>308</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>81</v>
+        <v>240</v>
       </c>
       <c r="E6" s="17" t="s">
         <v>26</v>
@@ -3323,117 +3724,119 @@
     </row>
     <row r="7" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
-        <v>267</v>
+        <v>309</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>268</v>
+        <v>310</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>269</v>
+        <v>311</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>81</v>
+        <v>240</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>270</v>
+        <v>312</v>
       </c>
       <c r="F7" s="17" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
-        <v>271</v>
+        <v>313</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>272</v>
+        <v>314</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>273</v>
+        <v>315</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>81</v>
+        <v>240</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>274</v>
+        <v>316</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>275</v>
+        <v>317</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>276</v>
+        <v>318</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>277</v>
+        <v>319</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>81</v>
+        <v>240</v>
       </c>
       <c r="E9" s="17" t="s">
-        <v>274</v>
+        <v>316</v>
       </c>
       <c r="F9" s="17" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="17" t="s">
-        <v>278</v>
+        <v>320</v>
       </c>
       <c r="B10" s="17" t="s">
         <v>52</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>279</v>
+        <v>321</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>81</v>
+        <v>240</v>
       </c>
       <c r="E10" s="17" t="s">
         <v>51</v>
       </c>
       <c r="F10" s="17" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="51" x14ac:dyDescent="0.25">
       <c r="A11" s="17" t="s">
-        <v>280</v>
+        <v>322</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>281</v>
+        <v>323</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>282</v>
+        <v>324</v>
       </c>
       <c r="D11" s="17" t="s">
         <v>81</v>
       </c>
       <c r="E11" s="17" t="s">
-        <v>283</v>
-      </c>
-      <c r="F11" s="17"/>
+        <v>325</v>
+      </c>
+      <c r="F11" s="17" t="s">
+        <v>326</v>
+      </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
-        <v>284</v>
+        <v>327</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>285</v>
+        <v>328</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>286</v>
+        <v>329</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>81</v>
+        <v>240</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>287</v>
+        <v>330</v>
       </c>
       <c r="F12" s="17" t="s">
         <v>96</v>
@@ -3459,121 +3862,121 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>288</v>
+        <v>331</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>289</v>
+        <v>332</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>290</v>
+        <v>333</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>291</v>
+        <v>334</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>292</v>
+        <v>335</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
-        <v>293</v>
+        <v>336</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>294</v>
+        <v>337</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>295</v>
+        <v>338</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>296</v>
+        <v>339</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>297</v>
+        <v>340</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
-        <v>298</v>
+        <v>341</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>299</v>
+        <v>342</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>300</v>
+        <v>343</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>301</v>
+        <v>344</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>302</v>
+        <v>345</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>303</v>
+        <v>346</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>304</v>
+        <v>347</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>304</v>
+        <v>347</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>305</v>
+        <v>348</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>306</v>
+        <v>349</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>307</v>
+        <v>350</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>308</v>
+        <v>351</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>309</v>
+        <v>352</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>310</v>
+        <v>353</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>302</v>
+        <v>345</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
-        <v>311</v>
+        <v>354</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>312</v>
+        <v>355</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>312</v>
+        <v>355</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>313</v>
+        <v>356</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>297</v>
+        <v>340</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
-        <v>314</v>
+        <v>357</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>315</v>
+        <v>358</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>316</v>
+        <v>359</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>317</v>
+        <v>360</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>297</v>
+        <v>340</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
SmartDoc 2.0 P3: document flow -- content, structure check, look, editor (S2-020)
/new is now the 2.0 flow (same links and parameters as the 1.x wizard it
replaces): add content (paste, or TXT/DOCX/PDF with their options), the
import job's real stages, then a structure check before any look is
applied -- project name, a block as Heading 1-3 or body text, a section
moved up or down, low-confidence blocks marked -- saved once with
PUT /content (formatting untouched, no new endpoint, no schema change).
Then the look: a template with its sample, a reference document, or none,
plus optional instructions that are called AI only when the server has a
model (GET /capabilities/ai). All copy in en/bg; signed out -> sign in and
back. E2E helpers drive the new flow, so every workflow goes through it.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/SMARTDOC_2_0_MASTER_TRACKER.xlsx
+++ b/docs/SMARTDOC_2_0_MASTER_TRACKER.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\speed\Desktop\Claude - ПРОЕКТ\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D521E408-5370-4543-BAC6-3462A8123C6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2396D6C2-42E2-48E5-B3F6-B31B404B8E0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Release Readiness'!$A$1:$E$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Roadmap!$A$1:$F$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Tasks!$A$1:$P$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Tests!$A$1:$G$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Tests!$A$1:$G$20</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="766" uniqueCount="452">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="790" uniqueCount="466">
   <si>
     <t>SmartDoc 2.0 -- master tracker</t>
   </si>
@@ -487,13 +487,22 @@
     <t>Add Content / Structure Review / Style screens (4-6)</t>
   </si>
   <si>
-    <t>Rebuild the create wizard as the approved 3-step flow on the existing import + structure + format APIs; structure review edits (rename, level, reorder, reclassify).</t>
-  </si>
-  <si>
-    <t>TXT/DOCX/PDF/paste reach the editor through review; original content preserved</t>
-  </si>
-  <si>
-    <t>Design in SPEC 5.1 (content -&gt; analyse -&gt; check structure -&gt; look -&gt; editor at /new, same APIs, PUT /content for structure edits, no schema change). GET /capabilities/ai (this commit) lets the look step call instructions AI only when a model is configured. Flow components in progress.</t>
+    <t>The 2.0 document flow at /new (replaces the 1.x wizard, same links): add content (paste / TXT, DOCX, PDF with its options) -&gt; the import job with its real stages -&gt; check the structure (project name; block as Heading 1-3 or body text; move a section up/down; low-confidence blocks marked) -&gt; choose the look (template with sample, reference document, none; optional instructions, called AI only when a model is configured) -&gt; the format job -&gt; editor.</t>
+  </si>
+  <si>
+    <t>TXT/DOCX/PDF/paste reach the editor through review; original content preserved; structure edits saved once with PUT /content (formatting untouched); no schema change; EN/BG; signed-out -&gt; sign in and back</t>
+  </si>
+  <si>
+    <t>(this commit)</t>
+  </si>
+  <si>
+    <t>pending push</t>
+  </si>
+  <si>
+    <t>structureEdits.test.ts 10, DocumentFlow.test.tsx 10 (steps, edits saved once, nothing saved without a change, ?template preselect, skip, AI label both ways, import error, BG); Playwright 66/1 skipped with every existing workflow (DOCX, PDF editable/layout, tracked changes, templates) through the new flow + documents.spec rewritten for structure edits; browser: paste BG text -&gt; move section -&gt; template -&gt; editor shows the new order (1280 light), upload + structure at 375 dark</t>
+  </si>
+  <si>
+    <t>Old CreateDocumentWizard removed. Screenshots docs/ui-review/2026-10-14/create-*. Next in P3: style recommendation (M3.3) once AI provider decision (D-007) allows; S2-017 BG copy for TrackedChangesChoice/ReferenceStyleSummary/JobProgressBar used inside the flow.</t>
   </si>
   <si>
     <t>S2-030</t>
@@ -610,10 +619,10 @@
     <t>Cards show the real first page, nothing invented; per-type fallback while loading and on error; no rendering on dashboard list requests (rendered on first request, cached per revision, immutable URL per updatedAt); another account gets 404; deleted with the document</t>
   </si>
   <si>
-    <t>(this commit)</t>
-  </si>
-  <si>
-    <t>pending push</t>
+    <t>719b8d7</t>
+  </si>
+  <si>
+    <t>dpl_3bYEX4jWjA2UHuRcJqPw8oK1fzKc (READY, 719b8d7)</t>
   </si>
   <si>
     <t>backend tests/test_thumbnails.py 6 (cache per revision, re-render after edit, stranger 404, deleted with document, render failure -&gt; 404); ProjectCard.test.tsx 4 (lazy src per version, loading/shown/missing, BG alt); e2e: real image on the card + stranger 404; local browser: 3 real thumbnails incl. Cyrillic, lazy on scroll</t>
@@ -856,7 +865,7 @@
     <t>Some thumbnails 404: 'Storage key escapes the storage root' -- resolving files written side by side came back with 8.3 short names</t>
   </si>
   <si>
-    <t>LocalStorageProvider: root created before resolve; keys checked by their parts, not by resolving (this commit)</t>
+    <t>LocalStorageProvider: root created before resolve; keys checked by their parts, not by resolving (719b8d7)</t>
   </si>
   <si>
     <t>tests/test_storage.py: escape params (.., empty, //, ., backslashes, drive, rooted), 12 concurrent writes into a new folder; browser: all thumbnails load, no errors in the log. Production uses S3 -- not affected</t>
@@ -874,7 +883,7 @@
     <t>The field collapsed to a sliver (flex-1 in a column)</t>
   </si>
   <si>
-    <t>Idea panel: field full card width on phones (this commit)</t>
+    <t>Idea panel: field full card width on phones (719b8d7)</t>
   </si>
   <si>
     <t>Browser 375: field 44 px high, full width</t>
@@ -892,7 +901,7 @@
     <t>Search squeezed to 'Searc' beside the heading</t>
   </si>
   <si>
-    <t>Search and 'All projects' on their own row on phones (this commit)</t>
+    <t>Search and 'All projects' on their own row on phones (719b8d7)</t>
   </si>
   <si>
     <t>Browser 375: full-width row, no overflow</t>
@@ -910,7 +919,7 @@
     <t>Focus lost (document body)</t>
   </si>
   <si>
-    <t>AppShell returns focus to the menu button on close (this commit)</t>
+    <t>AppShell returns focus to the menu button on close (719b8d7)</t>
   </si>
   <si>
     <t>AppShell.test.tsx; browser: activeElement = Open the menu</t>
@@ -928,7 +937,7 @@
     <t>The new thumbnail route was not registered in the suite (which demands every id-taking route be checked)</t>
   </si>
   <si>
-    <t>Registered GET /documents/{id}/thumbnail (this commit)</t>
+    <t>Registered GET /documents/{id}/thumbnail (719b8d7)</t>
   </si>
   <si>
     <t>test_security_suite.py 167/167: another workspace gets the same 404 as a missing document, 401 signed out, owner resources unchanged</t>
@@ -946,7 +955,7 @@
     <t>The committed OpenAPI schema (frontend/types/generated) lacked the thumbnail route added in b716a5f</t>
   </si>
   <si>
-    <t>scripts.export_openapi + npm run generate-types (this commit; also adds GET /capabilities/ai)</t>
+    <t>scripts.export_openapi + npm run generate-types (719b8d7; also adds GET /capabilities/ai)</t>
   </si>
   <si>
     <t>Full backend suite green (T-013); tsc clean</t>
@@ -1175,6 +1184,39 @@
   </si>
   <si>
     <t>docs/ui-review/2026-10-14/</t>
+  </si>
+  <si>
+    <t>T-017</t>
+  </si>
+  <si>
+    <t>Vitest + tsc + eslint with the document flow</t>
+  </si>
+  <si>
+    <t>PASS 452 / tsc clean / eslint clean</t>
+  </si>
+  <si>
+    <t>npx vitest run</t>
+  </si>
+  <si>
+    <t>T-018</t>
+  </si>
+  <si>
+    <t>Playwright on the new /new flow (all workflows go through createDocument)</t>
+  </si>
+  <si>
+    <t>PASS 66 / 1 skipped; after the last CSS change documents + accessibility specs 7/7</t>
+  </si>
+  <si>
+    <t>T-019</t>
+  </si>
+  <si>
+    <t>Document flow: sign-in redirect, paste -&gt; structure edit -&gt; template -&gt; editor (1280 light); upload mode + structure (375 dark)</t>
+  </si>
+  <si>
+    <t>PASS; indent tightened on phones after the check</t>
+  </si>
+  <si>
+    <t>docs/ui-review/2026-10-14/create-*</t>
   </si>
   <si>
     <t>Decision ID</t>
@@ -2059,7 +2101,7 @@
       </c>
       <c r="B7" s="5">
         <f>COUNTIF(Tasks!$G$2:$G$25,A7)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C7" s="5">
         <f>COUNTIF(Roadmap!$D$2:$D$10,A7)</f>
@@ -2098,7 +2140,7 @@
       </c>
       <c r="B10" s="5">
         <f>COUNTIF(Tasks!$G$2:$G$25,A10)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C10" s="5">
         <f>COUNTIF(Roadmap!$D$2:$D$10,A10)</f>
@@ -2137,7 +2179,7 @@
       </c>
       <c r="B13" s="14">
         <f>IFERROR((B11+B10)/B12,0)</f>
-        <v>0.70833333333333337</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -2961,7 +3003,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="12" spans="1:16" ht="76.5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:16" ht="255" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
         <v>144</v>
       </c>
@@ -2981,7 +3023,7 @@
         <v>26</v>
       </c>
       <c r="G12" s="17" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="H12" s="17" t="s">
         <v>138</v>
@@ -2995,31 +3037,37 @@
       <c r="K12" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="L12" s="17"/>
-      <c r="M12" s="17"/>
-      <c r="N12" s="17"/>
+      <c r="L12" s="17" t="s">
+        <v>148</v>
+      </c>
+      <c r="M12" s="17" t="s">
+        <v>149</v>
+      </c>
+      <c r="N12" s="17" t="s">
+        <v>150</v>
+      </c>
       <c r="O12" s="17" t="s">
         <v>81</v>
       </c>
       <c r="P12" s="17" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
     </row>
     <row r="13" spans="1:16" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A13" s="17" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="B13" s="17" t="s">
         <v>38</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="D13" s="17" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="E13" s="17" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="F13" s="17" t="s">
         <v>26</v>
@@ -3031,7 +3079,7 @@
         <v>122</v>
       </c>
       <c r="I13" s="17" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="J13" s="17" t="s">
         <v>78</v>
@@ -3049,19 +3097,19 @@
     </row>
     <row r="14" spans="1:16" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B14" s="17" t="s">
         <v>42</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="E14" s="17" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="F14" s="17" t="s">
         <v>26</v>
@@ -3070,10 +3118,10 @@
         <v>5</v>
       </c>
       <c r="H14" s="17" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="I14" s="17" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="J14" s="17" t="s">
         <v>78</v>
@@ -3088,24 +3136,24 @@
         <v>81</v>
       </c>
       <c r="P14" s="17" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
     </row>
     <row r="15" spans="1:16" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A15" s="17" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B15" s="17" t="s">
         <v>46</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="D15" s="17" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="E15" s="17" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="F15" s="17" t="s">
         <v>26</v>
@@ -3114,10 +3162,10 @@
         <v>5</v>
       </c>
       <c r="H15" s="17" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="I15" s="17" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="J15" s="17" t="s">
         <v>78</v>
@@ -3132,24 +3180,24 @@
         <v>81</v>
       </c>
       <c r="P15" s="17" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
     </row>
     <row r="16" spans="1:16" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A16" s="17" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="B16" s="17" t="s">
         <v>51</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="D16" s="17" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="E16" s="17" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="F16" s="17" t="s">
         <v>26</v>
@@ -3158,10 +3206,10 @@
         <v>5</v>
       </c>
       <c r="H16" s="17" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="I16" s="17" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="J16" s="17" t="s">
         <v>78</v>
@@ -3176,24 +3224,24 @@
         <v>81</v>
       </c>
       <c r="P16" s="17" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
     </row>
     <row r="17" spans="1:16" ht="127.5" x14ac:dyDescent="0.25">
       <c r="A17" s="17" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B17" s="17" t="s">
         <v>30</v>
       </c>
       <c r="C17" s="17" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="D17" s="17" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="E17" s="17" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="F17" s="17" t="s">
         <v>22</v>
@@ -3205,7 +3253,7 @@
         <v>110</v>
       </c>
       <c r="I17" s="17" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="J17" s="17" t="s">
         <v>78</v>
@@ -3220,30 +3268,30 @@
         <v>135</v>
       </c>
       <c r="N17" s="17" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="O17" s="17" t="s">
         <v>81</v>
       </c>
       <c r="P17" s="17" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
     </row>
     <row r="18" spans="1:16" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A18" s="17" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B18" s="17" t="s">
         <v>30</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="D18" s="17" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="E18" s="17" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="F18" s="17" t="s">
         <v>26</v>
@@ -3252,10 +3300,10 @@
         <v>5</v>
       </c>
       <c r="H18" s="17" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="I18" s="17" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="J18" s="17" t="s">
         <v>78</v>
@@ -3270,12 +3318,12 @@
         <v>81</v>
       </c>
       <c r="P18" s="17" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
     </row>
     <row r="19" spans="1:16" ht="165.75" x14ac:dyDescent="0.25">
       <c r="A19" s="17" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="B19" s="17" t="s">
         <v>30</v>
@@ -3284,10 +3332,10 @@
         <v>116</v>
       </c>
       <c r="D19" s="17" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="E19" s="17" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="F19" s="17" t="s">
         <v>22</v>
@@ -3299,7 +3347,7 @@
         <v>130</v>
       </c>
       <c r="I19" s="17" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="J19" s="17" t="s">
         <v>78</v>
@@ -3308,24 +3356,24 @@
         <v>79</v>
       </c>
       <c r="L19" s="17" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="M19" s="17" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="N19" s="17" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="O19" s="17" t="s">
         <v>81</v>
       </c>
       <c r="P19" s="17" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
     </row>
     <row r="20" spans="1:16" ht="102" x14ac:dyDescent="0.25">
       <c r="A20" s="17" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="B20" s="17" t="s">
         <v>30</v>
@@ -3334,10 +3382,10 @@
         <v>116</v>
       </c>
       <c r="D20" s="17" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="E20" s="17" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="F20" s="17" t="s">
         <v>22</v>
@@ -3349,7 +3397,7 @@
         <v>110</v>
       </c>
       <c r="I20" s="17" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="J20" s="17" t="s">
         <v>78</v>
@@ -3358,24 +3406,24 @@
         <v>79</v>
       </c>
       <c r="L20" s="17" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="M20" s="17" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="N20" s="17" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="O20" s="17" t="s">
         <v>81</v>
       </c>
       <c r="P20" s="17" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
     </row>
     <row r="21" spans="1:16" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A21" s="17" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B21" s="17" t="s">
         <v>30</v>
@@ -3384,10 +3432,10 @@
         <v>116</v>
       </c>
       <c r="D21" s="17" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="E21" s="17" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="F21" s="17" t="s">
         <v>22</v>
@@ -3399,7 +3447,7 @@
         <v>130</v>
       </c>
       <c r="I21" s="17" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="J21" s="17" t="s">
         <v>78</v>
@@ -3408,36 +3456,36 @@
         <v>79</v>
       </c>
       <c r="L21" s="17" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="M21" s="17" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="N21" s="17" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="O21" s="17" t="s">
         <v>81</v>
       </c>
       <c r="P21" s="17" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
     </row>
     <row r="22" spans="1:16" ht="51" x14ac:dyDescent="0.25">
       <c r="A22" s="17" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="B22" s="17" t="s">
         <v>30</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="D22" s="17" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E22" s="17" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="F22" s="17" t="s">
         <v>26</v>
@@ -3449,7 +3497,7 @@
         <v>122</v>
       </c>
       <c r="I22" s="17" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="J22" s="17" t="s">
         <v>78</v>
@@ -3458,24 +3506,24 @@
         <v>79</v>
       </c>
       <c r="L22" s="17" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="M22" s="17" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="N22" s="17" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="O22" s="17" t="s">
         <v>81</v>
       </c>
       <c r="P22" s="17" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
     </row>
     <row r="23" spans="1:16" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A23" s="17" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="B23" s="17" t="s">
         <v>30</v>
@@ -3484,10 +3532,10 @@
         <v>116</v>
       </c>
       <c r="D23" s="17" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="E23" s="17" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="F23" s="17" t="s">
         <v>26</v>
@@ -3499,7 +3547,7 @@
         <v>122</v>
       </c>
       <c r="I23" s="17" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="J23" s="17" t="s">
         <v>78</v>
@@ -3508,24 +3556,24 @@
         <v>79</v>
       </c>
       <c r="L23" s="17" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="M23" s="17" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="N23" s="17" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="O23" s="17" t="s">
         <v>81</v>
       </c>
       <c r="P23" s="17" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
     </row>
     <row r="24" spans="1:16" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A24" s="17" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="B24" s="17" t="s">
         <v>30</v>
@@ -3534,10 +3582,10 @@
         <v>116</v>
       </c>
       <c r="D24" s="17" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="E24" s="17" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="F24" s="17" t="s">
         <v>26</v>
@@ -3546,10 +3594,10 @@
         <v>10</v>
       </c>
       <c r="H24" s="17" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="I24" s="17" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="J24" s="17" t="s">
         <v>78</v>
@@ -3558,24 +3606,24 @@
         <v>79</v>
       </c>
       <c r="L24" s="17" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="M24" s="17" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="N24" s="17" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="O24" s="17" t="s">
         <v>81</v>
       </c>
       <c r="P24" s="17" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
     </row>
     <row r="25" spans="1:16" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A25" s="17" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="B25" s="17" t="s">
         <v>30</v>
@@ -3584,10 +3632,10 @@
         <v>116</v>
       </c>
       <c r="D25" s="17" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="E25" s="17" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="F25" s="17" t="s">
         <v>30</v>
@@ -3596,10 +3644,10 @@
         <v>5</v>
       </c>
       <c r="H25" s="17" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="I25" s="17" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="J25" s="17" t="s">
         <v>78</v>
@@ -3614,7 +3662,7 @@
         <v>81</v>
       </c>
       <c r="P25" s="17" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
     </row>
   </sheetData>
@@ -3663,312 +3711,312 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="F1" s="16" t="s">
         <v>2</v>
       </c>
       <c r="G1" s="16" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="H1" s="16" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="F2" s="17" t="s">
         <v>8</v>
       </c>
       <c r="G2" s="17" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="H2" s="17" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="F3" s="17" t="s">
         <v>5</v>
       </c>
       <c r="G3" s="17"/>
       <c r="H3" s="17" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="F4" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G4" s="17" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="H4" s="17" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="F5" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G5" s="17" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="H5" s="17" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="51" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="F6" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G6" s="17" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="H6" s="17" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="89.25" x14ac:dyDescent="0.25">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="F7" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G7" s="17" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="H7" s="17" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="51" x14ac:dyDescent="0.25">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="F8" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G8" s="17" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="H8" s="17" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="51" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="E9" s="17" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="F9" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G9" s="17" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="H9" s="17" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="51" x14ac:dyDescent="0.25">
       <c r="A10" s="17" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="E10" s="17" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="F10" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G10" s="17" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="H10" s="17" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" ht="51" x14ac:dyDescent="0.25">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A11" s="17" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="D11" s="17" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="E11" s="17" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="F11" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G11" s="17" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="H11" s="17" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="F12" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G12" s="17" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="H12" s="17" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
     </row>
   </sheetData>
@@ -4002,7 +4050,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -4016,226 +4064,226 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="F1" s="16" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="G1" s="16" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="G2" s="17" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="C3" s="17" t="s">
+        <v>320</v>
+      </c>
+      <c r="D3" s="17" t="s">
+        <v>314</v>
+      </c>
+      <c r="E3" s="17" t="s">
+        <v>321</v>
+      </c>
+      <c r="F3" s="17" t="s">
+        <v>322</v>
+      </c>
+      <c r="G3" s="17" t="s">
         <v>317</v>
-      </c>
-      <c r="D3" s="17" t="s">
-        <v>311</v>
-      </c>
-      <c r="E3" s="17" t="s">
-        <v>318</v>
-      </c>
-      <c r="F3" s="17" t="s">
-        <v>319</v>
-      </c>
-      <c r="G3" s="17" t="s">
-        <v>314</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="F4" s="17" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="G4" s="17" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="F5" s="17" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="G5" s="17" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="F6" s="17" t="s">
         <v>126</v>
       </c>
       <c r="G6" s="17" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="F7" s="17" t="s">
         <v>126</v>
       </c>
       <c r="G7" s="17" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="B8" s="17" t="s">
         <v>116</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="G8" s="17" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="E9" s="17" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="F9" s="17" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="G9" s="17" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="17" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E10" s="17" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="F10" s="17" t="s">
         <v>134</v>
@@ -4246,19 +4294,19 @@
     </row>
     <row r="11" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A11" s="17" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="D11" s="17" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="E11" s="17" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="F11" s="17" t="s">
         <v>134</v>
@@ -4269,22 +4317,22 @@
     </row>
     <row r="12" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="B12" s="17" t="s">
         <v>116</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="F12" s="17" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="G12" s="17" t="s">
         <v>81</v>
@@ -4292,22 +4340,22 @@
     </row>
     <row r="13" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A13" s="17" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="B13" s="17" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="D13" s="17" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="E13" s="17" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="F13" s="17" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="G13" s="17" t="s">
         <v>81</v>
@@ -4315,22 +4363,22 @@
     </row>
     <row r="14" spans="1:7" ht="51" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="B14" s="17" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E14" s="17" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="F14" s="17" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="G14" s="17" t="s">
         <v>81</v>
@@ -4338,22 +4386,22 @@
     </row>
     <row r="15" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A15" s="17" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="B15" s="17" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="D15" s="17" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E15" s="17" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="F15" s="17" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="G15" s="17" t="s">
         <v>81</v>
@@ -4361,22 +4409,22 @@
     </row>
     <row r="16" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A16" s="17" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="B16" s="17" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="D16" s="17" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="E16" s="17" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="F16" s="17" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="G16" s="17" t="s">
         <v>81</v>
@@ -4384,29 +4432,98 @@
     </row>
     <row r="17" spans="1:7" ht="51" x14ac:dyDescent="0.25">
       <c r="A17" s="17" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="B17" s="17" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="C17" s="17" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="D17" s="17" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="E17" s="17" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="F17" s="17" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="G17" s="17" t="s">
         <v>81</v>
       </c>
     </row>
+    <row r="18" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A18" s="17" t="s">
+        <v>379</v>
+      </c>
+      <c r="B18" s="17" t="s">
+        <v>319</v>
+      </c>
+      <c r="C18" s="17" t="s">
+        <v>380</v>
+      </c>
+      <c r="D18" s="17" t="s">
+        <v>314</v>
+      </c>
+      <c r="E18" s="17" t="s">
+        <v>381</v>
+      </c>
+      <c r="F18" s="17" t="s">
+        <v>382</v>
+      </c>
+      <c r="G18" s="17" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="51" x14ac:dyDescent="0.25">
+      <c r="A19" s="17" t="s">
+        <v>383</v>
+      </c>
+      <c r="B19" s="17" t="s">
+        <v>324</v>
+      </c>
+      <c r="C19" s="17" t="s">
+        <v>384</v>
+      </c>
+      <c r="D19" s="17" t="s">
+        <v>314</v>
+      </c>
+      <c r="E19" s="17" t="s">
+        <v>385</v>
+      </c>
+      <c r="F19" s="17" t="s">
+        <v>373</v>
+      </c>
+      <c r="G19" s="17" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A20" s="17" t="s">
+        <v>386</v>
+      </c>
+      <c r="B20" s="17" t="s">
+        <v>375</v>
+      </c>
+      <c r="C20" s="17" t="s">
+        <v>387</v>
+      </c>
+      <c r="D20" s="17" t="s">
+        <v>342</v>
+      </c>
+      <c r="E20" s="17" t="s">
+        <v>388</v>
+      </c>
+      <c r="F20" s="17" t="s">
+        <v>389</v>
+      </c>
+      <c r="G20" s="17" t="s">
+        <v>81</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G17" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
+  <autoFilter ref="A1:G20" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4425,39 +4542,39 @@
   <sheetData>
     <row r="1" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>376</v>
+        <v>390</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>377</v>
+        <v>391</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>378</v>
+        <v>392</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>379</v>
+        <v>393</v>
       </c>
       <c r="F1" s="16" t="s">
-        <v>380</v>
+        <v>394</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
-        <v>381</v>
+        <v>395</v>
       </c>
       <c r="B2" s="17" t="s">
         <v>67</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>382</v>
+        <v>396</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>383</v>
+        <v>397</v>
       </c>
       <c r="F2" s="17" t="s">
         <v>83</v>
@@ -4465,19 +4582,19 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
-        <v>384</v>
+        <v>398</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>385</v>
+        <v>399</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>386</v>
+        <v>400</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>387</v>
+        <v>401</v>
       </c>
       <c r="F3" s="17" t="s">
         <v>83</v>
@@ -4485,56 +4602,56 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>388</v>
+        <v>402</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>389</v>
+        <v>403</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>390</v>
+        <v>404</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>391</v>
+        <v>405</v>
       </c>
       <c r="F4" s="17" t="s">
-        <v>392</v>
+        <v>406</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>393</v>
+        <v>407</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>394</v>
+        <v>408</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>395</v>
+        <v>409</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>396</v>
+        <v>410</v>
       </c>
       <c r="F5" s="17" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
-        <v>397</v>
+        <v>411</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>398</v>
+        <v>412</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>399</v>
+        <v>413</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="E6" s="17" t="s">
         <v>26</v>
@@ -4545,119 +4662,119 @@
     </row>
     <row r="7" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
-        <v>400</v>
+        <v>414</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>401</v>
+        <v>415</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>402</v>
+        <v>416</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>403</v>
+        <v>417</v>
       </c>
       <c r="F7" s="17" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
-        <v>404</v>
+        <v>418</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>405</v>
+        <v>419</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>406</v>
+        <v>420</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>407</v>
+        <v>421</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>408</v>
+        <v>422</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>409</v>
+        <v>423</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>410</v>
+        <v>424</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="E9" s="17" t="s">
-        <v>407</v>
+        <v>421</v>
       </c>
       <c r="F9" s="17" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="17" t="s">
-        <v>411</v>
+        <v>425</v>
       </c>
       <c r="B10" s="17" t="s">
         <v>52</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>412</v>
+        <v>426</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="E10" s="17" t="s">
         <v>51</v>
       </c>
       <c r="F10" s="17" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="51" x14ac:dyDescent="0.25">
       <c r="A11" s="17" t="s">
-        <v>413</v>
+        <v>427</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>414</v>
+        <v>428</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>415</v>
+        <v>429</v>
       </c>
       <c r="D11" s="17" t="s">
         <v>81</v>
       </c>
       <c r="E11" s="17" t="s">
-        <v>416</v>
+        <v>430</v>
       </c>
       <c r="F11" s="17" t="s">
-        <v>417</v>
+        <v>431</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
-        <v>418</v>
+        <v>432</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>419</v>
+        <v>433</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>420</v>
+        <v>434</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>421</v>
+        <v>435</v>
       </c>
       <c r="F12" s="17" t="s">
         <v>96</v>
@@ -4683,121 +4800,121 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>422</v>
+        <v>436</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>423</v>
+        <v>437</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>424</v>
+        <v>438</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>425</v>
+        <v>439</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>426</v>
+        <v>440</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
-        <v>427</v>
+        <v>441</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>428</v>
+        <v>442</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>429</v>
+        <v>443</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>430</v>
+        <v>444</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>431</v>
+        <v>445</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
-        <v>432</v>
+        <v>446</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>433</v>
+        <v>447</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>434</v>
+        <v>448</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>435</v>
+        <v>449</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>436</v>
+        <v>450</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>437</v>
+        <v>451</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>438</v>
+        <v>452</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>438</v>
+        <v>452</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>439</v>
+        <v>453</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>440</v>
+        <v>454</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>441</v>
+        <v>455</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>442</v>
+        <v>456</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>443</v>
+        <v>457</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>444</v>
+        <v>458</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>436</v>
+        <v>450</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
+        <v>459</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>460</v>
+      </c>
+      <c r="C6" s="17" t="s">
+        <v>460</v>
+      </c>
+      <c r="D6" s="17" t="s">
+        <v>461</v>
+      </c>
+      <c r="E6" s="17" t="s">
         <v>445</v>
-      </c>
-      <c r="B6" s="17" t="s">
-        <v>446</v>
-      </c>
-      <c r="C6" s="17" t="s">
-        <v>446</v>
-      </c>
-      <c r="D6" s="17" t="s">
-        <v>447</v>
-      </c>
-      <c r="E6" s="17" t="s">
-        <v>431</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
-        <v>448</v>
+        <v>462</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>449</v>
+        <v>463</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>450</v>
+        <v>464</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>451</v>
+        <v>465</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>431</v>
+        <v>445</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
SmartDoc 2.0 S2-017/S2-R06 (part 1): old screens bilingual and on the theme tokens
Account settings, password reset, confirm dialog, plan-limit banner, header,
account menu, landing, projects list, batch bar, compare (now in the app
shell) and billing: every interface string in en/bg (with a small plural
helper), zinc/amber/red classes replaced by the light/dark tokens. The new
flow's 1.x pieces (tracked changes, reference summary, job progress) too.
Numbers follow the interface language; billing units are named by key.
Tracker: S2-020 preview recorded (dpl_AujyaJa3..., READY); S2-017/S2-R06 in
progress.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/SMARTDOC_2_0_MASTER_TRACKER.xlsx
+++ b/docs/SMARTDOC_2_0_MASTER_TRACKER.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\speed\Desktop\Claude - ПРОЕКТ\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2396D6C2-42E2-48E5-B3F6-B31B404B8E0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B01FE76-B2E0-4815-A112-BBA4AA11C05A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -493,10 +493,10 @@
     <t>TXT/DOCX/PDF/paste reach the editor through review; original content preserved; structure edits saved once with PUT /content (formatting untouched); no schema change; EN/BG; signed-out -&gt; sign in and back</t>
   </si>
   <si>
-    <t>(this commit)</t>
-  </si>
-  <si>
-    <t>pending push</t>
+    <t>52ec2ea</t>
+  </si>
+  <si>
+    <t>dpl_AujyaJa3fBsFvN1dAbaPN33G3vzu (READY, 52ec2ea; checked with the Vercel API 2026-10-14)</t>
   </si>
   <si>
     <t>structureEdits.test.ts 10, DocumentFlow.test.tsx 10 (steps, edits saved once, nothing saved without a change, ?template preselect, skip, AI label both ways, import error, BG); Playwright 66/1 skipped with every existing workflow (DOCX, PDF editable/layout, tracked changes, templates) through the new flow + documents.spec rewritten for structure edits; browser: paste BG text -&gt; move section -&gt; template -&gt; editor shows the new order (1280 light), upload + structure at 375 dark</t>
@@ -604,7 +604,7 @@
     <t>No hard-coded interface English left in those screens (a grep test); both languages rendered in their tests</t>
   </si>
   <si>
-    <t>Until then those screens show English in Bulgarian mode.</t>
+    <t>Done: flow pieces (TrackedChangesChoice, ReferenceStyleSummary, JobProgressBar), account settings, password reset, confirm dialog, plan-limit banner, header, account menu, landing, projects list, batch bar, compare, billing. Next: templates library/editor. Editor chrome (editor/*) moves with the 2.0 editor rather than being translated twice. Server messages (API errors, version descriptions) stay in English until the API returns codes for them.</t>
   </si>
   <si>
     <t>S2-018</t>
@@ -733,7 +733,7 @@
     <t>No zinc-* classes left in components (grep test); both themes checked in the browser</t>
   </si>
   <si>
-    <t>Found in the UI review: they already switch with the theme, but in a neutral grey that doesn't match the new palette. Do with S2-017 screen by screen.</t>
+    <t>Same screens as S2-017, done together; compare now inside the app shell.</t>
   </si>
   <si>
     <t>Bug ID</t>
@@ -2075,7 +2075,7 @@
       </c>
       <c r="B5" s="5">
         <f>COUNTIF(Tasks!$G$2:$G$25,A5)</f>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C5" s="5">
         <f>COUNTIF(Roadmap!$D$2:$D$10,A5)</f>
@@ -2101,7 +2101,7 @@
       </c>
       <c r="B7" s="5">
         <f>COUNTIF(Tasks!$G$2:$G$25,A7)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C7" s="5">
         <f>COUNTIF(Roadmap!$D$2:$D$10,A7)</f>
@@ -3277,7 +3277,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="18" spans="1:16" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:16" ht="114.75" x14ac:dyDescent="0.25">
       <c r="A18" s="17" t="s">
         <v>181</v>
       </c>
@@ -3297,7 +3297,7 @@
         <v>26</v>
       </c>
       <c r="G18" s="17" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H18" s="17" t="s">
         <v>174</v>
@@ -3641,7 +3641,7 @@
         <v>30</v>
       </c>
       <c r="G25" s="17" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H25" s="17" t="s">
         <v>194</v>

</xml_diff>

<commit_message>
SmartDoc 2.0 tracker/checkpoint: S2-017, S2-R06, S2-021 (M3.3), S2-022 verified; D-012 pending
Tracker: S2-017/S2-R06/S2-021/S2-022 VERIFIED with their tests; S2-030 and
S2-040 in progress (editor plan E0, design model E3); bugs B-012..B-015;
tests T-020..T-022. Decision D-012 (canvas documents vs the shared
database) written as pending. Editor plan aligned with D-006 naming
(Document.kind = flow | canvas). Session state: next is E1.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/SMARTDOC_2_0_MASTER_TRACKER.xlsx
+++ b/docs/SMARTDOC_2_0_MASTER_TRACKER.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\speed\Desktop\Claude - ПРОЕКТ\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B01FE76-B2E0-4815-A112-BBA4AA11C05A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80BE36E1-27F4-49EE-8824-FD2F00BA357C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,12 +22,12 @@
     <sheet name="Release Readiness" sheetId="7" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Bugs!$A$1:$H$12</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Decisions!$A$1:$F$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Bugs!$A$1:$H$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Decisions!$A$1:$F$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Release Readiness'!$A$1:$E$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Roadmap!$A$1:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Tasks!$A$1:$P$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Tests!$A$1:$G$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Tasks!$A$1:$P$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Tests!$A$1:$G$23</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="790" uniqueCount="466">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="890" uniqueCount="524">
   <si>
     <t>SmartDoc 2.0 -- master tracker</t>
   </si>
@@ -520,6 +520,12 @@
     <t>Existing editor tests and Playwright editor specs pass</t>
   </si>
   <si>
+    <t>bb571a8</t>
+  </si>
+  <si>
+    <t>E0 plan: docs/SMARTDOC_2_0_EDITOR_ARCHITECTURE.md (awaiting owner review). Next: E1 shell behind ?editor=2.</t>
+  </si>
+  <si>
     <t>S2-040</t>
   </si>
   <si>
@@ -532,7 +538,13 @@
     <t>Round-trip tests; old documents unaffected; no schema migration</t>
   </si>
   <si>
-    <t>D-004, D-006</t>
+    <t>b7d004e</t>
+  </si>
+  <si>
+    <t>editor/design/model.test.ts 18</t>
+  </si>
+  <si>
+    <t>E3 foundation: pure design model (select/marquee, move+snap with guides, nudge, resize from handles with aspect/centre, rotate with 15° snap, stacking, add/duplicate/remove, bounded undo with one step per drag). Persistence waits for D-012.</t>
   </si>
   <si>
     <t>S2-060</t>
@@ -604,7 +616,16 @@
     <t>No hard-coded interface English left in those screens (a grep test); both languages rendered in their tests</t>
   </si>
   <si>
-    <t>Done: flow pieces (TrackedChangesChoice, ReferenceStyleSummary, JobProgressBar), account settings, password reset, confirm dialog, plan-limit banner, header, account menu, landing, projects list, batch bar, compare, billing. Next: templates library/editor. Editor chrome (editor/*) moves with the 2.0 editor rather than being translated twice. Server messages (API errors, version descriptions) stay in English until the API returns codes for them.</t>
+    <t>d1ec879, f9037ec, d8af836</t>
+  </si>
+  <si>
+    <t>see SESSION_STATE (checked after push)</t>
+  </si>
+  <si>
+    <t>i18n/hardcoded.test.ts: 29 screens with no literal interface English (TypeScript parser over JSX text and readable attributes); i18n/screens.bg.test.tsx 7 (screens rendered in Bulgarian); i18n.test.tsx (no empty text, same placeholders); Vitest 518; Playwright 66/1 skipped; browser BG docs/ui-review/2026-10-14b/</t>
+  </si>
+  <si>
+    <t>All non-editor screens + the flow's 1.x pieces + page titles (&lt;title&gt;) in en/bg; plural helper; numbers follow the interface language. Out of scope by decision: the 1.x editor chrome (editor/*) moves to the dictionaries with the 2.0 editor (E1/E2) instead of being translated twice; server messages (API errors, version descriptions, plan/unit labels from the API) stay English until the API returns codes -- billing units are already named by key.</t>
   </si>
   <si>
     <t>S2-018</t>
@@ -733,7 +754,52 @@
     <t>No zinc-* classes left in components (grep test); both themes checked in the browser</t>
   </si>
   <si>
-    <t>Same screens as S2-017, done together; compare now inside the app shell.</t>
+    <t>see SESSION_STATE</t>
+  </si>
+  <si>
+    <t>hardcoded.test.ts: no zinc-* in components/ or app/; browser light/dark docs/ui-review/2026-10-14b/</t>
+  </si>
+  <si>
+    <t>Compare now inside the app shell. White 'paper' scope (.paper) keeps sample pages dark-on-white in the dark theme (B-012). editor/* keeps its 1.x classes until the 2.0 editor shell.</t>
+  </si>
+  <si>
+    <t>S2-021</t>
+  </si>
+  <si>
+    <t>Look suggestion from the document's structure (M3.3)</t>
+  </si>
+  <si>
+    <t>The look step suggests a template from the document's own words and structure (title, headings, first 3,000 characters; tables, pictures, heading count) by built-in rules; shows the evidence; labelled 'not AI'; preselected only when there is no link choice and no workspace default.</t>
+  </si>
+  <si>
+    <t>Clear real-AI vs rules distinction; evidence shown; no suggestion when evidence is thin or tied; nothing applied until chosen; EN/BG</t>
+  </si>
+  <si>
+    <t>recommendLook.test.ts 8 (CV, contract, report+table, coursework, application, nothing clear, word starts, no template of the kind); DocumentFlow.test (suggestion region, reasons, 'not by AI', preselection); browser BG 1280 + dark 375</t>
+  </si>
+  <si>
+    <t>No server call, no cost. An AI second opinion (existing /style-analysis, metered) can be offered when a provider is configured -- D-007.</t>
+  </si>
+  <si>
+    <t>S2-022</t>
+  </si>
+  <si>
+    <t>Document flow UX corrections (owner review 2026-10-14)</t>
+  </si>
+  <si>
+    <t>Steps in the address (?step=&amp;doc=): browser Back/Forward and reload keep the place; step 1's text kept in the tab; going back offers the analysed draft instead of a second import; structure filter (all/headings/to check) and sticky actions; clear selected state for templates; compact phone layout (two-row action bar).</t>
+  </si>
+  <si>
+    <t>Back without losing content; reload on step 2/3 restores the draft; filter works; selected template unmistakable; no horizontal scroll at 375</t>
+  </si>
+  <si>
+    <t>bb571a8, d8af836</t>
+  </si>
+  <si>
+    <t>DocumentFlow.test 14 (back keeps text + no re-import, reload by id, filter, selected); browser: in-app Back, browser Back, reload on step 2 (docs/ui-review/2026-10-14b/)</t>
+  </si>
+  <si>
+    <t>Mobile action bar 190 -&gt; 117 px (B-015).</t>
   </si>
   <si>
     <t>Bug ID</t>
@@ -961,6 +1027,75 @@
     <t>Full backend suite green (T-013); tsc clean</t>
   </si>
   <si>
+    <t>B-012</t>
+  </si>
+  <si>
+    <t>Dark theme: look step / template library</t>
+  </si>
+  <si>
+    <t>Sample headings readable</t>
+  </si>
+  <si>
+    <t>Sample page headings took the interface's light text colour on white paper</t>
+  </si>
+  <si>
+    <t>.paper scope in globals.css on the sample pages (d8af836)</t>
+  </si>
+  <si>
+    <t>Browser: computed colour rgb(15,23,42) in dark; screenshots</t>
+  </si>
+  <si>
+    <t>B-013</t>
+  </si>
+  <si>
+    <t>Bulgarian interface: any settings/projects/templates page</t>
+  </si>
+  <si>
+    <t>Tab title in Bulgarian</t>
+  </si>
+  <si>
+    <t>&lt;title&gt; hard-coded in English</t>
+  </si>
+  <si>
+    <t>pageMetadata() from the dictionaries; layout default too (d8af836)</t>
+  </si>
+  <si>
+    <t>Browser: 'План и плащане · SmartDoc'</t>
+  </si>
+  <si>
+    <t>B-014</t>
+  </si>
+  <si>
+    <t>Look step / templates: built-in 'Академичен (по подразбиране)'</t>
+  </si>
+  <si>
+    <t>'Default' shown only for the actual default</t>
+  </si>
+  <si>
+    <t>The built-in template's own name contains '(по подразбиране)'</t>
+  </si>
+  <si>
+    <t>Rename the built-in in backend/app/formatting/builtin_templates.json (check tests and existing workspaces' references by id, not name)</t>
+  </si>
+  <si>
+    <t>B-015</t>
+  </si>
+  <si>
+    <t>Look step at 375 px</t>
+  </si>
+  <si>
+    <t>Choices visible</t>
+  </si>
+  <si>
+    <t>Three stacked full-width buttons took a quarter of the screen</t>
+  </si>
+  <si>
+    <t>Two-row bar (d8af836)</t>
+  </si>
+  <si>
+    <t>Browser: bar 117 px</t>
+  </si>
+  <si>
     <t>Test ID</t>
   </si>
   <si>
@@ -1219,6 +1354,33 @@
     <t>docs/ui-review/2026-10-14/create-*</t>
   </si>
   <si>
+    <t>T-020</t>
+  </si>
+  <si>
+    <t>Vitest + tsc + eslint (S2-017/R06, M3.3, wizard UX, design model, guards)</t>
+  </si>
+  <si>
+    <t>PASS 518 + guards 31 / tsc / eslint</t>
+  </si>
+  <si>
+    <t>T-021</t>
+  </si>
+  <si>
+    <t>Playwright full suite after the old screens and the flow changed</t>
+  </si>
+  <si>
+    <t>T-022</t>
+  </si>
+  <si>
+    <t>BG flow: structure, Back keeps text, browser Back, reload, suggestion; dark 375; projects/templates dark; billing/account light</t>
+  </si>
+  <si>
+    <t>PASS after B-012/B-013/B-015 fixes</t>
+  </si>
+  <si>
+    <t>docs/ui-review/2026-10-14b/</t>
+  </si>
+  <si>
     <t>Decision ID</t>
   </si>
   <si>
@@ -1355,6 +1517,18 @@
   </si>
   <si>
     <t>Process</t>
+  </si>
+  <si>
+    <t>D-012</t>
+  </si>
+  <si>
+    <t>Design-mode documents in the shared database</t>
+  </si>
+  <si>
+    <t>PENDING (owner): before any design document is written from the Preview, either a separate 2.0 database (recommended) or a 1.x change keeping unknown fields; 1.x would otherwise drop the canvas on save (pydantic extra=ignore, checked 2026-10-14)</t>
+  </si>
+  <si>
+    <t>P5 persistence</t>
   </si>
   <si>
     <t>Requirement</t>
@@ -2074,8 +2248,8 @@
         <v>5</v>
       </c>
       <c r="B5" s="5">
-        <f>COUNTIF(Tasks!$G$2:$G$25,A5)</f>
-        <v>4</v>
+        <f>COUNTIF(Tasks!$G$2:$G$27,A5)</f>
+        <v>2</v>
       </c>
       <c r="C5" s="5">
         <f>COUNTIF(Roadmap!$D$2:$D$10,A5)</f>
@@ -2087,7 +2261,7 @@
         <v>6</v>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF(Tasks!$G$2:$G$25,A6)</f>
+        <f>COUNTIF(Tasks!$G$2:$G$27,A6)</f>
         <v>0</v>
       </c>
       <c r="C6" s="5">
@@ -2100,7 +2274,7 @@
         <v>7</v>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF(Tasks!$G$2:$G$25,A7)</f>
+        <f>COUNTIF(Tasks!$G$2:$G$27,A7)</f>
         <v>2</v>
       </c>
       <c r="C7" s="5">
@@ -2113,7 +2287,7 @@
         <v>8</v>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF(Tasks!$G$2:$G$25,A8)</f>
+        <f>COUNTIF(Tasks!$G$2:$G$27,A8)</f>
         <v>0</v>
       </c>
       <c r="C8" s="5">
@@ -2126,7 +2300,7 @@
         <v>9</v>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIF(Tasks!$G$2:$G$25,A9)</f>
+        <f>COUNTIF(Tasks!$G$2:$G$27,A9)</f>
         <v>0</v>
       </c>
       <c r="C9" s="5">
@@ -2139,8 +2313,8 @@
         <v>10</v>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIF(Tasks!$G$2:$G$25,A10)</f>
-        <v>14</v>
+        <f>COUNTIF(Tasks!$G$2:$G$27,A10)</f>
+        <v>18</v>
       </c>
       <c r="C10" s="5">
         <f>COUNTIF(Roadmap!$D$2:$D$10,A10)</f>
@@ -2152,7 +2326,7 @@
         <v>11</v>
       </c>
       <c r="B11" s="5">
-        <f>COUNTIF(Tasks!$G$2:$G$25,A11)</f>
+        <f>COUNTIF(Tasks!$G$2:$G$27,A11)</f>
         <v>4</v>
       </c>
       <c r="C11" s="5">
@@ -2166,7 +2340,7 @@
       </c>
       <c r="B12" s="12">
         <f>SUM(B5:B11)</f>
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C12" s="12">
         <f>SUM(C5:C11)</f>
@@ -2179,7 +2353,7 @@
       </c>
       <c r="B13" s="14">
         <f>IFERROR((B11+B10)/B12,0)</f>
-        <v>0.75</v>
+        <v>0.84615384615384615</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -2187,7 +2361,7 @@
         <v>14</v>
       </c>
       <c r="B14">
-        <f>COUNTIFS(Tasks!$F$2:$F$25,"P0",Tasks!$G$2:$G$25,"&lt;&gt;DONE",Tasks!$G$2:$G$25,"&lt;&gt;VERIFIED")</f>
+        <f>COUNTIFS(Tasks!$F$2:$F$27,"P0",Tasks!$G$2:$G$27,"&lt;&gt;DONE",Tasks!$G$2:$G$27,"&lt;&gt;VERIFIED")</f>
         <v>0</v>
       </c>
     </row>
@@ -2196,8 +2370,8 @@
         <v>15</v>
       </c>
       <c r="B15">
-        <f>COUNTA(Bugs!$A$2:$A$12)-COUNTIF(Bugs!$F$2:$F$12,"DONE")-COUNTIF(Bugs!$F$2:$F$12,"VERIFIED")</f>
-        <v>2</v>
+        <f>COUNTA(Bugs!$A$2:$A$16)-COUNTIF(Bugs!$F$2:$F$16,"DONE")-COUNTIF(Bugs!$F$2:$F$16,"VERIFIED")</f>
+        <v>3</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
@@ -2451,7 +2625,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:P25"/>
+  <dimension ref="A1:P27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
@@ -3073,7 +3247,7 @@
         <v>26</v>
       </c>
       <c r="G13" s="17" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H13" s="17" t="s">
         <v>122</v>
@@ -3087,17 +3261,21 @@
       <c r="K13" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="L13" s="17"/>
+      <c r="L13" s="17" t="s">
+        <v>157</v>
+      </c>
       <c r="M13" s="17"/>
       <c r="N13" s="17"/>
       <c r="O13" s="17" t="s">
         <v>81</v>
       </c>
-      <c r="P13" s="17"/>
-    </row>
-    <row r="14" spans="1:16" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="P13" s="17" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B14" s="17" t="s">
         <v>42</v>
@@ -3106,22 +3284,22 @@
         <v>153</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="E14" s="17" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="F14" s="17" t="s">
         <v>26</v>
       </c>
       <c r="G14" s="17" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H14" s="17" t="s">
         <v>152</v>
       </c>
       <c r="I14" s="17" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="J14" s="17" t="s">
         <v>78</v>
@@ -3129,31 +3307,35 @@
       <c r="K14" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="L14" s="17"/>
+      <c r="L14" s="17" t="s">
+        <v>163</v>
+      </c>
       <c r="M14" s="17"/>
-      <c r="N14" s="17"/>
+      <c r="N14" s="17" t="s">
+        <v>164</v>
+      </c>
       <c r="O14" s="17" t="s">
         <v>81</v>
       </c>
       <c r="P14" s="17" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
     </row>
     <row r="15" spans="1:16" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A15" s="17" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="B15" s="17" t="s">
         <v>46</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="D15" s="17" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="E15" s="17" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="F15" s="17" t="s">
         <v>26</v>
@@ -3165,7 +3347,7 @@
         <v>152</v>
       </c>
       <c r="I15" s="17" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="J15" s="17" t="s">
         <v>78</v>
@@ -3180,24 +3362,24 @@
         <v>81</v>
       </c>
       <c r="P15" s="17" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
     </row>
     <row r="16" spans="1:16" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A16" s="17" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="B16" s="17" t="s">
         <v>51</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="D16" s="17" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="E16" s="17" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="F16" s="17" t="s">
         <v>26</v>
@@ -3209,7 +3391,7 @@
         <v>152</v>
       </c>
       <c r="I16" s="17" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="J16" s="17" t="s">
         <v>78</v>
@@ -3224,24 +3406,24 @@
         <v>81</v>
       </c>
       <c r="P16" s="17" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
     </row>
     <row r="17" spans="1:16" ht="127.5" x14ac:dyDescent="0.25">
       <c r="A17" s="17" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="B17" s="17" t="s">
         <v>30</v>
       </c>
       <c r="C17" s="17" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="D17" s="17" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="E17" s="17" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="F17" s="17" t="s">
         <v>22</v>
@@ -3253,7 +3435,7 @@
         <v>110</v>
       </c>
       <c r="I17" s="17" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="J17" s="17" t="s">
         <v>78</v>
@@ -3268,42 +3450,42 @@
         <v>135</v>
       </c>
       <c r="N17" s="17" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="O17" s="17" t="s">
         <v>81</v>
       </c>
       <c r="P17" s="17" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="18" spans="1:16" ht="114.75" x14ac:dyDescent="0.25">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" ht="178.5" x14ac:dyDescent="0.25">
       <c r="A18" s="17" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="B18" s="17" t="s">
         <v>30</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="D18" s="17" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="E18" s="17" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="F18" s="17" t="s">
         <v>26</v>
       </c>
       <c r="G18" s="17" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="H18" s="17" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="I18" s="17" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="J18" s="17" t="s">
         <v>78</v>
@@ -3311,19 +3493,25 @@
       <c r="K18" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="L18" s="17"/>
-      <c r="M18" s="17"/>
-      <c r="N18" s="17"/>
+      <c r="L18" s="17" t="s">
+        <v>189</v>
+      </c>
+      <c r="M18" s="17" t="s">
+        <v>190</v>
+      </c>
+      <c r="N18" s="17" t="s">
+        <v>191</v>
+      </c>
       <c r="O18" s="17" t="s">
         <v>81</v>
       </c>
       <c r="P18" s="17" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
     </row>
     <row r="19" spans="1:16" ht="165.75" x14ac:dyDescent="0.25">
       <c r="A19" s="17" t="s">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="B19" s="17" t="s">
         <v>30</v>
@@ -3332,10 +3520,10 @@
         <v>116</v>
       </c>
       <c r="D19" s="17" t="s">
-        <v>187</v>
+        <v>194</v>
       </c>
       <c r="E19" s="17" t="s">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="F19" s="17" t="s">
         <v>22</v>
@@ -3347,7 +3535,7 @@
         <v>130</v>
       </c>
       <c r="I19" s="17" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="J19" s="17" t="s">
         <v>78</v>
@@ -3356,24 +3544,24 @@
         <v>79</v>
       </c>
       <c r="L19" s="17" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="M19" s="17" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="N19" s="17" t="s">
-        <v>192</v>
+        <v>199</v>
       </c>
       <c r="O19" s="17" t="s">
         <v>81</v>
       </c>
       <c r="P19" s="17" t="s">
-        <v>193</v>
+        <v>200</v>
       </c>
     </row>
     <row r="20" spans="1:16" ht="102" x14ac:dyDescent="0.25">
       <c r="A20" s="17" t="s">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="B20" s="17" t="s">
         <v>30</v>
@@ -3382,10 +3570,10 @@
         <v>116</v>
       </c>
       <c r="D20" s="17" t="s">
-        <v>195</v>
+        <v>202</v>
       </c>
       <c r="E20" s="17" t="s">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="F20" s="17" t="s">
         <v>22</v>
@@ -3397,7 +3585,7 @@
         <v>110</v>
       </c>
       <c r="I20" s="17" t="s">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="J20" s="17" t="s">
         <v>78</v>
@@ -3406,24 +3594,24 @@
         <v>79</v>
       </c>
       <c r="L20" s="17" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="M20" s="17" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="N20" s="17" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="O20" s="17" t="s">
         <v>81</v>
       </c>
       <c r="P20" s="17" t="s">
-        <v>199</v>
+        <v>206</v>
       </c>
     </row>
     <row r="21" spans="1:16" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A21" s="17" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="B21" s="17" t="s">
         <v>30</v>
@@ -3432,10 +3620,10 @@
         <v>116</v>
       </c>
       <c r="D21" s="17" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="E21" s="17" t="s">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="F21" s="17" t="s">
         <v>22</v>
@@ -3447,7 +3635,7 @@
         <v>130</v>
       </c>
       <c r="I21" s="17" t="s">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="J21" s="17" t="s">
         <v>78</v>
@@ -3456,36 +3644,36 @@
         <v>79</v>
       </c>
       <c r="L21" s="17" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="M21" s="17" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="N21" s="17" t="s">
-        <v>204</v>
+        <v>211</v>
       </c>
       <c r="O21" s="17" t="s">
         <v>81</v>
       </c>
       <c r="P21" s="17" t="s">
-        <v>205</v>
+        <v>212</v>
       </c>
     </row>
     <row r="22" spans="1:16" ht="51" x14ac:dyDescent="0.25">
       <c r="A22" s="17" t="s">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="B22" s="17" t="s">
         <v>30</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="D22" s="17" t="s">
-        <v>207</v>
+        <v>214</v>
       </c>
       <c r="E22" s="17" t="s">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="F22" s="17" t="s">
         <v>26</v>
@@ -3497,7 +3685,7 @@
         <v>122</v>
       </c>
       <c r="I22" s="17" t="s">
-        <v>209</v>
+        <v>216</v>
       </c>
       <c r="J22" s="17" t="s">
         <v>78</v>
@@ -3506,24 +3694,24 @@
         <v>79</v>
       </c>
       <c r="L22" s="17" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="M22" s="17" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="N22" s="17" t="s">
-        <v>210</v>
+        <v>217</v>
       </c>
       <c r="O22" s="17" t="s">
         <v>81</v>
       </c>
       <c r="P22" s="17" t="s">
-        <v>211</v>
+        <v>218</v>
       </c>
     </row>
     <row r="23" spans="1:16" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A23" s="17" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="B23" s="17" t="s">
         <v>30</v>
@@ -3532,10 +3720,10 @@
         <v>116</v>
       </c>
       <c r="D23" s="17" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="E23" s="17" t="s">
-        <v>214</v>
+        <v>221</v>
       </c>
       <c r="F23" s="17" t="s">
         <v>26</v>
@@ -3547,7 +3735,7 @@
         <v>122</v>
       </c>
       <c r="I23" s="17" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="J23" s="17" t="s">
         <v>78</v>
@@ -3556,24 +3744,24 @@
         <v>79</v>
       </c>
       <c r="L23" s="17" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="M23" s="17" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="N23" s="17" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
       <c r="O23" s="17" t="s">
         <v>81</v>
       </c>
       <c r="P23" s="17" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
     </row>
     <row r="24" spans="1:16" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A24" s="17" t="s">
-        <v>218</v>
+        <v>225</v>
       </c>
       <c r="B24" s="17" t="s">
         <v>30</v>
@@ -3582,10 +3770,10 @@
         <v>116</v>
       </c>
       <c r="D24" s="17" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
       <c r="E24" s="17" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="F24" s="17" t="s">
         <v>26</v>
@@ -3594,10 +3782,10 @@
         <v>10</v>
       </c>
       <c r="H24" s="17" t="s">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="I24" s="17" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="J24" s="17" t="s">
         <v>78</v>
@@ -3606,24 +3794,24 @@
         <v>79</v>
       </c>
       <c r="L24" s="17" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="M24" s="17" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="N24" s="17" t="s">
-        <v>222</v>
+        <v>229</v>
       </c>
       <c r="O24" s="17" t="s">
         <v>81</v>
       </c>
       <c r="P24" s="17" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="25" spans="1:16" ht="38.25" x14ac:dyDescent="0.25">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" ht="51" x14ac:dyDescent="0.25">
       <c r="A25" s="17" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="B25" s="17" t="s">
         <v>30</v>
@@ -3632,22 +3820,22 @@
         <v>116</v>
       </c>
       <c r="D25" s="17" t="s">
-        <v>225</v>
+        <v>232</v>
       </c>
       <c r="E25" s="17" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="F25" s="17" t="s">
         <v>30</v>
       </c>
       <c r="G25" s="17" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="H25" s="17" t="s">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="I25" s="17" t="s">
-        <v>227</v>
+        <v>234</v>
       </c>
       <c r="J25" s="17" t="s">
         <v>78</v>
@@ -3655,19 +3843,125 @@
       <c r="K25" s="17" t="s">
         <v>79</v>
       </c>
-      <c r="L25" s="17"/>
-      <c r="M25" s="17"/>
-      <c r="N25" s="17"/>
+      <c r="L25" s="17" t="s">
+        <v>189</v>
+      </c>
+      <c r="M25" s="17" t="s">
+        <v>235</v>
+      </c>
+      <c r="N25" s="17" t="s">
+        <v>236</v>
+      </c>
       <c r="O25" s="17" t="s">
         <v>81</v>
       </c>
       <c r="P25" s="17" t="s">
-        <v>228</v>
+        <v>237</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" ht="127.5" x14ac:dyDescent="0.25">
+      <c r="A26" s="17" t="s">
+        <v>238</v>
+      </c>
+      <c r="B26" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="C26" s="17" t="s">
+        <v>116</v>
+      </c>
+      <c r="D26" s="17" t="s">
+        <v>239</v>
+      </c>
+      <c r="E26" s="17" t="s">
+        <v>240</v>
+      </c>
+      <c r="F26" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="G26" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="H26" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="I26" s="17" t="s">
+        <v>241</v>
+      </c>
+      <c r="J26" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="K26" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="L26" s="17" t="s">
+        <v>157</v>
+      </c>
+      <c r="M26" s="17" t="s">
+        <v>235</v>
+      </c>
+      <c r="N26" s="17" t="s">
+        <v>242</v>
+      </c>
+      <c r="O26" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="P26" s="17" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" ht="89.25" x14ac:dyDescent="0.25">
+      <c r="A27" s="17" t="s">
+        <v>244</v>
+      </c>
+      <c r="B27" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="C27" s="17" t="s">
+        <v>116</v>
+      </c>
+      <c r="D27" s="17" t="s">
+        <v>245</v>
+      </c>
+      <c r="E27" s="17" t="s">
+        <v>246</v>
+      </c>
+      <c r="F27" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="G27" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="H27" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="I27" s="17" t="s">
+        <v>247</v>
+      </c>
+      <c r="J27" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="K27" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="L27" s="17" t="s">
+        <v>248</v>
+      </c>
+      <c r="M27" s="17" t="s">
+        <v>235</v>
+      </c>
+      <c r="N27" s="17" t="s">
+        <v>249</v>
+      </c>
+      <c r="O27" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="P27" s="17" t="s">
+        <v>250</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P25" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
-  <conditionalFormatting sqref="G2:G25">
+  <autoFilter ref="A1:P27" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
+  <conditionalFormatting sqref="G2:G27">
     <cfRule type="expression" dxfId="13" priority="1">
       <formula>$G2="BACKLOG"</formula>
     </cfRule>
@@ -3696,7 +3990,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -3711,317 +4005,419 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>229</v>
+        <v>251</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>230</v>
+        <v>252</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>231</v>
+        <v>253</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>232</v>
+        <v>254</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>233</v>
+        <v>255</v>
       </c>
       <c r="F1" s="16" t="s">
         <v>2</v>
       </c>
       <c r="G1" s="16" t="s">
-        <v>234</v>
+        <v>256</v>
       </c>
       <c r="H1" s="16" t="s">
-        <v>235</v>
+        <v>257</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
-        <v>236</v>
+        <v>258</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>237</v>
+        <v>259</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>238</v>
+        <v>260</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>239</v>
+        <v>261</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>240</v>
+        <v>262</v>
       </c>
       <c r="F2" s="17" t="s">
         <v>8</v>
       </c>
       <c r="G2" s="17" t="s">
-        <v>241</v>
+        <v>263</v>
       </c>
       <c r="H2" s="17" t="s">
-        <v>242</v>
+        <v>264</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
-        <v>243</v>
+        <v>265</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>244</v>
+        <v>266</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>245</v>
+        <v>267</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>246</v>
+        <v>268</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>247</v>
+        <v>269</v>
       </c>
       <c r="F3" s="17" t="s">
         <v>5</v>
       </c>
       <c r="G3" s="17"/>
       <c r="H3" s="17" t="s">
-        <v>248</v>
+        <v>270</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>249</v>
+        <v>271</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>244</v>
+        <v>266</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>250</v>
+        <v>272</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>251</v>
+        <v>273</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>252</v>
+        <v>274</v>
       </c>
       <c r="F4" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G4" s="17" t="s">
-        <v>253</v>
+        <v>275</v>
       </c>
       <c r="H4" s="17" t="s">
-        <v>254</v>
+        <v>276</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>255</v>
+        <v>277</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>256</v>
+        <v>278</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>257</v>
+        <v>279</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>258</v>
+        <v>280</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>259</v>
+        <v>281</v>
       </c>
       <c r="F5" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G5" s="17" t="s">
-        <v>260</v>
+        <v>282</v>
       </c>
       <c r="H5" s="17" t="s">
-        <v>261</v>
+        <v>283</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="51" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
-        <v>262</v>
+        <v>284</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>256</v>
+        <v>278</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>263</v>
+        <v>285</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>264</v>
+        <v>286</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>265</v>
+        <v>287</v>
       </c>
       <c r="F6" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G6" s="17" t="s">
-        <v>266</v>
+        <v>288</v>
       </c>
       <c r="H6" s="17" t="s">
-        <v>267</v>
+        <v>289</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
-        <v>268</v>
+        <v>290</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>256</v>
+        <v>278</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>269</v>
+        <v>291</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>270</v>
+        <v>292</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>271</v>
+        <v>293</v>
       </c>
       <c r="F7" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G7" s="17" t="s">
-        <v>272</v>
+        <v>294</v>
       </c>
       <c r="H7" s="17" t="s">
-        <v>273</v>
+        <v>295</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
-        <v>274</v>
+        <v>296</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>244</v>
+        <v>266</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>275</v>
+        <v>297</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>276</v>
+        <v>298</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>277</v>
+        <v>299</v>
       </c>
       <c r="F8" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G8" s="17" t="s">
-        <v>278</v>
+        <v>300</v>
       </c>
       <c r="H8" s="17" t="s">
-        <v>279</v>
+        <v>301</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="51" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
-        <v>280</v>
+        <v>302</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>244</v>
+        <v>266</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>281</v>
+        <v>303</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>282</v>
+        <v>304</v>
       </c>
       <c r="E9" s="17" t="s">
-        <v>283</v>
+        <v>305</v>
       </c>
       <c r="F9" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G9" s="17" t="s">
-        <v>284</v>
+        <v>306</v>
       </c>
       <c r="H9" s="17" t="s">
-        <v>285</v>
+        <v>307</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="51" x14ac:dyDescent="0.25">
       <c r="A10" s="17" t="s">
-        <v>286</v>
+        <v>308</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>244</v>
+        <v>266</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>287</v>
+        <v>309</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>288</v>
+        <v>310</v>
       </c>
       <c r="E10" s="17" t="s">
-        <v>289</v>
+        <v>311</v>
       </c>
       <c r="F10" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G10" s="17" t="s">
-        <v>290</v>
+        <v>312</v>
       </c>
       <c r="H10" s="17" t="s">
-        <v>291</v>
+        <v>313</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A11" s="17" t="s">
-        <v>292</v>
+        <v>314</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>244</v>
+        <v>266</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>293</v>
+        <v>315</v>
       </c>
       <c r="D11" s="17" t="s">
-        <v>294</v>
+        <v>316</v>
       </c>
       <c r="E11" s="17" t="s">
-        <v>295</v>
+        <v>317</v>
       </c>
       <c r="F11" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G11" s="17" t="s">
-        <v>296</v>
+        <v>318</v>
       </c>
       <c r="H11" s="17" t="s">
-        <v>297</v>
+        <v>319</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
-        <v>298</v>
+        <v>320</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>256</v>
+        <v>278</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>299</v>
+        <v>321</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>300</v>
+        <v>322</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>301</v>
+        <v>323</v>
       </c>
       <c r="F12" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G12" s="17" t="s">
-        <v>302</v>
+        <v>324</v>
       </c>
       <c r="H12" s="17" t="s">
-        <v>303</v>
+        <v>325</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="51" x14ac:dyDescent="0.25">
+      <c r="A13" s="17" t="s">
+        <v>326</v>
+      </c>
+      <c r="B13" s="17" t="s">
+        <v>278</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>327</v>
+      </c>
+      <c r="D13" s="17" t="s">
+        <v>328</v>
+      </c>
+      <c r="E13" s="17" t="s">
+        <v>329</v>
+      </c>
+      <c r="F13" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="G13" s="17" t="s">
+        <v>330</v>
+      </c>
+      <c r="H13" s="17" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="51" x14ac:dyDescent="0.25">
+      <c r="A14" s="17" t="s">
+        <v>332</v>
+      </c>
+      <c r="B14" s="17" t="s">
+        <v>266</v>
+      </c>
+      <c r="C14" s="17" t="s">
+        <v>333</v>
+      </c>
+      <c r="D14" s="17" t="s">
+        <v>334</v>
+      </c>
+      <c r="E14" s="17" t="s">
+        <v>335</v>
+      </c>
+      <c r="F14" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="G14" s="17" t="s">
+        <v>336</v>
+      </c>
+      <c r="H14" s="17" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="114.75" x14ac:dyDescent="0.25">
+      <c r="A15" s="17" t="s">
+        <v>338</v>
+      </c>
+      <c r="B15" s="17" t="s">
+        <v>266</v>
+      </c>
+      <c r="C15" s="17" t="s">
+        <v>339</v>
+      </c>
+      <c r="D15" s="17" t="s">
+        <v>340</v>
+      </c>
+      <c r="E15" s="17" t="s">
+        <v>341</v>
+      </c>
+      <c r="F15" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="G15" s="17" t="s">
+        <v>342</v>
+      </c>
+      <c r="H15" s="17"/>
+    </row>
+    <row r="16" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A16" s="17" t="s">
+        <v>343</v>
+      </c>
+      <c r="B16" s="17" t="s">
+        <v>266</v>
+      </c>
+      <c r="C16" s="17" t="s">
+        <v>344</v>
+      </c>
+      <c r="D16" s="17" t="s">
+        <v>345</v>
+      </c>
+      <c r="E16" s="17" t="s">
+        <v>346</v>
+      </c>
+      <c r="F16" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="G16" s="17" t="s">
+        <v>347</v>
+      </c>
+      <c r="H16" s="17" t="s">
+        <v>348</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H12" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
-  <conditionalFormatting sqref="F2:F12">
+  <autoFilter ref="A1:H16" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
+  <conditionalFormatting sqref="F2:F16">
     <cfRule type="expression" dxfId="6" priority="1">
       <formula>$F2="BACKLOG"</formula>
     </cfRule>
@@ -4050,7 +4446,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -4064,226 +4460,226 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>304</v>
+        <v>349</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>305</v>
+        <v>350</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>306</v>
+        <v>351</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>307</v>
+        <v>352</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>308</v>
+        <v>353</v>
       </c>
       <c r="F1" s="16" t="s">
-        <v>309</v>
+        <v>354</v>
       </c>
       <c r="G1" s="16" t="s">
-        <v>310</v>
+        <v>355</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
-        <v>311</v>
+        <v>356</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>312</v>
+        <v>357</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>313</v>
+        <v>358</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>314</v>
+        <v>359</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>315</v>
+        <v>360</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>316</v>
+        <v>361</v>
       </c>
       <c r="G2" s="17" t="s">
-        <v>317</v>
+        <v>362</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
-        <v>318</v>
+        <v>363</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>319</v>
+        <v>364</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>320</v>
+        <v>365</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>314</v>
+        <v>359</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>321</v>
+        <v>366</v>
       </c>
       <c r="F3" s="17" t="s">
-        <v>322</v>
+        <v>367</v>
       </c>
       <c r="G3" s="17" t="s">
-        <v>317</v>
+        <v>362</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>323</v>
+        <v>368</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>324</v>
+        <v>369</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>325</v>
+        <v>370</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>314</v>
+        <v>359</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>326</v>
+        <v>371</v>
       </c>
       <c r="F4" s="17" t="s">
-        <v>327</v>
+        <v>372</v>
       </c>
       <c r="G4" s="17" t="s">
-        <v>317</v>
+        <v>362</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>328</v>
+        <v>373</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>329</v>
+        <v>374</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>330</v>
+        <v>375</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>331</v>
+        <v>376</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>332</v>
+        <v>377</v>
       </c>
       <c r="F5" s="17" t="s">
-        <v>333</v>
+        <v>378</v>
       </c>
       <c r="G5" s="17" t="s">
-        <v>317</v>
+        <v>362</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
-        <v>334</v>
+        <v>379</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>319</v>
+        <v>364</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>335</v>
+        <v>380</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>314</v>
+        <v>359</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>336</v>
+        <v>381</v>
       </c>
       <c r="F6" s="17" t="s">
         <v>126</v>
       </c>
       <c r="G6" s="17" t="s">
-        <v>317</v>
+        <v>362</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
-        <v>337</v>
+        <v>382</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>324</v>
+        <v>369</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>338</v>
+        <v>383</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>314</v>
+        <v>359</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>339</v>
+        <v>384</v>
       </c>
       <c r="F7" s="17" t="s">
         <v>126</v>
       </c>
       <c r="G7" s="17" t="s">
-        <v>317</v>
+        <v>362</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
-        <v>340</v>
+        <v>385</v>
       </c>
       <c r="B8" s="17" t="s">
         <v>116</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>341</v>
+        <v>386</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>342</v>
+        <v>387</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>332</v>
+        <v>377</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>343</v>
+        <v>388</v>
       </c>
       <c r="G8" s="17" t="s">
-        <v>317</v>
+        <v>362</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
-        <v>344</v>
+        <v>389</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>345</v>
+        <v>390</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>346</v>
+        <v>391</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>347</v>
+        <v>392</v>
       </c>
       <c r="E9" s="17" t="s">
-        <v>348</v>
+        <v>393</v>
       </c>
       <c r="F9" s="17" t="s">
-        <v>349</v>
+        <v>394</v>
       </c>
       <c r="G9" s="17" t="s">
-        <v>317</v>
+        <v>362</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="17" t="s">
-        <v>350</v>
+        <v>395</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>319</v>
+        <v>364</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>335</v>
+        <v>380</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>314</v>
+        <v>359</v>
       </c>
       <c r="E10" s="17" t="s">
-        <v>351</v>
+        <v>396</v>
       </c>
       <c r="F10" s="17" t="s">
         <v>134</v>
@@ -4294,19 +4690,19 @@
     </row>
     <row r="11" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A11" s="17" t="s">
-        <v>352</v>
+        <v>397</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>324</v>
+        <v>369</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>353</v>
+        <v>398</v>
       </c>
       <c r="D11" s="17" t="s">
-        <v>354</v>
+        <v>399</v>
       </c>
       <c r="E11" s="17" t="s">
-        <v>355</v>
+        <v>400</v>
       </c>
       <c r="F11" s="17" t="s">
         <v>134</v>
@@ -4317,22 +4713,22 @@
     </row>
     <row r="12" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
-        <v>356</v>
+        <v>401</v>
       </c>
       <c r="B12" s="17" t="s">
         <v>116</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>357</v>
+        <v>402</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>342</v>
+        <v>387</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>358</v>
+        <v>403</v>
       </c>
       <c r="F12" s="17" t="s">
-        <v>343</v>
+        <v>388</v>
       </c>
       <c r="G12" s="17" t="s">
         <v>81</v>
@@ -4340,22 +4736,22 @@
     </row>
     <row r="13" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A13" s="17" t="s">
-        <v>359</v>
+        <v>404</v>
       </c>
       <c r="B13" s="17" t="s">
-        <v>345</v>
+        <v>390</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>346</v>
+        <v>391</v>
       </c>
       <c r="D13" s="17" t="s">
-        <v>347</v>
+        <v>392</v>
       </c>
       <c r="E13" s="17" t="s">
-        <v>360</v>
+        <v>405</v>
       </c>
       <c r="F13" s="17" t="s">
-        <v>361</v>
+        <v>406</v>
       </c>
       <c r="G13" s="17" t="s">
         <v>81</v>
@@ -4363,22 +4759,22 @@
     </row>
     <row r="14" spans="1:7" ht="51" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
-        <v>362</v>
+        <v>407</v>
       </c>
       <c r="B14" s="17" t="s">
-        <v>312</v>
+        <v>357</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>363</v>
+        <v>408</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>314</v>
+        <v>359</v>
       </c>
       <c r="E14" s="17" t="s">
-        <v>364</v>
+        <v>409</v>
       </c>
       <c r="F14" s="17" t="s">
-        <v>365</v>
+        <v>410</v>
       </c>
       <c r="G14" s="17" t="s">
         <v>81</v>
@@ -4386,22 +4782,22 @@
     </row>
     <row r="15" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A15" s="17" t="s">
-        <v>366</v>
+        <v>411</v>
       </c>
       <c r="B15" s="17" t="s">
-        <v>319</v>
+        <v>364</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>367</v>
+        <v>412</v>
       </c>
       <c r="D15" s="17" t="s">
-        <v>314</v>
+        <v>359</v>
       </c>
       <c r="E15" s="17" t="s">
-        <v>368</v>
+        <v>413</v>
       </c>
       <c r="F15" s="17" t="s">
-        <v>369</v>
+        <v>414</v>
       </c>
       <c r="G15" s="17" t="s">
         <v>81</v>
@@ -4409,22 +4805,22 @@
     </row>
     <row r="16" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A16" s="17" t="s">
-        <v>370</v>
+        <v>415</v>
       </c>
       <c r="B16" s="17" t="s">
-        <v>324</v>
+        <v>369</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>371</v>
+        <v>416</v>
       </c>
       <c r="D16" s="17" t="s">
-        <v>314</v>
+        <v>359</v>
       </c>
       <c r="E16" s="17" t="s">
-        <v>372</v>
+        <v>417</v>
       </c>
       <c r="F16" s="17" t="s">
-        <v>373</v>
+        <v>418</v>
       </c>
       <c r="G16" s="17" t="s">
         <v>81</v>
@@ -4432,22 +4828,22 @@
     </row>
     <row r="17" spans="1:7" ht="51" x14ac:dyDescent="0.25">
       <c r="A17" s="17" t="s">
-        <v>374</v>
+        <v>419</v>
       </c>
       <c r="B17" s="17" t="s">
-        <v>375</v>
+        <v>420</v>
       </c>
       <c r="C17" s="17" t="s">
-        <v>376</v>
+        <v>421</v>
       </c>
       <c r="D17" s="17" t="s">
-        <v>342</v>
+        <v>387</v>
       </c>
       <c r="E17" s="17" t="s">
-        <v>377</v>
+        <v>422</v>
       </c>
       <c r="F17" s="17" t="s">
-        <v>378</v>
+        <v>423</v>
       </c>
       <c r="G17" s="17" t="s">
         <v>81</v>
@@ -4455,22 +4851,22 @@
     </row>
     <row r="18" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A18" s="17" t="s">
-        <v>379</v>
+        <v>424</v>
       </c>
       <c r="B18" s="17" t="s">
-        <v>319</v>
+        <v>364</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>380</v>
+        <v>425</v>
       </c>
       <c r="D18" s="17" t="s">
-        <v>314</v>
+        <v>359</v>
       </c>
       <c r="E18" s="17" t="s">
-        <v>381</v>
+        <v>426</v>
       </c>
       <c r="F18" s="17" t="s">
-        <v>382</v>
+        <v>427</v>
       </c>
       <c r="G18" s="17" t="s">
         <v>81</v>
@@ -4478,22 +4874,22 @@
     </row>
     <row r="19" spans="1:7" ht="51" x14ac:dyDescent="0.25">
       <c r="A19" s="17" t="s">
-        <v>383</v>
+        <v>428</v>
       </c>
       <c r="B19" s="17" t="s">
-        <v>324</v>
+        <v>369</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>384</v>
+        <v>429</v>
       </c>
       <c r="D19" s="17" t="s">
-        <v>314</v>
+        <v>359</v>
       </c>
       <c r="E19" s="17" t="s">
-        <v>385</v>
+        <v>430</v>
       </c>
       <c r="F19" s="17" t="s">
-        <v>373</v>
+        <v>418</v>
       </c>
       <c r="G19" s="17" t="s">
         <v>81</v>
@@ -4501,36 +4897,105 @@
     </row>
     <row r="20" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A20" s="17" t="s">
-        <v>386</v>
+        <v>431</v>
       </c>
       <c r="B20" s="17" t="s">
-        <v>375</v>
+        <v>420</v>
       </c>
       <c r="C20" s="17" t="s">
+        <v>432</v>
+      </c>
+      <c r="D20" s="17" t="s">
         <v>387</v>
       </c>
-      <c r="D20" s="17" t="s">
-        <v>342</v>
-      </c>
       <c r="E20" s="17" t="s">
-        <v>388</v>
+        <v>433</v>
       </c>
       <c r="F20" s="17" t="s">
-        <v>389</v>
+        <v>434</v>
       </c>
       <c r="G20" s="17" t="s">
         <v>81</v>
       </c>
     </row>
+    <row r="21" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A21" s="17" t="s">
+        <v>435</v>
+      </c>
+      <c r="B21" s="17" t="s">
+        <v>364</v>
+      </c>
+      <c r="C21" s="17" t="s">
+        <v>436</v>
+      </c>
+      <c r="D21" s="17" t="s">
+        <v>359</v>
+      </c>
+      <c r="E21" s="17" t="s">
+        <v>437</v>
+      </c>
+      <c r="F21" s="17" t="s">
+        <v>427</v>
+      </c>
+      <c r="G21" s="17" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A22" s="17" t="s">
+        <v>438</v>
+      </c>
+      <c r="B22" s="17" t="s">
+        <v>369</v>
+      </c>
+      <c r="C22" s="17" t="s">
+        <v>439</v>
+      </c>
+      <c r="D22" s="17" t="s">
+        <v>359</v>
+      </c>
+      <c r="E22" s="17" t="s">
+        <v>417</v>
+      </c>
+      <c r="F22" s="17" t="s">
+        <v>418</v>
+      </c>
+      <c r="G22" s="17" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A23" s="17" t="s">
+        <v>440</v>
+      </c>
+      <c r="B23" s="17" t="s">
+        <v>420</v>
+      </c>
+      <c r="C23" s="17" t="s">
+        <v>441</v>
+      </c>
+      <c r="D23" s="17" t="s">
+        <v>387</v>
+      </c>
+      <c r="E23" s="17" t="s">
+        <v>442</v>
+      </c>
+      <c r="F23" s="17" t="s">
+        <v>443</v>
+      </c>
+      <c r="G23" s="17" t="s">
+        <v>81</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G20" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
+  <autoFilter ref="A1:G23" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -4542,39 +5007,39 @@
   <sheetData>
     <row r="1" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>390</v>
+        <v>444</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>391</v>
+        <v>445</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>392</v>
+        <v>446</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>310</v>
+        <v>355</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>393</v>
+        <v>447</v>
       </c>
       <c r="F1" s="16" t="s">
-        <v>394</v>
+        <v>448</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
-        <v>395</v>
+        <v>449</v>
       </c>
       <c r="B2" s="17" t="s">
         <v>67</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>396</v>
+        <v>450</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>317</v>
+        <v>362</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>397</v>
+        <v>451</v>
       </c>
       <c r="F2" s="17" t="s">
         <v>83</v>
@@ -4582,19 +5047,19 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
-        <v>398</v>
+        <v>452</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>399</v>
+        <v>453</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>400</v>
+        <v>454</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>317</v>
+        <v>362</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>401</v>
+        <v>455</v>
       </c>
       <c r="F3" s="17" t="s">
         <v>83</v>
@@ -4602,56 +5067,56 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>402</v>
+        <v>456</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>403</v>
+        <v>457</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>404</v>
+        <v>458</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>317</v>
+        <v>362</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>405</v>
+        <v>459</v>
       </c>
       <c r="F4" s="17" t="s">
-        <v>406</v>
+        <v>460</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>407</v>
+        <v>461</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>408</v>
+        <v>462</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>409</v>
+        <v>463</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>317</v>
+        <v>362</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>410</v>
+        <v>464</v>
       </c>
       <c r="F5" s="17" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
-        <v>411</v>
+        <v>465</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>412</v>
+        <v>466</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>413</v>
+        <v>467</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>317</v>
+        <v>362</v>
       </c>
       <c r="E6" s="17" t="s">
         <v>26</v>
@@ -4662,126 +5127,146 @@
     </row>
     <row r="7" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
-        <v>414</v>
+        <v>468</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>415</v>
+        <v>469</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>416</v>
+        <v>470</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>317</v>
+        <v>362</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>417</v>
+        <v>471</v>
       </c>
       <c r="F7" s="17" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
-        <v>418</v>
+        <v>472</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>419</v>
+        <v>473</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>420</v>
+        <v>474</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>317</v>
+        <v>362</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>421</v>
+        <v>475</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>422</v>
+        <v>476</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>423</v>
+        <v>477</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>424</v>
+        <v>478</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>317</v>
+        <v>362</v>
       </c>
       <c r="E9" s="17" t="s">
-        <v>421</v>
+        <v>475</v>
       </c>
       <c r="F9" s="17" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="17" t="s">
-        <v>425</v>
+        <v>479</v>
       </c>
       <c r="B10" s="17" t="s">
         <v>52</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>426</v>
+        <v>480</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>317</v>
+        <v>362</v>
       </c>
       <c r="E10" s="17" t="s">
         <v>51</v>
       </c>
       <c r="F10" s="17" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="51" x14ac:dyDescent="0.25">
       <c r="A11" s="17" t="s">
-        <v>427</v>
+        <v>481</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>428</v>
+        <v>482</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>429</v>
+        <v>483</v>
       </c>
       <c r="D11" s="17" t="s">
         <v>81</v>
       </c>
       <c r="E11" s="17" t="s">
-        <v>430</v>
+        <v>484</v>
       </c>
       <c r="F11" s="17" t="s">
-        <v>431</v>
+        <v>485</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
-        <v>432</v>
+        <v>486</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>433</v>
+        <v>487</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>434</v>
+        <v>488</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>317</v>
+        <v>362</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>435</v>
+        <v>489</v>
       </c>
       <c r="F12" s="17" t="s">
         <v>96</v>
       </c>
     </row>
+    <row r="13" spans="1:6" ht="51" x14ac:dyDescent="0.25">
+      <c r="A13" s="17" t="s">
+        <v>490</v>
+      </c>
+      <c r="B13" s="17" t="s">
+        <v>491</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>492</v>
+      </c>
+      <c r="D13" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="E13" s="17" t="s">
+        <v>493</v>
+      </c>
+      <c r="F13" s="17" t="s">
+        <v>159</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F12" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
+  <autoFilter ref="A1:F13" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4800,121 +5285,121 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>436</v>
+        <v>494</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>437</v>
+        <v>495</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>438</v>
+        <v>496</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>439</v>
+        <v>497</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>440</v>
+        <v>498</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
-        <v>441</v>
+        <v>499</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>442</v>
+        <v>500</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>443</v>
+        <v>501</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>444</v>
+        <v>502</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>445</v>
+        <v>503</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
-        <v>446</v>
+        <v>504</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>447</v>
+        <v>505</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>448</v>
+        <v>506</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>449</v>
+        <v>507</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>450</v>
+        <v>508</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>451</v>
+        <v>509</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>452</v>
+        <v>510</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>452</v>
+        <v>510</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>453</v>
+        <v>511</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>454</v>
+        <v>512</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>455</v>
+        <v>513</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>456</v>
+        <v>514</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>457</v>
+        <v>515</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>458</v>
+        <v>516</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>450</v>
+        <v>508</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
-        <v>459</v>
+        <v>517</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>460</v>
+        <v>518</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>460</v>
+        <v>518</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>461</v>
+        <v>519</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>445</v>
+        <v>503</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
-        <v>462</v>
+        <v>520</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>463</v>
+        <v>521</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>464</v>
+        <v>522</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>465</v>
+        <v>523</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>445</v>
+        <v>503</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
SmartDoc 2.0 tracker/checkpoint: E1 verified, S2-050 planned (blocked on approval), new UX tasks
S2-030 (E1 shell) VERIFIED with tests; S2-050 Preview isolation BLOCKED on
the owner's approval; S2-023/S2-024/S2-025 backlog from the review;
B-014 and B-016 verified; D-012 decided (a); T-023..T-026; session state:
next is E2.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/SMARTDOC_2_0_MASTER_TRACKER.xlsx
+++ b/docs/SMARTDOC_2_0_MASTER_TRACKER.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\speed\Desktop\Claude - ПРОЕКТ\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80BE36E1-27F4-49EE-8824-FD2F00BA357C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64122817-C1AD-467B-B184-3CA9EB38FA90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,12 +22,12 @@
     <sheet name="Release Readiness" sheetId="7" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Bugs!$A$1:$H$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Bugs!$A$1:$H$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Decisions!$A$1:$F$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Release Readiness'!$A$1:$E$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Roadmap!$A$1:$F$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Tasks!$A$1:$P$27</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Tests!$A$1:$G$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Tasks!$A$1:$P$31</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Tests!$A$1:$G$27</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="890" uniqueCount="524">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="982" uniqueCount="569">
   <si>
     <t>SmartDoc 2.0 -- master tracker</t>
   </si>
@@ -511,270 +511,276 @@
     <t>EDITOR</t>
   </si>
   <si>
-    <t>Editor layout v2 (screen 7, Document Mode)</t>
+    <t>Editor 2.0 shell, E1 (Document Mode, behind ?editor=2)</t>
   </si>
   <si>
     <t>Left (outline/pages/elements), center canvas, top contextual toolbar, right properties, collapsible AI panel; reuses the existing Tiptap editor modules.</t>
   </si>
   <si>
-    <t>Existing editor tests and Playwright editor specs pass</t>
+    <t>Same text engine and DOCX/PDF export; top bar, side panels, large central area, text tools, save state; EN/BG; light/dark; classic stays default; existing documents, import, export, undo/redo, autosave and save errors tested</t>
+  </si>
+  <si>
+    <t>b85cc79</t>
+  </si>
+  <si>
+    <t>see SESSION_STATE</t>
+  </si>
+  <si>
+    <t>e2e/editor-v2.spec.ts 8 (classic default + ?editor=2 on the same document, typing PATCH + reload, undo/redo from the top bar persisted, templates + formatting undo/redo, DOCX/PDF export with read-back, imported DOCX identical text, failed save -&gt; 'Not saved' -&gt; Retry -&gt; saved, Bulgarian); axe on the 2.0 shell light/dark/panel; all 66 classic specs green (74/1 skipped); browser docs/ui-review/2026-10-14c/</t>
+  </si>
+  <si>
+    <t>useEditorEngine: the 1.x shell's wiring moved verbatim into one hook used by both shells (classic markup unchanged). 2.0 shell: top bar (Projects, title, save state, undo/redo of typing, preview badge -&gt; classic, properties toggle, export), 84-px rail with 9 panels, one panel open, text tools above the pages, white paper in both themes (EditorCanvas paper prop, opt-in), properties panel (Edit/Styles). Measured at 1440: pages 75% of the width with properties only, ~57% with a left panel too. Phones: rail as a drawer; 1.x action/status bars hidden (read-mostly, plan section 3). Reused 1.x panels keep their own copy until E2 (editor/* onto the dictionaries).</t>
+  </si>
+  <si>
+    <t>S2-040</t>
+  </si>
+  <si>
+    <t>Canvas document kind and model</t>
+  </si>
+  <si>
+    <t>kind=canvas in documents.data with schema_version; adapter: old documents = flow; validation on the backend.</t>
+  </si>
+  <si>
+    <t>Round-trip tests; old documents unaffected; no schema migration</t>
+  </si>
+  <si>
+    <t>b7d004e</t>
+  </si>
+  <si>
+    <t>editor/design/model.test.ts 18</t>
+  </si>
+  <si>
+    <t>E3 foundation: pure design model (select/marquee, move+snap with guides, nudge, resize from handles with aspect/centre, rotate with 15° snap, stacking, add/duplicate/remove, bounded undo with one step per drag). Persistence waits for D-012.</t>
+  </si>
+  <si>
+    <t>S2-060</t>
+  </si>
+  <si>
+    <t>AI</t>
+  </si>
+  <si>
+    <t>AI proposal framework</t>
+  </si>
+  <si>
+    <t>Proposal = patch against a revision; preview/diff; accept -&gt; revision; reject -&gt; nothing.</t>
+  </si>
+  <si>
+    <t>Rejecting leaves the saved document byte-identical (test)</t>
+  </si>
+  <si>
+    <t>D-008</t>
+  </si>
+  <si>
+    <t>S2-070</t>
+  </si>
+  <si>
+    <t>TRANSLATION</t>
+  </si>
+  <si>
+    <t>Translate panel and review</t>
+  </si>
+  <si>
+    <t>Scope (selection/element/page/document), languages (auto-detect, BG/EN first), preview, side-by-side compare, save as new.</t>
+  </si>
+  <si>
+    <t>DOCX fidelity tests on representative documents; overflow warnings</t>
+  </si>
+  <si>
+    <t>Provider: D-007</t>
+  </si>
+  <si>
+    <t>S2-016</t>
+  </si>
+  <si>
+    <t>I18N</t>
+  </si>
+  <si>
+    <t>Bulgarian / English interface (D-010)</t>
+  </si>
+  <si>
+    <t>Typed dictionaries (en source, bg checked), cookie smartdoc_locale (1 year), first visit from Accept-Language (bg -&gt; BG, else EN), switch in Settings and on sign-in pages, &lt;html lang&gt;, Intl relative times; independent of document language and Translate.</t>
+  </si>
+  <si>
+    <t>Both languages render; choice persists across reloads; parity of keys and placeholders tested</t>
+  </si>
+  <si>
+    <t>i18n.test.tsx 19 (negotiation, cookie precedence, key/placeholder parity, switch + cookie + refresh, fallback); e2e: bg-BG browser starts in BG, switch to EN survives reload, Settings switch survives reload</t>
+  </si>
+  <si>
+    <t>Preference per browser (cookie), not per account: an account-level setting would need a schema change (D-004).</t>
+  </si>
+  <si>
+    <t>S2-017</t>
+  </si>
+  <si>
+    <t>Move the remaining 1.x screens onto the dictionaries</t>
+  </si>
+  <si>
+    <t>Editor, create wizard, templates, documents list, billing, account settings content, compare, password reset forms: their English strings into en/bg.</t>
+  </si>
+  <si>
+    <t>No hard-coded interface English left in those screens (a grep test); both languages rendered in their tests</t>
+  </si>
+  <si>
+    <t>d1ec879, f9037ec, d8af836</t>
+  </si>
+  <si>
+    <t>see SESSION_STATE (checked after push)</t>
+  </si>
+  <si>
+    <t>i18n/hardcoded.test.ts: 29 screens with no literal interface English (TypeScript parser over JSX text and readable attributes); i18n/screens.bg.test.tsx 7 (screens rendered in Bulgarian); i18n.test.tsx (no empty text, same placeholders); Vitest 518; Playwright 66/1 skipped; browser BG docs/ui-review/2026-10-14b/</t>
+  </si>
+  <si>
+    <t>All non-editor screens + the flow's 1.x pieces + page titles (&lt;title&gt;) in en/bg; plural helper; numbers follow the interface language. Out of scope by decision: the 1.x editor chrome (editor/*) moves to the dictionaries with the 2.0 editor (E1/E2) instead of being translated twice; server messages (API errors, version descriptions, plan/unit labels from the API) stay English until the API returns codes -- billing units are already named by key.</t>
+  </si>
+  <si>
+    <t>S2-018</t>
+  </si>
+  <si>
+    <t>Real project thumbnails</t>
+  </si>
+  <si>
+    <t>The real first page of a project on its card: rendered by the backend (first 60 blocks -&gt; PDF -&gt; pypdfium2, 480 px, 4:3), cached in storage per revision, loaded lazily by the card with a per-type fallback.</t>
+  </si>
+  <si>
+    <t>Cards show the real first page, nothing invented; per-type fallback while loading and on error; no rendering on dashboard list requests (rendered on first request, cached per revision, immutable URL per updatedAt); another account gets 404; deleted with the document</t>
+  </si>
+  <si>
+    <t>719b8d7</t>
+  </si>
+  <si>
+    <t>dpl_3bYEX4jWjA2UHuRcJqPw8oK1fzKc (READY, 719b8d7)</t>
+  </si>
+  <si>
+    <t>backend tests/test_thumbnails.py 6 (cache per revision, re-render after edit, stranger 404, deleted with document, render failure -&gt; 404); ProjectCard.test.tsx 4 (lazy src per version, loading/shown/missing, BG alt); e2e: real image on the card + stranger 404; local browser: 3 real thumbnails incl. Cyrillic, lazy on scroll</t>
+  </si>
+  <si>
+    <t>Code in b716a5f (backend) + this commit (card). Storage keys thumbnails/{id}.png + .rev -- objects only, no schema change. Local-only race fixed: B-006.</t>
+  </si>
+  <si>
+    <t>S2-R01</t>
+  </si>
+  <si>
+    <t>Light theme as standard, dark as an option</t>
+  </si>
+  <si>
+    <t>Centralised light/dark tokens (globals.css :root and [data-theme=dark]); server-rendered data-theme from the smartdoc_theme cookie; compact switch in the sidebar account card and a Light/Dark choice in Your account.</t>
+  </si>
+  <si>
+    <t>Light without a choice; the choice persists across reloads and visits; no flash (server renders the theme); both themes readable (contrast, focus, hover) at 1280/1440/375</t>
+  </si>
+  <si>
+    <t>theme.test.tsx 3; e2e: light by default -&gt; Settings Dark -&gt; holds after reload -&gt; sidebar back to light; browser check both themes 1280/1440/375 (screenshots docs/ui-review/2026-10-14/)</t>
+  </si>
+  <si>
+    <t>1.x screens that still use the zinc palette: S2-R06.</t>
+  </si>
+  <si>
+    <t>S2-R02</t>
+  </si>
+  <si>
+    <t>Dashboard refinement (UI review)</t>
+  </si>
+  <si>
+    <t>Idea panel that says plainly what works now (type suggestion from your words) and what comes later (AI drafts); coloured quick actions incl. Translate; lighter At-a-glance column (plan meter, exports, templates); project cards with the real first page.</t>
+  </si>
+  <si>
+    <t>No claim of AI for keyword matching; Translate visible from the dashboard; right column quieter than the main column; all copy in en/bg; no horizontal scroll at 375/1280/1440</t>
+  </si>
+  <si>
+    <t>Dashboard.test.tsx 14 (idea panel lines, Translate quick action, At-a-glance meter, BG); browser screenshots light/dark docs/ui-review/2026-10-14/</t>
+  </si>
+  <si>
+    <t>375 px fixes found in the review: B-007 (idea field), B-008 (search squeezed).</t>
+  </si>
+  <si>
+    <t>S2-R03</t>
+  </si>
+  <si>
+    <t>Translate entry point + 'in development' screen</t>
+  </si>
+  <si>
+    <t>Translate in the sidebar and as a dashboard quick action, leading to /translate: the planned flow, clearly marked as in development, no simulated translation.</t>
+  </si>
+  <si>
+    <t>Signed-in only; says it isn't available yet; nothing pretends to translate; EN/BG</t>
+  </si>
+  <si>
+    <t>Dashboard.test.tsx (quick action marked Coming soon); browser /translate at 375 light (screenshot)</t>
+  </si>
+  <si>
+    <t>The real flow is S2-070 (shared Translation Engine, D-007).</t>
+  </si>
+  <si>
+    <t>S2-R04</t>
+  </si>
+  <si>
+    <t>Sidebar polish</t>
+  </si>
+  <si>
+    <t>Places (Home, Projects, Templates, Translate) and Settings (Your account, Plan and billing) groups; active item with accent bar; account card with theme switch and sign out; phone drawer.</t>
+  </si>
+  <si>
+    <t>Active state visible in both themes; drawer opens as a dialog, Escape closes it and focus returns to the menu button</t>
+  </si>
+  <si>
+    <t>AppShell.test.tsx (drawer + focus return); browser drawer 375 dark</t>
+  </si>
+  <si>
+    <t>Focus return fixed in the review: B-009.</t>
+  </si>
+  <si>
+    <t>S2-R05</t>
+  </si>
+  <si>
+    <t>Theme choice in Your account</t>
+  </si>
+  <si>
+    <t>Interface language and Appearance side by side in Your account; the account page's cards on the theme tokens.</t>
+  </si>
+  <si>
+    <t>Light/Dark radio persists; cards follow the theme</t>
+  </si>
+  <si>
+    <t>e2e theme test uses this radio; browser 375 light/dark</t>
+  </si>
+  <si>
+    <t>The account page's remaining English copy moves with S2-017.</t>
+  </si>
+  <si>
+    <t>S2-R06</t>
+  </si>
+  <si>
+    <t>Move the remaining 1.x screens onto the theme tokens</t>
+  </si>
+  <si>
+    <t>Documents list, billing, templates editor, compare, create wizard, side panel, dialogs still use zinc/white classes with dark: variants instead of the surface/line/muted tokens.</t>
+  </si>
+  <si>
+    <t>No zinc-* classes left in components (grep test); both themes checked in the browser</t>
+  </si>
+  <si>
+    <t>hardcoded.test.ts: no zinc-* in components/ or app/; browser light/dark docs/ui-review/2026-10-14b/</t>
+  </si>
+  <si>
+    <t>Compare now inside the app shell. White 'paper' scope (.paper) keeps sample pages dark-on-white in the dark theme (B-012). editor/* keeps its 1.x classes until the 2.0 editor shell.</t>
+  </si>
+  <si>
+    <t>S2-021</t>
+  </si>
+  <si>
+    <t>Look suggestion from the document's structure (M3.3)</t>
+  </si>
+  <si>
+    <t>The look step suggests a template from the document's own words and structure (title, headings, first 3,000 characters; tables, pictures, heading count) by built-in rules; shows the evidence; labelled 'not AI'; preselected only when there is no link choice and no workspace default.</t>
+  </si>
+  <si>
+    <t>Clear real-AI vs rules distinction; evidence shown; no suggestion when evidence is thin or tied; nothing applied until chosen; EN/BG</t>
   </si>
   <si>
     <t>bb571a8</t>
   </si>
   <si>
-    <t>E0 plan: docs/SMARTDOC_2_0_EDITOR_ARCHITECTURE.md (awaiting owner review). Next: E1 shell behind ?editor=2.</t>
-  </si>
-  <si>
-    <t>S2-040</t>
-  </si>
-  <si>
-    <t>Canvas document kind and model</t>
-  </si>
-  <si>
-    <t>kind=canvas in documents.data with schema_version; adapter: old documents = flow; validation on the backend.</t>
-  </si>
-  <si>
-    <t>Round-trip tests; old documents unaffected; no schema migration</t>
-  </si>
-  <si>
-    <t>b7d004e</t>
-  </si>
-  <si>
-    <t>editor/design/model.test.ts 18</t>
-  </si>
-  <si>
-    <t>E3 foundation: pure design model (select/marquee, move+snap with guides, nudge, resize from handles with aspect/centre, rotate with 15° snap, stacking, add/duplicate/remove, bounded undo with one step per drag). Persistence waits for D-012.</t>
-  </si>
-  <si>
-    <t>S2-060</t>
-  </si>
-  <si>
-    <t>AI</t>
-  </si>
-  <si>
-    <t>AI proposal framework</t>
-  </si>
-  <si>
-    <t>Proposal = patch against a revision; preview/diff; accept -&gt; revision; reject -&gt; nothing.</t>
-  </si>
-  <si>
-    <t>Rejecting leaves the saved document byte-identical (test)</t>
-  </si>
-  <si>
-    <t>D-008</t>
-  </si>
-  <si>
-    <t>S2-070</t>
-  </si>
-  <si>
-    <t>TRANSLATION</t>
-  </si>
-  <si>
-    <t>Translate panel and review</t>
-  </si>
-  <si>
-    <t>Scope (selection/element/page/document), languages (auto-detect, BG/EN first), preview, side-by-side compare, save as new.</t>
-  </si>
-  <si>
-    <t>DOCX fidelity tests on representative documents; overflow warnings</t>
-  </si>
-  <si>
-    <t>Provider: D-007</t>
-  </si>
-  <si>
-    <t>S2-016</t>
-  </si>
-  <si>
-    <t>I18N</t>
-  </si>
-  <si>
-    <t>Bulgarian / English interface (D-010)</t>
-  </si>
-  <si>
-    <t>Typed dictionaries (en source, bg checked), cookie smartdoc_locale (1 year), first visit from Accept-Language (bg -&gt; BG, else EN), switch in Settings and on sign-in pages, &lt;html lang&gt;, Intl relative times; independent of document language and Translate.</t>
-  </si>
-  <si>
-    <t>Both languages render; choice persists across reloads; parity of keys and placeholders tested</t>
-  </si>
-  <si>
-    <t>i18n.test.tsx 19 (negotiation, cookie precedence, key/placeholder parity, switch + cookie + refresh, fallback); e2e: bg-BG browser starts in BG, switch to EN survives reload, Settings switch survives reload</t>
-  </si>
-  <si>
-    <t>Preference per browser (cookie), not per account: an account-level setting would need a schema change (D-004).</t>
-  </si>
-  <si>
-    <t>S2-017</t>
-  </si>
-  <si>
-    <t>Move the remaining 1.x screens onto the dictionaries</t>
-  </si>
-  <si>
-    <t>Editor, create wizard, templates, documents list, billing, account settings content, compare, password reset forms: their English strings into en/bg.</t>
-  </si>
-  <si>
-    <t>No hard-coded interface English left in those screens (a grep test); both languages rendered in their tests</t>
-  </si>
-  <si>
-    <t>d1ec879, f9037ec, d8af836</t>
-  </si>
-  <si>
-    <t>see SESSION_STATE (checked after push)</t>
-  </si>
-  <si>
-    <t>i18n/hardcoded.test.ts: 29 screens with no literal interface English (TypeScript parser over JSX text and readable attributes); i18n/screens.bg.test.tsx 7 (screens rendered in Bulgarian); i18n.test.tsx (no empty text, same placeholders); Vitest 518; Playwright 66/1 skipped; browser BG docs/ui-review/2026-10-14b/</t>
-  </si>
-  <si>
-    <t>All non-editor screens + the flow's 1.x pieces + page titles (&lt;title&gt;) in en/bg; plural helper; numbers follow the interface language. Out of scope by decision: the 1.x editor chrome (editor/*) moves to the dictionaries with the 2.0 editor (E1/E2) instead of being translated twice; server messages (API errors, version descriptions, plan/unit labels from the API) stay English until the API returns codes -- billing units are already named by key.</t>
-  </si>
-  <si>
-    <t>S2-018</t>
-  </si>
-  <si>
-    <t>Real project thumbnails</t>
-  </si>
-  <si>
-    <t>The real first page of a project on its card: rendered by the backend (first 60 blocks -&gt; PDF -&gt; pypdfium2, 480 px, 4:3), cached in storage per revision, loaded lazily by the card with a per-type fallback.</t>
-  </si>
-  <si>
-    <t>Cards show the real first page, nothing invented; per-type fallback while loading and on error; no rendering on dashboard list requests (rendered on first request, cached per revision, immutable URL per updatedAt); another account gets 404; deleted with the document</t>
-  </si>
-  <si>
-    <t>719b8d7</t>
-  </si>
-  <si>
-    <t>dpl_3bYEX4jWjA2UHuRcJqPw8oK1fzKc (READY, 719b8d7)</t>
-  </si>
-  <si>
-    <t>backend tests/test_thumbnails.py 6 (cache per revision, re-render after edit, stranger 404, deleted with document, render failure -&gt; 404); ProjectCard.test.tsx 4 (lazy src per version, loading/shown/missing, BG alt); e2e: real image on the card + stranger 404; local browser: 3 real thumbnails incl. Cyrillic, lazy on scroll</t>
-  </si>
-  <si>
-    <t>Code in b716a5f (backend) + this commit (card). Storage keys thumbnails/{id}.png + .rev -- objects only, no schema change. Local-only race fixed: B-006.</t>
-  </si>
-  <si>
-    <t>S2-R01</t>
-  </si>
-  <si>
-    <t>Light theme as standard, dark as an option</t>
-  </si>
-  <si>
-    <t>Centralised light/dark tokens (globals.css :root and [data-theme=dark]); server-rendered data-theme from the smartdoc_theme cookie; compact switch in the sidebar account card and a Light/Dark choice in Your account.</t>
-  </si>
-  <si>
-    <t>Light without a choice; the choice persists across reloads and visits; no flash (server renders the theme); both themes readable (contrast, focus, hover) at 1280/1440/375</t>
-  </si>
-  <si>
-    <t>theme.test.tsx 3; e2e: light by default -&gt; Settings Dark -&gt; holds after reload -&gt; sidebar back to light; browser check both themes 1280/1440/375 (screenshots docs/ui-review/2026-10-14/)</t>
-  </si>
-  <si>
-    <t>1.x screens that still use the zinc palette: S2-R06.</t>
-  </si>
-  <si>
-    <t>S2-R02</t>
-  </si>
-  <si>
-    <t>Dashboard refinement (UI review)</t>
-  </si>
-  <si>
-    <t>Idea panel that says plainly what works now (type suggestion from your words) and what comes later (AI drafts); coloured quick actions incl. Translate; lighter At-a-glance column (plan meter, exports, templates); project cards with the real first page.</t>
-  </si>
-  <si>
-    <t>No claim of AI for keyword matching; Translate visible from the dashboard; right column quieter than the main column; all copy in en/bg; no horizontal scroll at 375/1280/1440</t>
-  </si>
-  <si>
-    <t>Dashboard.test.tsx 14 (idea panel lines, Translate quick action, At-a-glance meter, BG); browser screenshots light/dark docs/ui-review/2026-10-14/</t>
-  </si>
-  <si>
-    <t>375 px fixes found in the review: B-007 (idea field), B-008 (search squeezed).</t>
-  </si>
-  <si>
-    <t>S2-R03</t>
-  </si>
-  <si>
-    <t>Translate entry point + 'in development' screen</t>
-  </si>
-  <si>
-    <t>Translate in the sidebar and as a dashboard quick action, leading to /translate: the planned flow, clearly marked as in development, no simulated translation.</t>
-  </si>
-  <si>
-    <t>Signed-in only; says it isn't available yet; nothing pretends to translate; EN/BG</t>
-  </si>
-  <si>
-    <t>Dashboard.test.tsx (quick action marked Coming soon); browser /translate at 375 light (screenshot)</t>
-  </si>
-  <si>
-    <t>The real flow is S2-070 (shared Translation Engine, D-007).</t>
-  </si>
-  <si>
-    <t>S2-R04</t>
-  </si>
-  <si>
-    <t>Sidebar polish</t>
-  </si>
-  <si>
-    <t>Places (Home, Projects, Templates, Translate) and Settings (Your account, Plan and billing) groups; active item with accent bar; account card with theme switch and sign out; phone drawer.</t>
-  </si>
-  <si>
-    <t>Active state visible in both themes; drawer opens as a dialog, Escape closes it and focus returns to the menu button</t>
-  </si>
-  <si>
-    <t>AppShell.test.tsx (drawer + focus return); browser drawer 375 dark</t>
-  </si>
-  <si>
-    <t>Focus return fixed in the review: B-009.</t>
-  </si>
-  <si>
-    <t>S2-R05</t>
-  </si>
-  <si>
-    <t>Theme choice in Your account</t>
-  </si>
-  <si>
-    <t>Interface language and Appearance side by side in Your account; the account page's cards on the theme tokens.</t>
-  </si>
-  <si>
-    <t>Light/Dark radio persists; cards follow the theme</t>
-  </si>
-  <si>
-    <t>e2e theme test uses this radio; browser 375 light/dark</t>
-  </si>
-  <si>
-    <t>The account page's remaining English copy moves with S2-017.</t>
-  </si>
-  <si>
-    <t>S2-R06</t>
-  </si>
-  <si>
-    <t>Move the remaining 1.x screens onto the theme tokens</t>
-  </si>
-  <si>
-    <t>Documents list, billing, templates editor, compare, create wizard, side panel, dialogs still use zinc/white classes with dark: variants instead of the surface/line/muted tokens.</t>
-  </si>
-  <si>
-    <t>No zinc-* classes left in components (grep test); both themes checked in the browser</t>
-  </si>
-  <si>
-    <t>see SESSION_STATE</t>
-  </si>
-  <si>
-    <t>hardcoded.test.ts: no zinc-* in components/ or app/; browser light/dark docs/ui-review/2026-10-14b/</t>
-  </si>
-  <si>
-    <t>Compare now inside the app shell. White 'paper' scope (.paper) keeps sample pages dark-on-white in the dark theme (B-012). editor/* keeps its 1.x classes until the 2.0 editor shell.</t>
-  </si>
-  <si>
-    <t>S2-021</t>
-  </si>
-  <si>
-    <t>Look suggestion from the document's structure (M3.3)</t>
-  </si>
-  <si>
-    <t>The look step suggests a template from the document's own words and structure (title, headings, first 3,000 characters; tables, pictures, heading count) by built-in rules; shows the evidence; labelled 'not AI'; preselected only when there is no link choice and no workspace default.</t>
-  </si>
-  <si>
-    <t>Clear real-AI vs rules distinction; evidence shown; no suggestion when evidence is thin or tied; nothing applied until chosen; EN/BG</t>
-  </si>
-  <si>
     <t>recommendLook.test.ts 8 (CV, contract, report+table, coursework, application, nothing clear, word starts, no template of the kind); DocumentFlow.test (suggestion region, reasons, 'not by AI', preselection); browser BG 1280 + dark 375</t>
   </si>
   <si>
@@ -802,6 +808,69 @@
     <t>Mobile action bar 190 -&gt; 117 px (B-015).</t>
   </si>
   <si>
+    <t>S2-050</t>
+  </si>
+  <si>
+    <t>RELEASE</t>
+  </si>
+  <si>
+    <t>Isolated database and storage for the 2.0 Preview (D-012 option a)</t>
+  </si>
+  <si>
+    <t>Own Supabase project (free, $0/month), schema from alembic --sql (14 migrations, head d41f7a60c9e2), own private bucket and S3 keys, branch-scoped Preview variables for feature/smartdoc-2.0 entered by the owner, write guard, synthetic data only, rollback by removing the branch-scoped variables.</t>
+  </si>
+  <si>
+    <t>Preview health shows environment preview-2.0 and the new database's fingerprint; no Preview connection or object in production during a test session; guard refuses a production URL</t>
+  </si>
+  <si>
+    <t>Owner + Claude</t>
+  </si>
+  <si>
+    <t>tests/test_preview_isolation.py 6 (guard refuses production DB/storage in preview mode, accepts own, production/local unaffected, health fingerprint never shows the host); alembic upgrade head --sql generated offline without a database</t>
+  </si>
+  <si>
+    <t>Waiting for the owner's explicit approval of docs/SMARTDOC_2_0_PREVIEW_ISOLATION_PLAN.md. Nothing switched; no Production change.</t>
+  </si>
+  <si>
+    <t>S2-023</t>
+  </si>
+  <si>
+    <t>Look step on phones: lighter template choice</t>
+  </si>
+  <si>
+    <t>On phones each template card with its sample is tall; a compact list (name + small swatch, sample on demand) or a horizontal carousel, the suggestion first.</t>
+  </si>
+  <si>
+    <t>All five templates reachable within two screen heights at 375 px; selected state unchanged; no horizontal page scroll</t>
+  </si>
+  <si>
+    <t>Owner review 2026-10-14; not blocking E1.</t>
+  </si>
+  <si>
+    <t>S2-024</t>
+  </si>
+  <si>
+    <t>Structure review: a readable preview of tables</t>
+  </si>
+  <si>
+    <t>A table row in the structure check shows its size (rows x columns), header row and first cells as a small grid instead of one line of text; tables with merged cells marked.</t>
+  </si>
+  <si>
+    <t>Tables recognisable at a glance in EN/BG; long tables don't push the outline away</t>
+  </si>
+  <si>
+    <t>S2-025</t>
+  </si>
+  <si>
+    <t>Projects screen: gallery like the dashboard</t>
+  </si>
+  <si>
+    <t>/documents as a grid of project cards with real thumbnails (list view as an option), filters (type, status), sort and search kept, batch actions kept.</t>
+  </si>
+  <si>
+    <t>Same functions as today's list (search, sort, pages, batch, compare, delete) with thumbnails; EN/BG; light/dark; no thumbnail rendering on list requests</t>
+  </si>
+  <si>
     <t>Bug ID</t>
   </si>
   <si>
@@ -1075,7 +1144,10 @@
     <t>The built-in template's own name contains '(по подразбиране)'</t>
   </si>
   <si>
-    <t>Rename the built-in in backend/app/formatting/builtin_templates.json (check tests and existing workspaces' references by id, not name)</t>
+    <t>Built-in renamed 'Академичен' -- ids unchanged, names looked up by id, so documents and workspace defaults keep working (b85cc79)</t>
+  </si>
+  <si>
+    <t>tests/test_templates.py: ids pinned, no built-in name says 'default'; template API/access tests 43 green; e2e uses /Академичен/</t>
   </si>
   <si>
     <t>B-015</t>
@@ -1096,6 +1168,24 @@
     <t>Browser: bar 117 px</t>
   </si>
   <si>
+    <t>B-016</t>
+  </si>
+  <si>
+    <t>Editor in the dark theme: properties, page settings, export menu, action bar</t>
+  </si>
+  <si>
+    <t>WCAG AA contrast</t>
+  </si>
+  <si>
+    <t>Grey labels (zinc-500 on dark) below AA -- found by axe on the 2.0 shell; the classic editor had the same</t>
+  </si>
+  <si>
+    <t>Those labels on the muted token (b85cc79)</t>
+  </si>
+  <si>
+    <t>e2e/accessibility.spec.ts: 2.0 shell light, panel open, dark -- no serious violations</t>
+  </si>
+  <si>
     <t>Test ID</t>
   </si>
   <si>
@@ -1381,6 +1471,48 @@
     <t>docs/ui-review/2026-10-14b/</t>
   </si>
   <si>
+    <t>T-023</t>
+  </si>
+  <si>
+    <t>Full pytest (isolation guard, built-in rename)</t>
+  </si>
+  <si>
+    <t>PASS 2625 / 11 skipped (2624 + OpenAPI contract after re-export)</t>
+  </si>
+  <si>
+    <t>pytest -q</t>
+  </si>
+  <si>
+    <t>T-024</t>
+  </si>
+  <si>
+    <t>Vitest + tsc + eslint (engine refactor, 2.0 shell)</t>
+  </si>
+  <si>
+    <t>PASS 520 / tsc / eslint</t>
+  </si>
+  <si>
+    <t>T-025</t>
+  </si>
+  <si>
+    <t>Playwright: all classic specs + e2e/editor-v2.spec.ts + axe on the 2.0 shell</t>
+  </si>
+  <si>
+    <t>PASS 74 / 1 skipped</t>
+  </si>
+  <si>
+    <t>T-026</t>
+  </si>
+  <si>
+    <t>2.0 editor: 1440 light with panel, 1280 dark paper, 375 dark + drawer; typing/autosave/reload, undo/redo, classic default</t>
+  </si>
+  <si>
+    <t>PASS after rail width, paper, phone fixes</t>
+  </si>
+  <si>
+    <t>docs/ui-review/2026-10-14c/</t>
+  </si>
+  <si>
     <t>Decision ID</t>
   </si>
   <si>
@@ -1522,13 +1654,16 @@
     <t>D-012</t>
   </si>
   <si>
-    <t>Design-mode documents in the shared database</t>
-  </si>
-  <si>
-    <t>PENDING (owner): before any design document is written from the Preview, either a separate 2.0 database (recommended) or a 1.x change keeping unknown fields; 1.x would otherwise drop the canvas on save (pydantic extra=ignore, checked 2026-10-14)</t>
-  </si>
-  <si>
-    <t>P5 persistence</t>
+    <t>Canvas documents and the shared database</t>
+  </si>
+  <si>
+    <t>DECIDED 2026-10-14 (owner): option (a), a separate database for the 2.0 Preview. The switch itself waits for the owner's approval of docs/SMARTDOC_2_0_PREVIEW_ISOLATION_PLAN.md; no Production change, no data moved or deleted.</t>
+  </si>
+  <si>
+    <t>S2-050, P5 persistence</t>
+  </si>
+  <si>
+    <t>S2-050, S2-040</t>
   </si>
   <si>
     <t>Requirement</t>
@@ -2248,8 +2383,8 @@
         <v>5</v>
       </c>
       <c r="B5" s="5">
-        <f>COUNTIF(Tasks!$G$2:$G$27,A5)</f>
-        <v>2</v>
+        <f>COUNTIF(Tasks!$G$2:$G$31,A5)</f>
+        <v>5</v>
       </c>
       <c r="C5" s="5">
         <f>COUNTIF(Roadmap!$D$2:$D$10,A5)</f>
@@ -2261,7 +2396,7 @@
         <v>6</v>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF(Tasks!$G$2:$G$27,A6)</f>
+        <f>COUNTIF(Tasks!$G$2:$G$31,A6)</f>
         <v>0</v>
       </c>
       <c r="C6" s="5">
@@ -2274,8 +2409,8 @@
         <v>7</v>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF(Tasks!$G$2:$G$27,A7)</f>
-        <v>2</v>
+        <f>COUNTIF(Tasks!$G$2:$G$31,A7)</f>
+        <v>1</v>
       </c>
       <c r="C7" s="5">
         <f>COUNTIF(Roadmap!$D$2:$D$10,A7)</f>
@@ -2287,8 +2422,8 @@
         <v>8</v>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF(Tasks!$G$2:$G$27,A8)</f>
-        <v>0</v>
+        <f>COUNTIF(Tasks!$G$2:$G$31,A8)</f>
+        <v>1</v>
       </c>
       <c r="C8" s="5">
         <f>COUNTIF(Roadmap!$D$2:$D$10,A8)</f>
@@ -2300,7 +2435,7 @@
         <v>9</v>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIF(Tasks!$G$2:$G$27,A9)</f>
+        <f>COUNTIF(Tasks!$G$2:$G$31,A9)</f>
         <v>0</v>
       </c>
       <c r="C9" s="5">
@@ -2313,8 +2448,8 @@
         <v>10</v>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIF(Tasks!$G$2:$G$27,A10)</f>
-        <v>18</v>
+        <f>COUNTIF(Tasks!$G$2:$G$31,A10)</f>
+        <v>19</v>
       </c>
       <c r="C10" s="5">
         <f>COUNTIF(Roadmap!$D$2:$D$10,A10)</f>
@@ -2326,7 +2461,7 @@
         <v>11</v>
       </c>
       <c r="B11" s="5">
-        <f>COUNTIF(Tasks!$G$2:$G$27,A11)</f>
+        <f>COUNTIF(Tasks!$G$2:$G$31,A11)</f>
         <v>4</v>
       </c>
       <c r="C11" s="5">
@@ -2340,7 +2475,7 @@
       </c>
       <c r="B12" s="12">
         <f>SUM(B5:B11)</f>
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C12" s="12">
         <f>SUM(C5:C11)</f>
@@ -2353,7 +2488,7 @@
       </c>
       <c r="B13" s="14">
         <f>IFERROR((B11+B10)/B12,0)</f>
-        <v>0.84615384615384615</v>
+        <v>0.76666666666666672</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -2361,8 +2496,8 @@
         <v>14</v>
       </c>
       <c r="B14">
-        <f>COUNTIFS(Tasks!$F$2:$F$27,"P0",Tasks!$G$2:$G$27,"&lt;&gt;DONE",Tasks!$G$2:$G$27,"&lt;&gt;VERIFIED")</f>
-        <v>0</v>
+        <f>COUNTIFS(Tasks!$F$2:$F$31,"P0",Tasks!$G$2:$G$31,"&lt;&gt;DONE",Tasks!$G$2:$G$31,"&lt;&gt;VERIFIED")</f>
+        <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -2370,8 +2505,8 @@
         <v>15</v>
       </c>
       <c r="B15">
-        <f>COUNTA(Bugs!$A$2:$A$16)-COUNTIF(Bugs!$F$2:$F$16,"DONE")-COUNTIF(Bugs!$F$2:$F$16,"VERIFIED")</f>
-        <v>3</v>
+        <f>COUNTA(Bugs!$A$2:$A$17)-COUNTIF(Bugs!$F$2:$F$17,"DONE")-COUNTIF(Bugs!$F$2:$F$17,"VERIFIED")</f>
+        <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
@@ -2625,7 +2760,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:P27"/>
+  <dimension ref="A1:P31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
@@ -3227,7 +3362,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="13" spans="1:16" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" ht="216.75" x14ac:dyDescent="0.25">
       <c r="A13" s="17" t="s">
         <v>152</v>
       </c>
@@ -3247,7 +3382,7 @@
         <v>26</v>
       </c>
       <c r="G13" s="17" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="H13" s="17" t="s">
         <v>122</v>
@@ -3264,18 +3399,22 @@
       <c r="L13" s="17" t="s">
         <v>157</v>
       </c>
-      <c r="M13" s="17"/>
-      <c r="N13" s="17"/>
+      <c r="M13" s="17" t="s">
+        <v>158</v>
+      </c>
+      <c r="N13" s="17" t="s">
+        <v>159</v>
+      </c>
       <c r="O13" s="17" t="s">
         <v>81</v>
       </c>
       <c r="P13" s="17" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="14" spans="1:16" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B14" s="17" t="s">
         <v>42</v>
@@ -3284,10 +3423,10 @@
         <v>153</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="E14" s="17" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="F14" s="17" t="s">
         <v>26</v>
@@ -3299,7 +3438,7 @@
         <v>152</v>
       </c>
       <c r="I14" s="17" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="J14" s="17" t="s">
         <v>78</v>
@@ -3308,34 +3447,34 @@
         <v>79</v>
       </c>
       <c r="L14" s="17" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="M14" s="17"/>
       <c r="N14" s="17" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="O14" s="17" t="s">
         <v>81</v>
       </c>
       <c r="P14" s="17" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="15" spans="1:16" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A15" s="17" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B15" s="17" t="s">
         <v>46</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D15" s="17" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="E15" s="17" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="F15" s="17" t="s">
         <v>26</v>
@@ -3347,7 +3486,7 @@
         <v>152</v>
       </c>
       <c r="I15" s="17" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="J15" s="17" t="s">
         <v>78</v>
@@ -3362,24 +3501,24 @@
         <v>81</v>
       </c>
       <c r="P15" s="17" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="16" spans="1:16" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A16" s="17" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B16" s="17" t="s">
         <v>51</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="D16" s="17" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="E16" s="17" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="F16" s="17" t="s">
         <v>26</v>
@@ -3391,7 +3530,7 @@
         <v>152</v>
       </c>
       <c r="I16" s="17" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="J16" s="17" t="s">
         <v>78</v>
@@ -3406,24 +3545,24 @@
         <v>81</v>
       </c>
       <c r="P16" s="17" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
     </row>
     <row r="17" spans="1:16" ht="127.5" x14ac:dyDescent="0.25">
       <c r="A17" s="17" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B17" s="17" t="s">
         <v>30</v>
       </c>
       <c r="C17" s="17" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="D17" s="17" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="E17" s="17" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="F17" s="17" t="s">
         <v>22</v>
@@ -3435,7 +3574,7 @@
         <v>110</v>
       </c>
       <c r="I17" s="17" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="J17" s="17" t="s">
         <v>78</v>
@@ -3450,30 +3589,30 @@
         <v>135</v>
       </c>
       <c r="N17" s="17" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="O17" s="17" t="s">
         <v>81</v>
       </c>
       <c r="P17" s="17" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
     </row>
     <row r="18" spans="1:16" ht="178.5" x14ac:dyDescent="0.25">
       <c r="A18" s="17" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B18" s="17" t="s">
         <v>30</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="D18" s="17" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="E18" s="17" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="F18" s="17" t="s">
         <v>26</v>
@@ -3482,10 +3621,10 @@
         <v>10</v>
       </c>
       <c r="H18" s="17" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="I18" s="17" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="J18" s="17" t="s">
         <v>78</v>
@@ -3494,24 +3633,24 @@
         <v>79</v>
       </c>
       <c r="L18" s="17" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="M18" s="17" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="N18" s="17" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="O18" s="17" t="s">
         <v>81</v>
       </c>
       <c r="P18" s="17" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="19" spans="1:16" ht="165.75" x14ac:dyDescent="0.25">
       <c r="A19" s="17" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="B19" s="17" t="s">
         <v>30</v>
@@ -3520,10 +3659,10 @@
         <v>116</v>
       </c>
       <c r="D19" s="17" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="E19" s="17" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="F19" s="17" t="s">
         <v>22</v>
@@ -3535,7 +3674,7 @@
         <v>130</v>
       </c>
       <c r="I19" s="17" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="J19" s="17" t="s">
         <v>78</v>
@@ -3544,24 +3683,24 @@
         <v>79</v>
       </c>
       <c r="L19" s="17" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="M19" s="17" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="N19" s="17" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="O19" s="17" t="s">
         <v>81</v>
       </c>
       <c r="P19" s="17" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
     </row>
     <row r="20" spans="1:16" ht="102" x14ac:dyDescent="0.25">
       <c r="A20" s="17" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="B20" s="17" t="s">
         <v>30</v>
@@ -3570,10 +3709,10 @@
         <v>116</v>
       </c>
       <c r="D20" s="17" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="E20" s="17" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="F20" s="17" t="s">
         <v>22</v>
@@ -3585,7 +3724,7 @@
         <v>110</v>
       </c>
       <c r="I20" s="17" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="J20" s="17" t="s">
         <v>78</v>
@@ -3594,24 +3733,24 @@
         <v>79</v>
       </c>
       <c r="L20" s="17" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="M20" s="17" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="N20" s="17" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="O20" s="17" t="s">
         <v>81</v>
       </c>
       <c r="P20" s="17" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
     </row>
     <row r="21" spans="1:16" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A21" s="17" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B21" s="17" t="s">
         <v>30</v>
@@ -3620,10 +3759,10 @@
         <v>116</v>
       </c>
       <c r="D21" s="17" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="E21" s="17" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="F21" s="17" t="s">
         <v>22</v>
@@ -3635,7 +3774,7 @@
         <v>130</v>
       </c>
       <c r="I21" s="17" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="J21" s="17" t="s">
         <v>78</v>
@@ -3644,36 +3783,36 @@
         <v>79</v>
       </c>
       <c r="L21" s="17" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="M21" s="17" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="N21" s="17" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="O21" s="17" t="s">
         <v>81</v>
       </c>
       <c r="P21" s="17" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
     </row>
     <row r="22" spans="1:16" ht="51" x14ac:dyDescent="0.25">
       <c r="A22" s="17" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B22" s="17" t="s">
         <v>30</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="D22" s="17" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="E22" s="17" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="F22" s="17" t="s">
         <v>26</v>
@@ -3685,7 +3824,7 @@
         <v>122</v>
       </c>
       <c r="I22" s="17" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="J22" s="17" t="s">
         <v>78</v>
@@ -3694,24 +3833,24 @@
         <v>79</v>
       </c>
       <c r="L22" s="17" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="M22" s="17" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="N22" s="17" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="O22" s="17" t="s">
         <v>81</v>
       </c>
       <c r="P22" s="17" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
     </row>
     <row r="23" spans="1:16" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A23" s="17" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B23" s="17" t="s">
         <v>30</v>
@@ -3720,10 +3859,10 @@
         <v>116</v>
       </c>
       <c r="D23" s="17" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="E23" s="17" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="F23" s="17" t="s">
         <v>26</v>
@@ -3735,7 +3874,7 @@
         <v>122</v>
       </c>
       <c r="I23" s="17" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="J23" s="17" t="s">
         <v>78</v>
@@ -3744,24 +3883,24 @@
         <v>79</v>
       </c>
       <c r="L23" s="17" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="M23" s="17" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="N23" s="17" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="O23" s="17" t="s">
         <v>81</v>
       </c>
       <c r="P23" s="17" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
     </row>
     <row r="24" spans="1:16" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A24" s="17" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B24" s="17" t="s">
         <v>30</v>
@@ -3770,10 +3909,10 @@
         <v>116</v>
       </c>
       <c r="D24" s="17" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="E24" s="17" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="F24" s="17" t="s">
         <v>26</v>
@@ -3782,10 +3921,10 @@
         <v>10</v>
       </c>
       <c r="H24" s="17" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="I24" s="17" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="J24" s="17" t="s">
         <v>78</v>
@@ -3794,24 +3933,24 @@
         <v>79</v>
       </c>
       <c r="L24" s="17" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="M24" s="17" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="N24" s="17" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="O24" s="17" t="s">
         <v>81</v>
       </c>
       <c r="P24" s="17" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="25" spans="1:16" ht="51" x14ac:dyDescent="0.25">
       <c r="A25" s="17" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="B25" s="17" t="s">
         <v>30</v>
@@ -3820,10 +3959,10 @@
         <v>116</v>
       </c>
       <c r="D25" s="17" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="E25" s="17" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="F25" s="17" t="s">
         <v>30</v>
@@ -3832,10 +3971,10 @@
         <v>10</v>
       </c>
       <c r="H25" s="17" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="I25" s="17" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="J25" s="17" t="s">
         <v>78</v>
@@ -3844,24 +3983,24 @@
         <v>79</v>
       </c>
       <c r="L25" s="17" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="M25" s="17" t="s">
-        <v>235</v>
+        <v>158</v>
       </c>
       <c r="N25" s="17" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="O25" s="17" t="s">
         <v>81</v>
       </c>
       <c r="P25" s="17" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="26" spans="1:16" ht="127.5" x14ac:dyDescent="0.25">
       <c r="A26" s="17" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B26" s="17" t="s">
         <v>34</v>
@@ -3870,10 +4009,10 @@
         <v>116</v>
       </c>
       <c r="D26" s="17" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E26" s="17" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F26" s="17" t="s">
         <v>26</v>
@@ -3885,7 +4024,7 @@
         <v>144</v>
       </c>
       <c r="I26" s="17" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="J26" s="17" t="s">
         <v>78</v>
@@ -3894,24 +4033,24 @@
         <v>79</v>
       </c>
       <c r="L26" s="17" t="s">
-        <v>157</v>
+        <v>243</v>
       </c>
       <c r="M26" s="17" t="s">
-        <v>235</v>
+        <v>158</v>
       </c>
       <c r="N26" s="17" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="O26" s="17" t="s">
         <v>81</v>
       </c>
       <c r="P26" s="17" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
     </row>
     <row r="27" spans="1:16" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A27" s="17" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B27" s="17" t="s">
         <v>34</v>
@@ -3920,10 +4059,10 @@
         <v>116</v>
       </c>
       <c r="D27" s="17" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="E27" s="17" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="F27" s="17" t="s">
         <v>26</v>
@@ -3935,7 +4074,7 @@
         <v>144</v>
       </c>
       <c r="I27" s="17" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="J27" s="17" t="s">
         <v>78</v>
@@ -3944,24 +4083,202 @@
         <v>79</v>
       </c>
       <c r="L27" s="17" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="M27" s="17" t="s">
-        <v>235</v>
+        <v>158</v>
       </c>
       <c r="N27" s="17" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="O27" s="17" t="s">
         <v>81</v>
       </c>
       <c r="P27" s="17" t="s">
-        <v>250</v>
+        <v>252</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" ht="127.5" x14ac:dyDescent="0.25">
+      <c r="A28" s="17" t="s">
+        <v>253</v>
+      </c>
+      <c r="B28" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="C28" s="17" t="s">
+        <v>254</v>
+      </c>
+      <c r="D28" s="17" t="s">
+        <v>255</v>
+      </c>
+      <c r="E28" s="17" t="s">
+        <v>256</v>
+      </c>
+      <c r="F28" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="G28" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="H28" s="17"/>
+      <c r="I28" s="17" t="s">
+        <v>257</v>
+      </c>
+      <c r="J28" s="17" t="s">
+        <v>258</v>
+      </c>
+      <c r="K28" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="L28" s="17" t="s">
+        <v>157</v>
+      </c>
+      <c r="M28" s="17"/>
+      <c r="N28" s="17" t="s">
+        <v>259</v>
+      </c>
+      <c r="O28" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="P28" s="17" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A29" s="17" t="s">
+        <v>261</v>
+      </c>
+      <c r="B29" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="C29" s="17" t="s">
+        <v>116</v>
+      </c>
+      <c r="D29" s="17" t="s">
+        <v>262</v>
+      </c>
+      <c r="E29" s="17" t="s">
+        <v>263</v>
+      </c>
+      <c r="F29" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="G29" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="H29" s="17" t="s">
+        <v>246</v>
+      </c>
+      <c r="I29" s="17" t="s">
+        <v>264</v>
+      </c>
+      <c r="J29" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="K29" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="L29" s="17"/>
+      <c r="M29" s="17"/>
+      <c r="N29" s="17"/>
+      <c r="O29" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="P29" s="17" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A30" s="17" t="s">
+        <v>266</v>
+      </c>
+      <c r="B30" s="17" t="s">
+        <v>34</v>
+      </c>
+      <c r="C30" s="17" t="s">
+        <v>116</v>
+      </c>
+      <c r="D30" s="17" t="s">
+        <v>267</v>
+      </c>
+      <c r="E30" s="17" t="s">
+        <v>268</v>
+      </c>
+      <c r="F30" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="G30" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="H30" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="I30" s="17" t="s">
+        <v>269</v>
+      </c>
+      <c r="J30" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="K30" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="L30" s="17"/>
+      <c r="M30" s="17"/>
+      <c r="N30" s="17"/>
+      <c r="O30" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="P30" s="17" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A31" s="17" t="s">
+        <v>270</v>
+      </c>
+      <c r="B31" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="C31" s="17" t="s">
+        <v>116</v>
+      </c>
+      <c r="D31" s="17" t="s">
+        <v>271</v>
+      </c>
+      <c r="E31" s="17" t="s">
+        <v>272</v>
+      </c>
+      <c r="F31" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="G31" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="H31" s="17" t="s">
+        <v>195</v>
+      </c>
+      <c r="I31" s="17" t="s">
+        <v>273</v>
+      </c>
+      <c r="J31" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="K31" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="L31" s="17"/>
+      <c r="M31" s="17"/>
+      <c r="N31" s="17"/>
+      <c r="O31" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="P31" s="17" t="s">
+        <v>265</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P27" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
-  <conditionalFormatting sqref="G2:G27">
+  <autoFilter ref="A1:P31" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
+  <conditionalFormatting sqref="G2:G31">
     <cfRule type="expression" dxfId="13" priority="1">
       <formula>$G2="BACKLOG"</formula>
     </cfRule>
@@ -3990,7 +4307,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -4005,419 +4322,447 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>251</v>
+        <v>274</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>252</v>
+        <v>275</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>253</v>
+        <v>276</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>254</v>
+        <v>277</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>255</v>
+        <v>278</v>
       </c>
       <c r="F1" s="16" t="s">
         <v>2</v>
       </c>
       <c r="G1" s="16" t="s">
-        <v>256</v>
+        <v>279</v>
       </c>
       <c r="H1" s="16" t="s">
-        <v>257</v>
+        <v>280</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
-        <v>258</v>
+        <v>281</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>259</v>
+        <v>282</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>260</v>
+        <v>283</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>261</v>
+        <v>284</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>262</v>
+        <v>285</v>
       </c>
       <c r="F2" s="17" t="s">
         <v>8</v>
       </c>
       <c r="G2" s="17" t="s">
-        <v>263</v>
+        <v>286</v>
       </c>
       <c r="H2" s="17" t="s">
-        <v>264</v>
+        <v>287</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
-        <v>265</v>
+        <v>288</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>266</v>
+        <v>289</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>267</v>
+        <v>290</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>268</v>
+        <v>291</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>269</v>
+        <v>292</v>
       </c>
       <c r="F3" s="17" t="s">
         <v>5</v>
       </c>
       <c r="G3" s="17"/>
       <c r="H3" s="17" t="s">
-        <v>270</v>
+        <v>293</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>271</v>
+        <v>294</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>266</v>
+        <v>289</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>272</v>
+        <v>295</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>273</v>
+        <v>296</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>274</v>
+        <v>297</v>
       </c>
       <c r="F4" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G4" s="17" t="s">
-        <v>275</v>
+        <v>298</v>
       </c>
       <c r="H4" s="17" t="s">
-        <v>276</v>
+        <v>299</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>277</v>
+        <v>300</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>278</v>
+        <v>301</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>279</v>
+        <v>302</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>280</v>
+        <v>303</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>281</v>
+        <v>304</v>
       </c>
       <c r="F5" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G5" s="17" t="s">
-        <v>282</v>
+        <v>305</v>
       </c>
       <c r="H5" s="17" t="s">
-        <v>283</v>
+        <v>306</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="51" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
-        <v>284</v>
+        <v>307</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>278</v>
+        <v>301</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>285</v>
+        <v>308</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>286</v>
+        <v>309</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>287</v>
+        <v>310</v>
       </c>
       <c r="F6" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G6" s="17" t="s">
-        <v>288</v>
+        <v>311</v>
       </c>
       <c r="H6" s="17" t="s">
-        <v>289</v>
+        <v>312</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
-        <v>290</v>
+        <v>313</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>278</v>
+        <v>301</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>291</v>
+        <v>314</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>292</v>
+        <v>315</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>293</v>
+        <v>316</v>
       </c>
       <c r="F7" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G7" s="17" t="s">
-        <v>294</v>
+        <v>317</v>
       </c>
       <c r="H7" s="17" t="s">
-        <v>295</v>
+        <v>318</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
-        <v>296</v>
+        <v>319</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>266</v>
+        <v>289</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>297</v>
+        <v>320</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>298</v>
+        <v>321</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>299</v>
+        <v>322</v>
       </c>
       <c r="F8" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G8" s="17" t="s">
-        <v>300</v>
+        <v>323</v>
       </c>
       <c r="H8" s="17" t="s">
-        <v>301</v>
+        <v>324</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="51" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
-        <v>302</v>
+        <v>325</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>266</v>
+        <v>289</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>303</v>
+        <v>326</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>304</v>
+        <v>327</v>
       </c>
       <c r="E9" s="17" t="s">
-        <v>305</v>
+        <v>328</v>
       </c>
       <c r="F9" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G9" s="17" t="s">
-        <v>306</v>
+        <v>329</v>
       </c>
       <c r="H9" s="17" t="s">
-        <v>307</v>
+        <v>330</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="51" x14ac:dyDescent="0.25">
       <c r="A10" s="17" t="s">
-        <v>308</v>
+        <v>331</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>266</v>
+        <v>289</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>309</v>
+        <v>332</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>310</v>
+        <v>333</v>
       </c>
       <c r="E10" s="17" t="s">
-        <v>311</v>
+        <v>334</v>
       </c>
       <c r="F10" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G10" s="17" t="s">
-        <v>312</v>
+        <v>335</v>
       </c>
       <c r="H10" s="17" t="s">
-        <v>313</v>
+        <v>336</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A11" s="17" t="s">
-        <v>314</v>
+        <v>337</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>266</v>
+        <v>289</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>315</v>
+        <v>338</v>
       </c>
       <c r="D11" s="17" t="s">
-        <v>316</v>
+        <v>339</v>
       </c>
       <c r="E11" s="17" t="s">
-        <v>317</v>
+        <v>340</v>
       </c>
       <c r="F11" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G11" s="17" t="s">
-        <v>318</v>
+        <v>341</v>
       </c>
       <c r="H11" s="17" t="s">
-        <v>319</v>
+        <v>342</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
-        <v>320</v>
+        <v>343</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>278</v>
+        <v>301</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>321</v>
+        <v>344</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>322</v>
+        <v>345</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>323</v>
+        <v>346</v>
       </c>
       <c r="F12" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G12" s="17" t="s">
-        <v>324</v>
+        <v>347</v>
       </c>
       <c r="H12" s="17" t="s">
-        <v>325</v>
+        <v>348</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="51" x14ac:dyDescent="0.25">
       <c r="A13" s="17" t="s">
-        <v>326</v>
+        <v>349</v>
       </c>
       <c r="B13" s="17" t="s">
-        <v>278</v>
+        <v>301</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>327</v>
+        <v>350</v>
       </c>
       <c r="D13" s="17" t="s">
-        <v>328</v>
+        <v>351</v>
       </c>
       <c r="E13" s="17" t="s">
-        <v>329</v>
+        <v>352</v>
       </c>
       <c r="F13" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G13" s="17" t="s">
-        <v>330</v>
+        <v>353</v>
       </c>
       <c r="H13" s="17" t="s">
-        <v>331</v>
+        <v>354</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="51" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
-        <v>332</v>
+        <v>355</v>
       </c>
       <c r="B14" s="17" t="s">
-        <v>266</v>
+        <v>289</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>333</v>
+        <v>356</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>334</v>
+        <v>357</v>
       </c>
       <c r="E14" s="17" t="s">
-        <v>335</v>
+        <v>358</v>
       </c>
       <c r="F14" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G14" s="17" t="s">
-        <v>336</v>
+        <v>359</v>
       </c>
       <c r="H14" s="17" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="114.75" x14ac:dyDescent="0.25">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="102" x14ac:dyDescent="0.25">
       <c r="A15" s="17" t="s">
-        <v>338</v>
+        <v>361</v>
       </c>
       <c r="B15" s="17" t="s">
-        <v>266</v>
+        <v>289</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>339</v>
+        <v>362</v>
       </c>
       <c r="D15" s="17" t="s">
-        <v>340</v>
+        <v>363</v>
       </c>
       <c r="E15" s="17" t="s">
-        <v>341</v>
+        <v>364</v>
       </c>
       <c r="F15" s="17" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G15" s="17" t="s">
-        <v>342</v>
-      </c>
-      <c r="H15" s="17"/>
+        <v>365</v>
+      </c>
+      <c r="H15" s="17" t="s">
+        <v>366</v>
+      </c>
     </row>
     <row r="16" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A16" s="17" t="s">
-        <v>343</v>
+        <v>367</v>
       </c>
       <c r="B16" s="17" t="s">
-        <v>266</v>
+        <v>289</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>344</v>
+        <v>368</v>
       </c>
       <c r="D16" s="17" t="s">
-        <v>345</v>
+        <v>369</v>
       </c>
       <c r="E16" s="17" t="s">
-        <v>346</v>
+        <v>370</v>
       </c>
       <c r="F16" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G16" s="17" t="s">
-        <v>347</v>
+        <v>371</v>
       </c>
       <c r="H16" s="17" t="s">
-        <v>348</v>
+        <v>372</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A17" s="17" t="s">
+        <v>373</v>
+      </c>
+      <c r="B17" s="17" t="s">
+        <v>301</v>
+      </c>
+      <c r="C17" s="17" t="s">
+        <v>374</v>
+      </c>
+      <c r="D17" s="17" t="s">
+        <v>375</v>
+      </c>
+      <c r="E17" s="17" t="s">
+        <v>376</v>
+      </c>
+      <c r="F17" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="G17" s="17" t="s">
+        <v>377</v>
+      </c>
+      <c r="H17" s="17" t="s">
+        <v>378</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H16" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
-  <conditionalFormatting sqref="F2:F16">
+  <autoFilter ref="A1:H17" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
+  <conditionalFormatting sqref="F2:F17">
     <cfRule type="expression" dxfId="6" priority="1">
       <formula>$F2="BACKLOG"</formula>
     </cfRule>
@@ -4446,7 +4791,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -4460,226 +4805,226 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>349</v>
+        <v>379</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>350</v>
+        <v>380</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>351</v>
+        <v>381</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>352</v>
+        <v>382</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>353</v>
+        <v>383</v>
       </c>
       <c r="F1" s="16" t="s">
-        <v>354</v>
+        <v>384</v>
       </c>
       <c r="G1" s="16" t="s">
-        <v>355</v>
+        <v>385</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
-        <v>356</v>
+        <v>386</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>357</v>
+        <v>387</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>358</v>
+        <v>388</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>359</v>
+        <v>389</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>360</v>
+        <v>390</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>361</v>
+        <v>391</v>
       </c>
       <c r="G2" s="17" t="s">
-        <v>362</v>
+        <v>392</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
-        <v>363</v>
+        <v>393</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>364</v>
+        <v>394</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>365</v>
+        <v>395</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>359</v>
+        <v>389</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>366</v>
+        <v>396</v>
       </c>
       <c r="F3" s="17" t="s">
-        <v>367</v>
+        <v>397</v>
       </c>
       <c r="G3" s="17" t="s">
-        <v>362</v>
+        <v>392</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>368</v>
+        <v>398</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>369</v>
+        <v>399</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>370</v>
+        <v>400</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>359</v>
+        <v>389</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>371</v>
+        <v>401</v>
       </c>
       <c r="F4" s="17" t="s">
-        <v>372</v>
+        <v>402</v>
       </c>
       <c r="G4" s="17" t="s">
-        <v>362</v>
+        <v>392</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>373</v>
+        <v>403</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>374</v>
+        <v>404</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>375</v>
+        <v>405</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>376</v>
+        <v>406</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>377</v>
+        <v>407</v>
       </c>
       <c r="F5" s="17" t="s">
-        <v>378</v>
+        <v>408</v>
       </c>
       <c r="G5" s="17" t="s">
-        <v>362</v>
+        <v>392</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
-        <v>379</v>
+        <v>409</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>364</v>
+        <v>394</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>380</v>
+        <v>410</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>359</v>
+        <v>389</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>381</v>
+        <v>411</v>
       </c>
       <c r="F6" s="17" t="s">
         <v>126</v>
       </c>
       <c r="G6" s="17" t="s">
-        <v>362</v>
+        <v>392</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
-        <v>382</v>
+        <v>412</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>369</v>
+        <v>399</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>383</v>
+        <v>413</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>359</v>
+        <v>389</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>384</v>
+        <v>414</v>
       </c>
       <c r="F7" s="17" t="s">
         <v>126</v>
       </c>
       <c r="G7" s="17" t="s">
-        <v>362</v>
+        <v>392</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
-        <v>385</v>
+        <v>415</v>
       </c>
       <c r="B8" s="17" t="s">
         <v>116</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>386</v>
+        <v>416</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>387</v>
+        <v>417</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>377</v>
+        <v>407</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>388</v>
+        <v>418</v>
       </c>
       <c r="G8" s="17" t="s">
-        <v>362</v>
+        <v>392</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
-        <v>389</v>
+        <v>419</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>390</v>
+        <v>420</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>391</v>
+        <v>421</v>
       </c>
       <c r="D9" s="17" t="s">
+        <v>422</v>
+      </c>
+      <c r="E9" s="17" t="s">
+        <v>423</v>
+      </c>
+      <c r="F9" s="17" t="s">
+        <v>424</v>
+      </c>
+      <c r="G9" s="17" t="s">
         <v>392</v>
-      </c>
-      <c r="E9" s="17" t="s">
-        <v>393</v>
-      </c>
-      <c r="F9" s="17" t="s">
-        <v>394</v>
-      </c>
-      <c r="G9" s="17" t="s">
-        <v>362</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="17" t="s">
-        <v>395</v>
+        <v>425</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>364</v>
+        <v>394</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>380</v>
+        <v>410</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>359</v>
+        <v>389</v>
       </c>
       <c r="E10" s="17" t="s">
-        <v>396</v>
+        <v>426</v>
       </c>
       <c r="F10" s="17" t="s">
         <v>134</v>
@@ -4690,19 +5035,19 @@
     </row>
     <row r="11" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A11" s="17" t="s">
-        <v>397</v>
+        <v>427</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>369</v>
+        <v>399</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>398</v>
+        <v>428</v>
       </c>
       <c r="D11" s="17" t="s">
-        <v>399</v>
+        <v>429</v>
       </c>
       <c r="E11" s="17" t="s">
-        <v>400</v>
+        <v>430</v>
       </c>
       <c r="F11" s="17" t="s">
         <v>134</v>
@@ -4713,22 +5058,22 @@
     </row>
     <row r="12" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
-        <v>401</v>
+        <v>431</v>
       </c>
       <c r="B12" s="17" t="s">
         <v>116</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>402</v>
+        <v>432</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>387</v>
+        <v>417</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>403</v>
+        <v>433</v>
       </c>
       <c r="F12" s="17" t="s">
-        <v>388</v>
+        <v>418</v>
       </c>
       <c r="G12" s="17" t="s">
         <v>81</v>
@@ -4736,22 +5081,22 @@
     </row>
     <row r="13" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A13" s="17" t="s">
-        <v>404</v>
+        <v>434</v>
       </c>
       <c r="B13" s="17" t="s">
-        <v>390</v>
+        <v>420</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>391</v>
+        <v>421</v>
       </c>
       <c r="D13" s="17" t="s">
-        <v>392</v>
+        <v>422</v>
       </c>
       <c r="E13" s="17" t="s">
-        <v>405</v>
+        <v>435</v>
       </c>
       <c r="F13" s="17" t="s">
-        <v>406</v>
+        <v>436</v>
       </c>
       <c r="G13" s="17" t="s">
         <v>81</v>
@@ -4759,22 +5104,22 @@
     </row>
     <row r="14" spans="1:7" ht="51" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
-        <v>407</v>
+        <v>437</v>
       </c>
       <c r="B14" s="17" t="s">
-        <v>357</v>
+        <v>387</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>408</v>
+        <v>438</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>359</v>
+        <v>389</v>
       </c>
       <c r="E14" s="17" t="s">
-        <v>409</v>
+        <v>439</v>
       </c>
       <c r="F14" s="17" t="s">
-        <v>410</v>
+        <v>440</v>
       </c>
       <c r="G14" s="17" t="s">
         <v>81</v>
@@ -4782,22 +5127,22 @@
     </row>
     <row r="15" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A15" s="17" t="s">
-        <v>411</v>
+        <v>441</v>
       </c>
       <c r="B15" s="17" t="s">
-        <v>364</v>
+        <v>394</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>412</v>
+        <v>442</v>
       </c>
       <c r="D15" s="17" t="s">
-        <v>359</v>
+        <v>389</v>
       </c>
       <c r="E15" s="17" t="s">
-        <v>413</v>
+        <v>443</v>
       </c>
       <c r="F15" s="17" t="s">
-        <v>414</v>
+        <v>444</v>
       </c>
       <c r="G15" s="17" t="s">
         <v>81</v>
@@ -4805,22 +5150,22 @@
     </row>
     <row r="16" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A16" s="17" t="s">
-        <v>415</v>
+        <v>445</v>
       </c>
       <c r="B16" s="17" t="s">
-        <v>369</v>
+        <v>399</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>416</v>
+        <v>446</v>
       </c>
       <c r="D16" s="17" t="s">
-        <v>359</v>
+        <v>389</v>
       </c>
       <c r="E16" s="17" t="s">
-        <v>417</v>
+        <v>447</v>
       </c>
       <c r="F16" s="17" t="s">
-        <v>418</v>
+        <v>448</v>
       </c>
       <c r="G16" s="17" t="s">
         <v>81</v>
@@ -4828,22 +5173,22 @@
     </row>
     <row r="17" spans="1:7" ht="51" x14ac:dyDescent="0.25">
       <c r="A17" s="17" t="s">
-        <v>419</v>
+        <v>449</v>
       </c>
       <c r="B17" s="17" t="s">
-        <v>420</v>
+        <v>450</v>
       </c>
       <c r="C17" s="17" t="s">
-        <v>421</v>
+        <v>451</v>
       </c>
       <c r="D17" s="17" t="s">
-        <v>387</v>
+        <v>417</v>
       </c>
       <c r="E17" s="17" t="s">
-        <v>422</v>
+        <v>452</v>
       </c>
       <c r="F17" s="17" t="s">
-        <v>423</v>
+        <v>453</v>
       </c>
       <c r="G17" s="17" t="s">
         <v>81</v>
@@ -4851,22 +5196,22 @@
     </row>
     <row r="18" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A18" s="17" t="s">
-        <v>424</v>
+        <v>454</v>
       </c>
       <c r="B18" s="17" t="s">
-        <v>364</v>
+        <v>394</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>425</v>
+        <v>455</v>
       </c>
       <c r="D18" s="17" t="s">
-        <v>359</v>
+        <v>389</v>
       </c>
       <c r="E18" s="17" t="s">
-        <v>426</v>
+        <v>456</v>
       </c>
       <c r="F18" s="17" t="s">
-        <v>427</v>
+        <v>457</v>
       </c>
       <c r="G18" s="17" t="s">
         <v>81</v>
@@ -4874,22 +5219,22 @@
     </row>
     <row r="19" spans="1:7" ht="51" x14ac:dyDescent="0.25">
       <c r="A19" s="17" t="s">
-        <v>428</v>
+        <v>458</v>
       </c>
       <c r="B19" s="17" t="s">
-        <v>369</v>
+        <v>399</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>429</v>
+        <v>459</v>
       </c>
       <c r="D19" s="17" t="s">
-        <v>359</v>
+        <v>389</v>
       </c>
       <c r="E19" s="17" t="s">
-        <v>430</v>
+        <v>460</v>
       </c>
       <c r="F19" s="17" t="s">
-        <v>418</v>
+        <v>448</v>
       </c>
       <c r="G19" s="17" t="s">
         <v>81</v>
@@ -4897,22 +5242,22 @@
     </row>
     <row r="20" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A20" s="17" t="s">
-        <v>431</v>
+        <v>461</v>
       </c>
       <c r="B20" s="17" t="s">
-        <v>420</v>
+        <v>450</v>
       </c>
       <c r="C20" s="17" t="s">
-        <v>432</v>
+        <v>462</v>
       </c>
       <c r="D20" s="17" t="s">
-        <v>387</v>
+        <v>417</v>
       </c>
       <c r="E20" s="17" t="s">
-        <v>433</v>
+        <v>463</v>
       </c>
       <c r="F20" s="17" t="s">
-        <v>434</v>
+        <v>464</v>
       </c>
       <c r="G20" s="17" t="s">
         <v>81</v>
@@ -4920,22 +5265,22 @@
     </row>
     <row r="21" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A21" s="17" t="s">
-        <v>435</v>
+        <v>465</v>
       </c>
       <c r="B21" s="17" t="s">
-        <v>364</v>
+        <v>394</v>
       </c>
       <c r="C21" s="17" t="s">
-        <v>436</v>
+        <v>466</v>
       </c>
       <c r="D21" s="17" t="s">
-        <v>359</v>
+        <v>389</v>
       </c>
       <c r="E21" s="17" t="s">
-        <v>437</v>
+        <v>467</v>
       </c>
       <c r="F21" s="17" t="s">
-        <v>427</v>
+        <v>457</v>
       </c>
       <c r="G21" s="17" t="s">
         <v>81</v>
@@ -4943,22 +5288,22 @@
     </row>
     <row r="22" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A22" s="17" t="s">
-        <v>438</v>
+        <v>468</v>
       </c>
       <c r="B22" s="17" t="s">
-        <v>369</v>
+        <v>399</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>439</v>
+        <v>469</v>
       </c>
       <c r="D22" s="17" t="s">
-        <v>359</v>
+        <v>389</v>
       </c>
       <c r="E22" s="17" t="s">
-        <v>417</v>
+        <v>447</v>
       </c>
       <c r="F22" s="17" t="s">
-        <v>418</v>
+        <v>448</v>
       </c>
       <c r="G22" s="17" t="s">
         <v>81</v>
@@ -4966,29 +5311,121 @@
     </row>
     <row r="23" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A23" s="17" t="s">
-        <v>440</v>
+        <v>470</v>
       </c>
       <c r="B23" s="17" t="s">
-        <v>420</v>
+        <v>450</v>
       </c>
       <c r="C23" s="17" t="s">
-        <v>441</v>
+        <v>471</v>
       </c>
       <c r="D23" s="17" t="s">
-        <v>387</v>
+        <v>417</v>
       </c>
       <c r="E23" s="17" t="s">
-        <v>442</v>
+        <v>472</v>
       </c>
       <c r="F23" s="17" t="s">
-        <v>443</v>
+        <v>473</v>
       </c>
       <c r="G23" s="17" t="s">
         <v>81</v>
       </c>
     </row>
+    <row r="24" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A24" s="17" t="s">
+        <v>474</v>
+      </c>
+      <c r="B24" s="17" t="s">
+        <v>387</v>
+      </c>
+      <c r="C24" s="17" t="s">
+        <v>475</v>
+      </c>
+      <c r="D24" s="17" t="s">
+        <v>389</v>
+      </c>
+      <c r="E24" s="17" t="s">
+        <v>476</v>
+      </c>
+      <c r="F24" s="17" t="s">
+        <v>477</v>
+      </c>
+      <c r="G24" s="17" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="17" t="s">
+        <v>478</v>
+      </c>
+      <c r="B25" s="17" t="s">
+        <v>394</v>
+      </c>
+      <c r="C25" s="17" t="s">
+        <v>479</v>
+      </c>
+      <c r="D25" s="17" t="s">
+        <v>389</v>
+      </c>
+      <c r="E25" s="17" t="s">
+        <v>480</v>
+      </c>
+      <c r="F25" s="17" t="s">
+        <v>457</v>
+      </c>
+      <c r="G25" s="17" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A26" s="17" t="s">
+        <v>481</v>
+      </c>
+      <c r="B26" s="17" t="s">
+        <v>399</v>
+      </c>
+      <c r="C26" s="17" t="s">
+        <v>482</v>
+      </c>
+      <c r="D26" s="17" t="s">
+        <v>389</v>
+      </c>
+      <c r="E26" s="17" t="s">
+        <v>483</v>
+      </c>
+      <c r="F26" s="17" t="s">
+        <v>448</v>
+      </c>
+      <c r="G26" s="17" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A27" s="17" t="s">
+        <v>484</v>
+      </c>
+      <c r="B27" s="17" t="s">
+        <v>450</v>
+      </c>
+      <c r="C27" s="17" t="s">
+        <v>485</v>
+      </c>
+      <c r="D27" s="17" t="s">
+        <v>417</v>
+      </c>
+      <c r="E27" s="17" t="s">
+        <v>486</v>
+      </c>
+      <c r="F27" s="17" t="s">
+        <v>487</v>
+      </c>
+      <c r="G27" s="17" t="s">
+        <v>81</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G23" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
+  <autoFilter ref="A1:G27" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5007,39 +5444,39 @@
   <sheetData>
     <row r="1" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>444</v>
+        <v>488</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>445</v>
+        <v>489</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>446</v>
+        <v>490</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>355</v>
+        <v>385</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>447</v>
+        <v>491</v>
       </c>
       <c r="F1" s="16" t="s">
-        <v>448</v>
+        <v>492</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
-        <v>449</v>
+        <v>493</v>
       </c>
       <c r="B2" s="17" t="s">
         <v>67</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>450</v>
+        <v>494</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>362</v>
+        <v>392</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>451</v>
+        <v>495</v>
       </c>
       <c r="F2" s="17" t="s">
         <v>83</v>
@@ -5047,19 +5484,19 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
-        <v>452</v>
+        <v>496</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>453</v>
+        <v>497</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>454</v>
+        <v>498</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>362</v>
+        <v>392</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>455</v>
+        <v>499</v>
       </c>
       <c r="F3" s="17" t="s">
         <v>83</v>
@@ -5067,56 +5504,56 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>456</v>
+        <v>500</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>457</v>
+        <v>501</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>458</v>
+        <v>502</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>362</v>
+        <v>392</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>459</v>
+        <v>503</v>
       </c>
       <c r="F4" s="17" t="s">
-        <v>460</v>
+        <v>504</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>461</v>
+        <v>505</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>462</v>
+        <v>506</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>463</v>
+        <v>507</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>362</v>
+        <v>392</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>464</v>
+        <v>508</v>
       </c>
       <c r="F5" s="17" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
-        <v>465</v>
+        <v>509</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>466</v>
+        <v>510</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>467</v>
+        <v>511</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>362</v>
+        <v>392</v>
       </c>
       <c r="E6" s="17" t="s">
         <v>26</v>
@@ -5127,119 +5564,119 @@
     </row>
     <row r="7" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
-        <v>468</v>
+        <v>512</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>469</v>
+        <v>513</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>470</v>
+        <v>514</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>362</v>
+        <v>392</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>471</v>
+        <v>515</v>
       </c>
       <c r="F7" s="17" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
-        <v>472</v>
+        <v>516</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>473</v>
+        <v>517</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>474</v>
+        <v>518</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>362</v>
+        <v>392</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>475</v>
+        <v>519</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>476</v>
+        <v>520</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>477</v>
+        <v>521</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>478</v>
+        <v>522</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>362</v>
+        <v>392</v>
       </c>
       <c r="E9" s="17" t="s">
-        <v>475</v>
+        <v>519</v>
       </c>
       <c r="F9" s="17" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="17" t="s">
-        <v>479</v>
+        <v>523</v>
       </c>
       <c r="B10" s="17" t="s">
         <v>52</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>480</v>
+        <v>524</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>362</v>
+        <v>392</v>
       </c>
       <c r="E10" s="17" t="s">
         <v>51</v>
       </c>
       <c r="F10" s="17" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="51" x14ac:dyDescent="0.25">
       <c r="A11" s="17" t="s">
-        <v>481</v>
+        <v>525</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>482</v>
+        <v>526</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>483</v>
+        <v>527</v>
       </c>
       <c r="D11" s="17" t="s">
         <v>81</v>
       </c>
       <c r="E11" s="17" t="s">
-        <v>484</v>
+        <v>528</v>
       </c>
       <c r="F11" s="17" t="s">
-        <v>485</v>
+        <v>529</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
-        <v>486</v>
+        <v>530</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>487</v>
+        <v>531</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>488</v>
+        <v>532</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>362</v>
+        <v>392</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>489</v>
+        <v>533</v>
       </c>
       <c r="F12" s="17" t="s">
         <v>96</v>
@@ -5247,22 +5684,22 @@
     </row>
     <row r="13" spans="1:6" ht="51" x14ac:dyDescent="0.25">
       <c r="A13" s="17" t="s">
-        <v>490</v>
+        <v>534</v>
       </c>
       <c r="B13" s="17" t="s">
-        <v>491</v>
+        <v>535</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>492</v>
+        <v>536</v>
       </c>
       <c r="D13" s="17" t="s">
         <v>81</v>
       </c>
       <c r="E13" s="17" t="s">
-        <v>493</v>
+        <v>537</v>
       </c>
       <c r="F13" s="17" t="s">
-        <v>159</v>
+        <v>538</v>
       </c>
     </row>
   </sheetData>
@@ -5285,121 +5722,121 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>494</v>
+        <v>539</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>495</v>
+        <v>540</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>496</v>
+        <v>541</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>497</v>
+        <v>542</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>498</v>
+        <v>543</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
-        <v>499</v>
+        <v>544</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>500</v>
+        <v>545</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>501</v>
+        <v>546</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>502</v>
+        <v>547</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>503</v>
+        <v>548</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
-        <v>504</v>
+        <v>549</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>505</v>
+        <v>550</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>506</v>
+        <v>551</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>507</v>
+        <v>552</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>508</v>
+        <v>553</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>509</v>
+        <v>554</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>510</v>
+        <v>555</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>510</v>
+        <v>555</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>511</v>
+        <v>556</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>512</v>
+        <v>557</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>513</v>
+        <v>558</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>514</v>
+        <v>559</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>515</v>
+        <v>560</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>516</v>
+        <v>561</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>508</v>
+        <v>553</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
-        <v>517</v>
+        <v>562</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>518</v>
+        <v>563</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>518</v>
+        <v>563</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>519</v>
+        <v>564</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>503</v>
+        <v>548</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
-        <v>520</v>
+        <v>565</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>521</v>
+        <v>566</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>522</v>
+        <v>567</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>523</v>
+        <v>568</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>503</v>
+        <v>548</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Checkpoint: tracker, session state and the owner's D-012 steps (Doctor v0, CI isolation, S1-S5)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/SMARTDOC_2_0_MASTER_TRACKER.xlsx
+++ b/docs/SMARTDOC_2_0_MASTER_TRACKER.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\speed\Desktop\Claude - ПРОЕКТ\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A36C7A77-99E8-45C6-ADB6-CDB3C484D947}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79E22CCE-591B-49A0-BBB5-9EE59E662F39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,12 +22,12 @@
     <sheet name="Release Readiness" sheetId="7" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Bugs!$A$1:$H$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Decisions!$A$1:$F$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Bugs!$A$1:$H$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Decisions!$A$1:$F$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Release Readiness'!$A$1:$E$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Roadmap!$A$1:$F$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Tasks!$A$1:$P$34</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Tests!$A$1:$G$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Tasks!$A$1:$P$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Tests!$A$1:$G$37</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1105" uniqueCount="647">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1219" uniqueCount="709">
   <si>
     <t>SmartDoc 2.0 -- master tracker</t>
   </si>
@@ -241,7 +241,7 @@
     <t>P4 (E2), owner approval</t>
   </si>
   <si>
-    <t>Analysis done (S2-080); Doctor v0 MVP planned (S2-081)</t>
+    <t>Analysis done (S2-080); Doctor v0 prototype built and measured (S2-081, behind ?doctor=1)</t>
   </si>
   <si>
     <t>Task ID</t>
@@ -841,66 +841,69 @@
     <t>Owner + Claude</t>
   </si>
   <si>
+    <t>f48e84a</t>
+  </si>
+  <si>
+    <t>Isolated GitHub Actions workflow on a throwaway PostgreSQL (no secrets, read-only token): https://github.com/Drajeto07/claude/actions/runs/38701081333 -- empty database, migrations up / check / down / up, isolation tests 49 passed (owner's negative cases incl. wrong/missing bucket through the real S3 code, missing configuration, production resources, no start-up writes or worker while unproven, wrong database id and second marker row on PostgreSQL), every PostgreSQL-marked test 14 passed.</t>
+  </si>
+  <si>
+    <t>S1 project smartdoc-preview (ksmwhnnupkrtzrupcitc, free, $0 checked); S4 schema on the new empty project only (head d41f7a60c9e2, 16 tables, RLS on all, same as production -- production only read); S5 database marker written, private bucket created, bucket marker file docs/d012-preview/identity.json waits for the owner's upload; S2 (password) and S3 key pair: owner, in Supabase. NOT done (owner): S6 Vercel variables, S7 switching redeploy, S8 Free Design writes, S9 old test accounts.</t>
+  </si>
+  <si>
+    <t>S2-023</t>
+  </si>
+  <si>
+    <t>Look step on phones: lighter template choice</t>
+  </si>
+  <si>
+    <t>On phones each template card with its sample is tall; a compact list (name + small swatch, sample on demand) or a horizontal carousel, the suggestion first.</t>
+  </si>
+  <si>
+    <t>All five templates reachable within two screen heights at 375 px; selected state unchanged; no horizontal page scroll</t>
+  </si>
+  <si>
+    <t>Owner review 2026-10-14; not blocking E1.</t>
+  </si>
+  <si>
+    <t>S2-024</t>
+  </si>
+  <si>
+    <t>Structure review: a readable preview of tables</t>
+  </si>
+  <si>
+    <t>A table row in the structure check shows its size (rows x columns), header row and first cells as a small grid instead of one line of text; tables with merged cells marked.</t>
+  </si>
+  <si>
+    <t>Tables recognisable at a glance in EN/BG; long tables don't push the outline away</t>
+  </si>
+  <si>
+    <t>S2-025</t>
+  </si>
+  <si>
+    <t>Projects screen: gallery like the dashboard</t>
+  </si>
+  <si>
+    <t>/documents as a grid of project cards with real thumbnails (list view as an option), filters (type, status), sort and search kept, batch actions kept.</t>
+  </si>
+  <si>
+    <t>Same functions as today's list (search, sort, pages, batch, compare, delete) with thumbnails; EN/BG; light/dark; no thumbnail rendering on list requests</t>
+  </si>
+  <si>
+    <t>S2-031</t>
+  </si>
+  <si>
+    <t>Editor 2.0, E2: selection model, command registry, contextual toolbar, one Undo/Redo (behind ?editor=2)</t>
+  </si>
+  <si>
+    <t>Shared selection model (none/text/table/image); central command registry (toolbar, shortcuts); contextual toolbar by selection; unified Undo/Redo (typing first, then saved steps); panels hide/show; phone page navigation, zoom, Fit width; every editor bar, dialog and panel bilingual and on the theme tokens.</t>
+  </si>
+  <si>
+    <t>Editing, Undo/Redo, autosave, reload, failed save; DOCX/PDF; axe; phone; classic and new editor on the same documents; BG/EN; light/dark</t>
+  </si>
+  <si>
     <t>029acd4</t>
   </si>
   <si>
-    <t>tests/test_preview_isolation.py 30 (28 pass locally; the 2 PostgreSQL setup-script tests have NOT run yet: CI runs only on pull requests and main, and Docker Desktop was not running -- they must pass before step S5): pooler/direct/any-case production URLs refused at start, missing ref or ids refused, identity markers -- missing, second row, other environment, other instance, unreadable, bucket missing -- all refused; unproven preview: 503 on every route but health, retried after 30 s; production/local untouched; fingerprints differ on one pooler; backend 2647 passed / 13 skipped</t>
-  </si>
-  <si>
-    <t>Plan rev 2 (docs/SMARTDOC_2_0_PREVIEW_ISOLATION_PLAN.md) answers the owner's 6 points; section 9 lists S1-S9 awaiting permission. Nothing switched; no cloud resource, Vercel variable or Production data touched. The guard is inactive until SMARTDOC_ENVIRONMENT is set in the approved switch.</t>
-  </si>
-  <si>
-    <t>S2-023</t>
-  </si>
-  <si>
-    <t>Look step on phones: lighter template choice</t>
-  </si>
-  <si>
-    <t>On phones each template card with its sample is tall; a compact list (name + small swatch, sample on demand) or a horizontal carousel, the suggestion first.</t>
-  </si>
-  <si>
-    <t>All five templates reachable within two screen heights at 375 px; selected state unchanged; no horizontal page scroll</t>
-  </si>
-  <si>
-    <t>Owner review 2026-10-14; not blocking E1.</t>
-  </si>
-  <si>
-    <t>S2-024</t>
-  </si>
-  <si>
-    <t>Structure review: a readable preview of tables</t>
-  </si>
-  <si>
-    <t>A table row in the structure check shows its size (rows x columns), header row and first cells as a small grid instead of one line of text; tables with merged cells marked.</t>
-  </si>
-  <si>
-    <t>Tables recognisable at a glance in EN/BG; long tables don't push the outline away</t>
-  </si>
-  <si>
-    <t>S2-025</t>
-  </si>
-  <si>
-    <t>Projects screen: gallery like the dashboard</t>
-  </si>
-  <si>
-    <t>/documents as a grid of project cards with real thumbnails (list view as an option), filters (type, status), sort and search kept, batch actions kept.</t>
-  </si>
-  <si>
-    <t>Same functions as today's list (search, sort, pages, batch, compare, delete) with thumbnails; EN/BG; light/dark; no thumbnail rendering on list requests</t>
-  </si>
-  <si>
-    <t>S2-031</t>
-  </si>
-  <si>
-    <t>Editor 2.0, E2: selection model, command registry, contextual toolbar, one Undo/Redo (behind ?editor=2)</t>
-  </si>
-  <si>
-    <t>Shared selection model (none/text/table/image); central command registry (toolbar, shortcuts); contextual toolbar by selection; unified Undo/Redo (typing first, then saved steps); panels hide/show; phone page navigation, zoom, Fit width; every editor bar, dialog and panel bilingual and on the theme tokens.</t>
-  </si>
-  <si>
-    <t>Editing, Undo/Redo, autosave, reload, failed save; DOCX/PDF; axe; phone; classic and new editor on the same documents; BG/EN; light/dark</t>
-  </si>
-  <si>
     <t>smartdoc-git-feature-smartdoc-20-drajeto.vercel.app (see SESSION_STATE for the deployment)</t>
   </si>
   <si>
@@ -937,19 +940,64 @@
     <t>S2-081</t>
   </si>
   <si>
-    <t>Doctor v0 (Word): five verified repairs + three flags, defect corpus, invariant tests</t>
-  </si>
-  <si>
-    <t>Empty paragraphs as spacing, one role in several looks, repeated direct formatting, too-wide tables/pictures, typed numbering -&gt; Word numbering (labels checked against Word); flags: heading jumps, alt text, malformed links. Every repair verified (words, untouched blocks, valid package) or rolled back.</t>
+    <t>Doctor v0 (Word): verified repairs behind ?doctor=1 (prototype)</t>
+  </si>
+  <si>
+    <t>Upload DOCX -&gt; analyse -&gt; proposed repairs -&gt; review -&gt; repaired file -&gt; SafeEdit check -&gt; download only when verified. Repairs in the Word file (empty paragraphs as spacing, too-wide pictures/tables) and safe editor repairs (proposals). Refusals: no Word file, unusable source, import word check not passed, undecided tracked changes, signed, macros, damaged package, a file the export itself would change; per block: preserved features.</t>
   </si>
   <si>
     <t>S2-080, owner approval after E2</t>
   </si>
   <si>
-    <t>On the labelled corpus: 100% text preservation, 100% untouched-block identity, 100% valid packages; precision &gt;= 95% for the five repairs; recall reported</t>
-  </si>
-  <si>
-    <t>Not started (no large implementation without approval). Open: size limit, real anonymised documents, competitor trial (cost).</t>
+    <t>Every repaired file verified (words, header/footer words, untouched blocks byte for byte, preserved features, valid package) or nothing handed out; refused files say why; original never written; no AI; feature flag</t>
+  </si>
+  <si>
+    <t>4f75d19</t>
+  </si>
+  <si>
+    <t>tests/test_doctor.py 72 (whole Word corpus refused-for-a-reason or verified; labelled corpus vs ground truth; each SafeEdit check caught on a damaged result; refusals; repairs in the file never touch tables, last paragraph, carriers; skipped when not lined up), tests/test_doctor_api.py 9, e2e/doctor.spec.ts 4 (flag, full flow + download, signed refused, Bulgarian), axe light/dark on the panel. Measured: 15/23 planted defects repaired (65 %), 15/15 of the kinds v0 repairs bar one left on purpose; 0 wrong proposals.</t>
+  </si>
+  <si>
+    <t>Gaps: fonts set on a whole paragraph (imported as a paragraph rule), formatting repeating the style (folded away on import). SafeEdit found: the export rewrites a neighbouring block when the editor rewrites a table (B-022) -- mitigated by preferring repairs in the file. Not a finished product.</t>
+  </si>
+  <si>
+    <t>S2-026</t>
+  </si>
+  <si>
+    <t>More readable mobile editor view</t>
+  </si>
+  <si>
+    <t>Bigger default reading zoom on phones, comfortable line length, quicker page navigation.</t>
+  </si>
+  <si>
+    <t>Owner's UI backlog 2026-10-15</t>
+  </si>
+  <si>
+    <t>S2-027</t>
+  </si>
+  <si>
+    <t>Compact mobile toolbar</t>
+  </si>
+  <si>
+    <t>On phones the contextual toolbar takes two rows: one row with the most used tools, the rest behind 'More'.</t>
+  </si>
+  <si>
+    <t>S2-028</t>
+  </si>
+  <si>
+    <t>Backend messages in both languages</t>
+  </si>
+  <si>
+    <t>Health check titles/summaries, version descriptions, SafeEdit check details and export notes come from the server in English: message codes + parameters, worded by the client's dictionaries.</t>
+  </si>
+  <si>
+    <t>S2-083</t>
+  </si>
+  <si>
+    <t>Doctor: repairs for paragraph-level fonts and repeated formatting (in the file)</t>
+  </si>
+  <si>
+    <t>The two measured gaps of v0, as minimal edits in the Word file, verified by SafeEdit.</t>
   </si>
   <si>
     <t>Bug ID</t>
@@ -1339,6 +1387,63 @@
     <t>docs/ui-review/2026-10-14d/e2-light-history-bg.png, e2-dark-review-bg.png</t>
   </si>
   <si>
+    <t>B-021</t>
+  </si>
+  <si>
+    <t>Export to PDF a Word paragraph marked right to left that starts with a Latin word (a11-multilingual, on a machine with shaping)</t>
+  </si>
+  <si>
+    <t>Words in reading order, right to left</t>
+  </si>
+  <si>
+    <t>The line's words drawn in reverse order (each word itself correct)</t>
+  </si>
+  <si>
+    <t>pdf_export._for_text honours the paragraph's own direction (27e3bfc)</t>
+  </si>
+  <si>
+    <t>tests/test_multilingual.py: 2 new tests fail without the fix; a11 Hebrew reads back exactly</t>
+  </si>
+  <si>
+    <t>B-022</t>
+  </si>
+  <si>
+    <t>Editor repair rewrites a table (layout fix) in a Word-backed document, export into the original</t>
+  </si>
+  <si>
+    <t>Only the table's block changes</t>
+  </si>
+  <si>
+    <t>The empty paragraph after the table is rewritten too (found by SafeEdit on d13)</t>
+  </si>
+  <si>
+    <t>OPEN</t>
+  </si>
+  <si>
+    <t>Mitigated in Doctor: repairs in the file are preferred and the overlapping editor repair dropped; exporter root cause open</t>
+  </si>
+  <si>
+    <t>tests/test_doctor.py d13 verified</t>
+  </si>
+  <si>
+    <t>B-023</t>
+  </si>
+  <si>
+    <t>a11-multilingual exported to PDF, text copied</t>
+  </si>
+  <si>
+    <t>Arabic yeh U+064A</t>
+  </si>
+  <si>
+    <t>Persian yeh U+06CC in 2 words (same glyph in those positions)</t>
+  </si>
+  <si>
+    <t>Known limit of the PDF text layer; the word check stays 'changed'</t>
+  </si>
+  <si>
+    <t>scratchpad investigation; docs analysis section 13</t>
+  </si>
+  <si>
     <t>Test ID</t>
   </si>
   <si>
@@ -1735,6 +1840,75 @@
     <t>docs/ui-review/2026-10-14d/</t>
   </si>
   <si>
+    <t>T-032</t>
+  </si>
+  <si>
+    <t>CI</t>
+  </si>
+  <si>
+    <t>Isolated PostgreSQL workflow: empty DB, migrations, 49 isolation + 14 PostgreSQL tests</t>
+  </si>
+  <si>
+    <t>GitHub Actions, throwaway postgres:17, no secrets</t>
+  </si>
+  <si>
+    <t>https://github.com/Drajeto07/claude/actions/runs/38701081333</t>
+  </si>
+  <si>
+    <t>T-033</t>
+  </si>
+  <si>
+    <t>Doctor v0: corpus invariants, labelled corpus, SafeEdit tamper tests, refusals</t>
+  </si>
+  <si>
+    <t>PASS 72</t>
+  </si>
+  <si>
+    <t>tests/test_doctor.py</t>
+  </si>
+  <si>
+    <t>T-034</t>
+  </si>
+  <si>
+    <t>Doctor API: flow, refusals, flag, other user's document, original kept</t>
+  </si>
+  <si>
+    <t>PASS 9 (+4 routes in the security suite)</t>
+  </si>
+  <si>
+    <t>tests/test_doctor_api.py</t>
+  </si>
+  <si>
+    <t>T-035</t>
+  </si>
+  <si>
+    <t>Doctor panel: flag, check-choose-verify-download, signed refused, Bulgarian; axe light/dark</t>
+  </si>
+  <si>
+    <t>PASS 5</t>
+  </si>
+  <si>
+    <t>e2e/doctor.spec.ts, e2e/accessibility.spec.ts</t>
+  </si>
+  <si>
+    <t>T-036</t>
+  </si>
+  <si>
+    <t>Fidelity</t>
+  </si>
+  <si>
+    <t>The 1 of 111 unverified content check investigated (a11 PDF on Windows)</t>
+  </si>
+  <si>
+    <t>Local, pypdfium2 render + glyph positions</t>
+  </si>
+  <si>
+    <t>Real RTL defect fixed (B-021); 2-letter text-layer limit documented (B-023)</t>
+  </si>
+  <si>
+    <t>docs/SMARTDOC_DOCUMENT_DOCTOR_SAFEEDIT_ANALYSIS.md section 13</t>
+  </si>
+  <si>
     <t>Decision ID</t>
   </si>
   <si>
@@ -1879,7 +2053,7 @@
     <t>Canvas documents and the shared database</t>
   </si>
   <si>
-    <t>DECIDED 2026-10-14 (owner): option (a). Plan revision 2 (2026-10-14): all Previews on one separate project, no Production credential for any Preview, fail-closed identity guard, rollback never back to Production. The switch waits for the owner's approval of each step S1-S9.</t>
+    <t>Option (a). Rev 2 approved in part (2026-10-15): S1-S5 done (separate free project, schema, markers, private bucket; production only read); S6-S9 refused for now (no Vercel variables, no switching redeploy, no Free Design writes, old test accounts untouched).</t>
   </si>
   <si>
     <t>S2-050, P5 persistence</t>
@@ -1898,6 +2072,18 @@
   </si>
   <si>
     <t>S2-080, S2-081</t>
+  </si>
+  <si>
+    <t>D-014</t>
+  </si>
+  <si>
+    <t>Doctor v0 architecture</t>
+  </si>
+  <si>
+    <t>Repairs either in the Word file itself (minimal edits) or in the editor (proposals); the smaller edit wins on the same block; a repaired file is handed out only when SafeEdit verified it against the original; refusals are explicit; deterministic, no AI; prototype behind ?doctor=1 and DOCTOR_ENABLED.</t>
+  </si>
+  <si>
+    <t>S2-081, S2-083</t>
   </si>
   <si>
     <t>Requirement</t>
@@ -2617,12 +2803,12 @@
         <v>5</v>
       </c>
       <c r="B5" s="5">
-        <f>COUNTIF(Tasks!$G$2:$G$34,A5)</f>
-        <v>6</v>
+        <f>COUNTIF(Tasks!$G$2:$G$38,A5)</f>
+        <v>9</v>
       </c>
       <c r="C5" s="5">
         <f>COUNTIF(Roadmap!$D$2:$D$11,A5)</f>
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -2630,7 +2816,7 @@
         <v>6</v>
       </c>
       <c r="B6" s="5">
-        <f>COUNTIF(Tasks!$G$2:$G$34,A6)</f>
+        <f>COUNTIF(Tasks!$G$2:$G$38,A6)</f>
         <v>0</v>
       </c>
       <c r="C6" s="5">
@@ -2643,12 +2829,12 @@
         <v>7</v>
       </c>
       <c r="B7" s="5">
-        <f>COUNTIF(Tasks!$G$2:$G$34,A7)</f>
-        <v>1</v>
+        <f>COUNTIF(Tasks!$G$2:$G$38,A7)</f>
+        <v>2</v>
       </c>
       <c r="C7" s="5">
         <f>COUNTIF(Roadmap!$D$2:$D$11,A7)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -2656,8 +2842,8 @@
         <v>8</v>
       </c>
       <c r="B8" s="5">
-        <f>COUNTIF(Tasks!$G$2:$G$34,A8)</f>
-        <v>1</v>
+        <f>COUNTIF(Tasks!$G$2:$G$38,A8)</f>
+        <v>0</v>
       </c>
       <c r="C8" s="5">
         <f>COUNTIF(Roadmap!$D$2:$D$11,A8)</f>
@@ -2669,8 +2855,8 @@
         <v>9</v>
       </c>
       <c r="B9" s="5">
-        <f>COUNTIF(Tasks!$G$2:$G$34,A9)</f>
-        <v>0</v>
+        <f>COUNTIF(Tasks!$G$2:$G$38,A9)</f>
+        <v>1</v>
       </c>
       <c r="C9" s="5">
         <f>COUNTIF(Roadmap!$D$2:$D$11,A9)</f>
@@ -2682,7 +2868,7 @@
         <v>10</v>
       </c>
       <c r="B10" s="5">
-        <f>COUNTIF(Tasks!$G$2:$G$34,A10)</f>
+        <f>COUNTIF(Tasks!$G$2:$G$38,A10)</f>
         <v>20</v>
       </c>
       <c r="C10" s="5">
@@ -2695,7 +2881,7 @@
         <v>11</v>
       </c>
       <c r="B11" s="5">
-        <f>COUNTIF(Tasks!$G$2:$G$34,A11)</f>
+        <f>COUNTIF(Tasks!$G$2:$G$38,A11)</f>
         <v>5</v>
       </c>
       <c r="C11" s="5">
@@ -2709,7 +2895,7 @@
       </c>
       <c r="B12" s="12">
         <f>SUM(B5:B11)</f>
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="C12" s="12">
         <f>SUM(C5:C11)</f>
@@ -2722,7 +2908,7 @@
       </c>
       <c r="B13" s="14">
         <f>IFERROR((B11+B10)/B12,0)</f>
-        <v>0.75757575757575757</v>
+        <v>0.67567567567567566</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -2730,7 +2916,7 @@
         <v>14</v>
       </c>
       <c r="B14">
-        <f>COUNTIFS(Tasks!$F$2:$F$34,"P0",Tasks!$G$2:$G$34,"&lt;&gt;DONE",Tasks!$G$2:$G$34,"&lt;&gt;VERIFIED")</f>
+        <f>COUNTIFS(Tasks!$F$2:$F$38,"P0",Tasks!$G$2:$G$38,"&lt;&gt;DONE",Tasks!$G$2:$G$38,"&lt;&gt;VERIFIED")</f>
         <v>1</v>
       </c>
     </row>
@@ -2739,8 +2925,8 @@
         <v>15</v>
       </c>
       <c r="B15">
-        <f>COUNTA(Bugs!$A$2:$A$21)-COUNTIF(Bugs!$F$2:$F$21,"DONE")-COUNTIF(Bugs!$F$2:$F$21,"VERIFIED")</f>
-        <v>2</v>
+        <f>COUNTA(Bugs!$A$2:$A$24)-COUNTIF(Bugs!$F$2:$F$24,"DONE")-COUNTIF(Bugs!$F$2:$F$24,"VERIFIED")</f>
+        <v>4</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
@@ -2974,7 +3160,7 @@
         <v>62</v>
       </c>
       <c r="D11" s="17" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E11" s="17" t="s">
         <v>63</v>
@@ -3014,7 +3200,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:P34"/>
+  <dimension ref="A1:P38"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
@@ -4352,7 +4538,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="28" spans="1:16" ht="318.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:16" ht="280.5" x14ac:dyDescent="0.25">
       <c r="A28" s="17" t="s">
         <v>258</v>
       </c>
@@ -4372,7 +4558,7 @@
         <v>22</v>
       </c>
       <c r="G28" s="17" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H28" s="17"/>
       <c r="I28" s="17" t="s">
@@ -4565,36 +4751,36 @@
         <v>84</v>
       </c>
       <c r="L32" s="17" t="s">
-        <v>264</v>
+        <v>284</v>
       </c>
       <c r="M32" s="17" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="N32" s="17" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="O32" s="17" t="s">
         <v>86</v>
       </c>
       <c r="P32" s="17" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
     </row>
     <row r="33" spans="1:16" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A33" s="17" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B33" s="17" t="s">
         <v>60</v>
       </c>
       <c r="C33" s="17" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D33" s="17" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="E33" s="17" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="F33" s="17" t="s">
         <v>30</v>
@@ -4603,10 +4789,10 @@
         <v>11</v>
       </c>
       <c r="H33" s="17" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="I33" s="17" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="J33" s="17" t="s">
         <v>83</v>
@@ -4615,46 +4801,46 @@
         <v>84</v>
       </c>
       <c r="L33" s="17" t="s">
-        <v>264</v>
+        <v>284</v>
       </c>
       <c r="M33" s="17"/>
       <c r="N33" s="17" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="O33" s="17" t="s">
         <v>86</v>
       </c>
       <c r="P33" s="17" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="34" spans="1:16" ht="63.75" x14ac:dyDescent="0.25">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16" ht="280.5" x14ac:dyDescent="0.25">
       <c r="A34" s="17" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B34" s="17" t="s">
         <v>60</v>
       </c>
       <c r="C34" s="17" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D34" s="17" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E34" s="17" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="F34" s="17" t="s">
         <v>30</v>
       </c>
       <c r="G34" s="17" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="H34" s="17" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="I34" s="17" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="J34" s="17" t="s">
         <v>83</v>
@@ -4662,19 +4848,189 @@
       <c r="K34" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="L34" s="17"/>
+      <c r="L34" s="17" t="s">
+        <v>301</v>
+      </c>
       <c r="M34" s="17"/>
-      <c r="N34" s="17"/>
+      <c r="N34" s="17" t="s">
+        <v>302</v>
+      </c>
       <c r="O34" s="17" t="s">
         <v>86</v>
       </c>
       <c r="P34" s="17" t="s">
-        <v>300</v>
-      </c>
+        <v>303</v>
+      </c>
+    </row>
+    <row r="35" spans="1:16" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A35" s="17" t="s">
+        <v>304</v>
+      </c>
+      <c r="B35" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="C35" s="17" t="s">
+        <v>121</v>
+      </c>
+      <c r="D35" s="17" t="s">
+        <v>305</v>
+      </c>
+      <c r="E35" s="17" t="s">
+        <v>306</v>
+      </c>
+      <c r="F35" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="G35" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="H35" s="17" t="s">
+        <v>280</v>
+      </c>
+      <c r="I35" s="17"/>
+      <c r="J35" s="17" t="s">
+        <v>83</v>
+      </c>
+      <c r="K35" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="L35" s="17"/>
+      <c r="M35" s="17"/>
+      <c r="N35" s="17"/>
+      <c r="O35" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="P35" s="17" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A36" s="17" t="s">
+        <v>308</v>
+      </c>
+      <c r="B36" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="C36" s="17" t="s">
+        <v>121</v>
+      </c>
+      <c r="D36" s="17" t="s">
+        <v>309</v>
+      </c>
+      <c r="E36" s="17" t="s">
+        <v>310</v>
+      </c>
+      <c r="F36" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="G36" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="H36" s="17" t="s">
+        <v>280</v>
+      </c>
+      <c r="I36" s="17"/>
+      <c r="J36" s="17" t="s">
+        <v>83</v>
+      </c>
+      <c r="K36" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="L36" s="17"/>
+      <c r="M36" s="17"/>
+      <c r="N36" s="17"/>
+      <c r="O36" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="P36" s="17" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A37" s="17" t="s">
+        <v>311</v>
+      </c>
+      <c r="B37" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="C37" s="17" t="s">
+        <v>186</v>
+      </c>
+      <c r="D37" s="17" t="s">
+        <v>312</v>
+      </c>
+      <c r="E37" s="17" t="s">
+        <v>313</v>
+      </c>
+      <c r="F37" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="G37" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="H37" s="17" t="s">
+        <v>280</v>
+      </c>
+      <c r="I37" s="17"/>
+      <c r="J37" s="17" t="s">
+        <v>83</v>
+      </c>
+      <c r="K37" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="L37" s="17"/>
+      <c r="M37" s="17"/>
+      <c r="N37" s="17"/>
+      <c r="O37" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="P37" s="17" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A38" s="17" t="s">
+        <v>314</v>
+      </c>
+      <c r="B38" s="17" t="s">
+        <v>60</v>
+      </c>
+      <c r="C38" s="17" t="s">
+        <v>289</v>
+      </c>
+      <c r="D38" s="17" t="s">
+        <v>315</v>
+      </c>
+      <c r="E38" s="17" t="s">
+        <v>316</v>
+      </c>
+      <c r="F38" s="17" t="s">
+        <v>30</v>
+      </c>
+      <c r="G38" s="17" t="s">
+        <v>5</v>
+      </c>
+      <c r="H38" s="17" t="s">
+        <v>296</v>
+      </c>
+      <c r="I38" s="17"/>
+      <c r="J38" s="17" t="s">
+        <v>83</v>
+      </c>
+      <c r="K38" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="L38" s="17"/>
+      <c r="M38" s="17"/>
+      <c r="N38" s="17"/>
+      <c r="O38" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="P38" s="17"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P34" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
-  <conditionalFormatting sqref="G2:G34">
+  <autoFilter ref="A1:P38" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
+  <conditionalFormatting sqref="G2:G38">
     <cfRule type="expression" dxfId="13" priority="1">
       <formula>$G2="BACKLOG"</formula>
     </cfRule>
@@ -4703,7 +5059,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -4718,551 +5074,629 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>301</v>
+        <v>317</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>302</v>
+        <v>318</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>303</v>
+        <v>319</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>304</v>
+        <v>320</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>305</v>
+        <v>321</v>
       </c>
       <c r="F1" s="16" t="s">
         <v>2</v>
       </c>
       <c r="G1" s="16" t="s">
-        <v>306</v>
+        <v>322</v>
       </c>
       <c r="H1" s="16" t="s">
-        <v>307</v>
+        <v>323</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
-        <v>308</v>
+        <v>324</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>309</v>
+        <v>325</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>310</v>
+        <v>326</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>311</v>
+        <v>327</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>312</v>
+        <v>328</v>
       </c>
       <c r="F2" s="17" t="s">
         <v>8</v>
       </c>
       <c r="G2" s="17" t="s">
-        <v>313</v>
+        <v>329</v>
       </c>
       <c r="H2" s="17" t="s">
-        <v>314</v>
+        <v>330</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
-        <v>315</v>
+        <v>331</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>316</v>
+        <v>332</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>317</v>
+        <v>333</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>318</v>
+        <v>334</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>319</v>
+        <v>335</v>
       </c>
       <c r="F3" s="17" t="s">
         <v>5</v>
       </c>
       <c r="G3" s="17"/>
       <c r="H3" s="17" t="s">
-        <v>320</v>
+        <v>336</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>321</v>
+        <v>337</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>316</v>
+        <v>332</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>322</v>
+        <v>338</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>323</v>
+        <v>339</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>324</v>
+        <v>340</v>
       </c>
       <c r="F4" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G4" s="17" t="s">
-        <v>325</v>
+        <v>341</v>
       </c>
       <c r="H4" s="17" t="s">
-        <v>326</v>
+        <v>342</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>327</v>
+        <v>343</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>328</v>
+        <v>344</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>329</v>
+        <v>345</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>330</v>
+        <v>346</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>331</v>
+        <v>347</v>
       </c>
       <c r="F5" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G5" s="17" t="s">
-        <v>332</v>
+        <v>348</v>
       </c>
       <c r="H5" s="17" t="s">
-        <v>333</v>
+        <v>349</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="51" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
-        <v>334</v>
+        <v>350</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>328</v>
+        <v>344</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>335</v>
+        <v>351</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>336</v>
+        <v>352</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>337</v>
+        <v>353</v>
       </c>
       <c r="F6" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G6" s="17" t="s">
-        <v>338</v>
+        <v>354</v>
       </c>
       <c r="H6" s="17" t="s">
-        <v>339</v>
+        <v>355</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
-        <v>340</v>
+        <v>356</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>328</v>
+        <v>344</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>341</v>
+        <v>357</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>342</v>
+        <v>358</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>343</v>
+        <v>359</v>
       </c>
       <c r="F7" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G7" s="17" t="s">
-        <v>344</v>
+        <v>360</v>
       </c>
       <c r="H7" s="17" t="s">
-        <v>345</v>
+        <v>361</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
-        <v>346</v>
+        <v>362</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>316</v>
+        <v>332</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>347</v>
+        <v>363</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>348</v>
+        <v>364</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>349</v>
+        <v>365</v>
       </c>
       <c r="F8" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G8" s="17" t="s">
-        <v>350</v>
+        <v>366</v>
       </c>
       <c r="H8" s="17" t="s">
-        <v>351</v>
+        <v>367</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="51" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
-        <v>352</v>
+        <v>368</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>316</v>
+        <v>332</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>353</v>
+        <v>369</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>354</v>
+        <v>370</v>
       </c>
       <c r="E9" s="17" t="s">
-        <v>355</v>
+        <v>371</v>
       </c>
       <c r="F9" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G9" s="17" t="s">
-        <v>356</v>
+        <v>372</v>
       </c>
       <c r="H9" s="17" t="s">
-        <v>357</v>
+        <v>373</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="51" x14ac:dyDescent="0.25">
       <c r="A10" s="17" t="s">
-        <v>358</v>
+        <v>374</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>316</v>
+        <v>332</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>359</v>
+        <v>375</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>360</v>
+        <v>376</v>
       </c>
       <c r="E10" s="17" t="s">
-        <v>361</v>
+        <v>377</v>
       </c>
       <c r="F10" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G10" s="17" t="s">
-        <v>362</v>
+        <v>378</v>
       </c>
       <c r="H10" s="17" t="s">
-        <v>363</v>
+        <v>379</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A11" s="17" t="s">
-        <v>364</v>
+        <v>380</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>316</v>
+        <v>332</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>365</v>
+        <v>381</v>
       </c>
       <c r="D11" s="17" t="s">
-        <v>366</v>
+        <v>382</v>
       </c>
       <c r="E11" s="17" t="s">
-        <v>367</v>
+        <v>383</v>
       </c>
       <c r="F11" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G11" s="17" t="s">
-        <v>368</v>
+        <v>384</v>
       </c>
       <c r="H11" s="17" t="s">
-        <v>369</v>
+        <v>385</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
-        <v>370</v>
+        <v>386</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>328</v>
+        <v>344</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>371</v>
+        <v>387</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>372</v>
+        <v>388</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>373</v>
+        <v>389</v>
       </c>
       <c r="F12" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G12" s="17" t="s">
-        <v>374</v>
+        <v>390</v>
       </c>
       <c r="H12" s="17" t="s">
-        <v>375</v>
+        <v>391</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="51" x14ac:dyDescent="0.25">
       <c r="A13" s="17" t="s">
-        <v>376</v>
+        <v>392</v>
       </c>
       <c r="B13" s="17" t="s">
-        <v>328</v>
+        <v>344</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>377</v>
+        <v>393</v>
       </c>
       <c r="D13" s="17" t="s">
-        <v>378</v>
+        <v>394</v>
       </c>
       <c r="E13" s="17" t="s">
-        <v>379</v>
+        <v>395</v>
       </c>
       <c r="F13" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G13" s="17" t="s">
-        <v>380</v>
+        <v>396</v>
       </c>
       <c r="H13" s="17" t="s">
-        <v>381</v>
+        <v>397</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="51" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
-        <v>382</v>
+        <v>398</v>
       </c>
       <c r="B14" s="17" t="s">
-        <v>316</v>
+        <v>332</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>383</v>
+        <v>399</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>384</v>
+        <v>400</v>
       </c>
       <c r="E14" s="17" t="s">
-        <v>385</v>
+        <v>401</v>
       </c>
       <c r="F14" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G14" s="17" t="s">
-        <v>386</v>
+        <v>402</v>
       </c>
       <c r="H14" s="17" t="s">
-        <v>387</v>
+        <v>403</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="102" x14ac:dyDescent="0.25">
       <c r="A15" s="17" t="s">
-        <v>388</v>
+        <v>404</v>
       </c>
       <c r="B15" s="17" t="s">
-        <v>316</v>
+        <v>332</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>389</v>
+        <v>405</v>
       </c>
       <c r="D15" s="17" t="s">
-        <v>390</v>
+        <v>406</v>
       </c>
       <c r="E15" s="17" t="s">
-        <v>391</v>
+        <v>407</v>
       </c>
       <c r="F15" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G15" s="17" t="s">
-        <v>392</v>
+        <v>408</v>
       </c>
       <c r="H15" s="17" t="s">
-        <v>393</v>
+        <v>409</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A16" s="17" t="s">
-        <v>394</v>
+        <v>410</v>
       </c>
       <c r="B16" s="17" t="s">
-        <v>316</v>
+        <v>332</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>395</v>
+        <v>411</v>
       </c>
       <c r="D16" s="17" t="s">
-        <v>396</v>
+        <v>412</v>
       </c>
       <c r="E16" s="17" t="s">
-        <v>397</v>
+        <v>413</v>
       </c>
       <c r="F16" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G16" s="17" t="s">
-        <v>398</v>
+        <v>414</v>
       </c>
       <c r="H16" s="17" t="s">
-        <v>399</v>
+        <v>415</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A17" s="17" t="s">
-        <v>400</v>
+        <v>416</v>
       </c>
       <c r="B17" s="17" t="s">
-        <v>328</v>
+        <v>344</v>
       </c>
       <c r="C17" s="17" t="s">
-        <v>401</v>
+        <v>417</v>
       </c>
       <c r="D17" s="17" t="s">
-        <v>402</v>
+        <v>418</v>
       </c>
       <c r="E17" s="17" t="s">
-        <v>403</v>
+        <v>419</v>
       </c>
       <c r="F17" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G17" s="17" t="s">
-        <v>404</v>
+        <v>420</v>
       </c>
       <c r="H17" s="17" t="s">
-        <v>405</v>
+        <v>421</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A18" s="17" t="s">
-        <v>406</v>
+        <v>422</v>
       </c>
       <c r="B18" s="17" t="s">
-        <v>309</v>
+        <v>325</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>407</v>
+        <v>423</v>
       </c>
       <c r="D18" s="17" t="s">
-        <v>408</v>
+        <v>424</v>
       </c>
       <c r="E18" s="17" t="s">
-        <v>409</v>
+        <v>425</v>
       </c>
       <c r="F18" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G18" s="17" t="s">
-        <v>410</v>
+        <v>426</v>
       </c>
       <c r="H18" s="17" t="s">
-        <v>411</v>
+        <v>427</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="51" x14ac:dyDescent="0.25">
       <c r="A19" s="17" t="s">
-        <v>412</v>
+        <v>428</v>
       </c>
       <c r="B19" s="17" t="s">
-        <v>316</v>
+        <v>332</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>413</v>
+        <v>429</v>
       </c>
       <c r="D19" s="17" t="s">
-        <v>414</v>
+        <v>430</v>
       </c>
       <c r="E19" s="17" t="s">
-        <v>415</v>
+        <v>431</v>
       </c>
       <c r="F19" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G19" s="17" t="s">
-        <v>416</v>
+        <v>432</v>
       </c>
       <c r="H19" s="17" t="s">
-        <v>417</v>
+        <v>433</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="102" x14ac:dyDescent="0.25">
       <c r="A20" s="17" t="s">
-        <v>418</v>
+        <v>434</v>
       </c>
       <c r="B20" s="17" t="s">
-        <v>309</v>
+        <v>325</v>
       </c>
       <c r="C20" s="17" t="s">
-        <v>419</v>
+        <v>435</v>
       </c>
       <c r="D20" s="17" t="s">
-        <v>420</v>
+        <v>436</v>
       </c>
       <c r="E20" s="17" t="s">
-        <v>421</v>
+        <v>437</v>
       </c>
       <c r="F20" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G20" s="17" t="s">
-        <v>422</v>
+        <v>438</v>
       </c>
       <c r="H20" s="17" t="s">
-        <v>423</v>
+        <v>439</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A21" s="17" t="s">
-        <v>424</v>
+        <v>440</v>
       </c>
       <c r="B21" s="17" t="s">
-        <v>316</v>
+        <v>332</v>
       </c>
       <c r="C21" s="17" t="s">
-        <v>425</v>
+        <v>441</v>
       </c>
       <c r="D21" s="17" t="s">
-        <v>426</v>
+        <v>442</v>
       </c>
       <c r="E21" s="17" t="s">
-        <v>427</v>
+        <v>443</v>
       </c>
       <c r="F21" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G21" s="17" t="s">
-        <v>428</v>
+        <v>444</v>
       </c>
       <c r="H21" s="17" t="s">
-        <v>429</v>
+        <v>445</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="51" x14ac:dyDescent="0.25">
+      <c r="A22" s="17" t="s">
+        <v>446</v>
+      </c>
+      <c r="B22" s="17" t="s">
+        <v>344</v>
+      </c>
+      <c r="C22" s="17" t="s">
+        <v>447</v>
+      </c>
+      <c r="D22" s="17" t="s">
+        <v>448</v>
+      </c>
+      <c r="E22" s="17" t="s">
+        <v>449</v>
+      </c>
+      <c r="F22" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="G22" s="17" t="s">
+        <v>450</v>
+      </c>
+      <c r="H22" s="17" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="89.25" x14ac:dyDescent="0.25">
+      <c r="A23" s="17" t="s">
+        <v>452</v>
+      </c>
+      <c r="B23" s="17" t="s">
+        <v>344</v>
+      </c>
+      <c r="C23" s="17" t="s">
+        <v>453</v>
+      </c>
+      <c r="D23" s="17" t="s">
+        <v>454</v>
+      </c>
+      <c r="E23" s="17" t="s">
+        <v>455</v>
+      </c>
+      <c r="F23" s="17" t="s">
+        <v>456</v>
+      </c>
+      <c r="G23" s="17" t="s">
+        <v>457</v>
+      </c>
+      <c r="H23" s="17" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="51" x14ac:dyDescent="0.25">
+      <c r="A24" s="17" t="s">
+        <v>459</v>
+      </c>
+      <c r="B24" s="17" t="s">
+        <v>332</v>
+      </c>
+      <c r="C24" s="17" t="s">
+        <v>460</v>
+      </c>
+      <c r="D24" s="17" t="s">
+        <v>461</v>
+      </c>
+      <c r="E24" s="17" t="s">
+        <v>462</v>
+      </c>
+      <c r="F24" s="17" t="s">
+        <v>456</v>
+      </c>
+      <c r="G24" s="17" t="s">
+        <v>463</v>
+      </c>
+      <c r="H24" s="17" t="s">
+        <v>464</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H21" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
-  <conditionalFormatting sqref="F2:F21">
+  <autoFilter ref="A1:H24" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
+  <conditionalFormatting sqref="F2:F24">
     <cfRule type="expression" dxfId="6" priority="1">
       <formula>$F2="BACKLOG"</formula>
     </cfRule>
@@ -5291,7 +5725,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -5305,643 +5739,643 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>430</v>
+        <v>465</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>431</v>
+        <v>466</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>432</v>
+        <v>467</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>433</v>
+        <v>468</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>434</v>
+        <v>469</v>
       </c>
       <c r="F1" s="16" t="s">
-        <v>435</v>
+        <v>470</v>
       </c>
       <c r="G1" s="16" t="s">
-        <v>436</v>
+        <v>471</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
-        <v>437</v>
+        <v>472</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>438</v>
+        <v>473</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>439</v>
+        <v>474</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>440</v>
+        <v>475</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>441</v>
+        <v>476</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>442</v>
+        <v>477</v>
       </c>
       <c r="G2" s="17" t="s">
-        <v>443</v>
+        <v>478</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
-        <v>444</v>
+        <v>479</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>445</v>
+        <v>480</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>446</v>
+        <v>481</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>440</v>
+        <v>475</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>447</v>
+        <v>482</v>
       </c>
       <c r="F3" s="17" t="s">
-        <v>448</v>
+        <v>483</v>
       </c>
       <c r="G3" s="17" t="s">
-        <v>443</v>
+        <v>478</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>449</v>
+        <v>484</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>450</v>
+        <v>485</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>451</v>
+        <v>486</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>440</v>
+        <v>475</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>452</v>
+        <v>487</v>
       </c>
       <c r="F4" s="17" t="s">
-        <v>453</v>
+        <v>488</v>
       </c>
       <c r="G4" s="17" t="s">
-        <v>443</v>
+        <v>478</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>454</v>
+        <v>489</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>455</v>
+        <v>490</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>456</v>
+        <v>491</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>457</v>
+        <v>492</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>458</v>
+        <v>493</v>
       </c>
       <c r="F5" s="17" t="s">
-        <v>459</v>
+        <v>494</v>
       </c>
       <c r="G5" s="17" t="s">
-        <v>443</v>
+        <v>478</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
-        <v>460</v>
+        <v>495</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>445</v>
+        <v>480</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>461</v>
+        <v>496</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>440</v>
+        <v>475</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>462</v>
+        <v>497</v>
       </c>
       <c r="F6" s="17" t="s">
         <v>131</v>
       </c>
       <c r="G6" s="17" t="s">
-        <v>443</v>
+        <v>478</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
-        <v>463</v>
+        <v>498</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>450</v>
+        <v>485</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>464</v>
+        <v>499</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>440</v>
+        <v>475</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>465</v>
+        <v>500</v>
       </c>
       <c r="F7" s="17" t="s">
         <v>131</v>
       </c>
       <c r="G7" s="17" t="s">
-        <v>443</v>
+        <v>478</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
-        <v>466</v>
+        <v>501</v>
       </c>
       <c r="B8" s="17" t="s">
         <v>121</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>467</v>
+        <v>502</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>468</v>
+        <v>503</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>458</v>
+        <v>493</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>469</v>
+        <v>504</v>
       </c>
       <c r="G8" s="17" t="s">
-        <v>443</v>
+        <v>478</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
-        <v>470</v>
+        <v>505</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>471</v>
+        <v>506</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>472</v>
+        <v>507</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>473</v>
+        <v>508</v>
       </c>
       <c r="E9" s="17" t="s">
-        <v>474</v>
+        <v>509</v>
       </c>
       <c r="F9" s="17" t="s">
-        <v>475</v>
+        <v>510</v>
       </c>
       <c r="G9" s="17" t="s">
-        <v>443</v>
+        <v>478</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="17" t="s">
-        <v>476</v>
+        <v>511</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>445</v>
+        <v>480</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>461</v>
+        <v>496</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>440</v>
+        <v>475</v>
       </c>
       <c r="E10" s="17" t="s">
-        <v>477</v>
+        <v>512</v>
       </c>
       <c r="F10" s="17" t="s">
         <v>139</v>
       </c>
       <c r="G10" s="17" t="s">
-        <v>478</v>
+        <v>513</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A11" s="17" t="s">
-        <v>479</v>
+        <v>514</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>450</v>
+        <v>485</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>480</v>
+        <v>515</v>
       </c>
       <c r="D11" s="17" t="s">
-        <v>481</v>
+        <v>516</v>
       </c>
       <c r="E11" s="17" t="s">
-        <v>482</v>
+        <v>517</v>
       </c>
       <c r="F11" s="17" t="s">
         <v>139</v>
       </c>
       <c r="G11" s="17" t="s">
-        <v>478</v>
+        <v>513</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
-        <v>483</v>
+        <v>518</v>
       </c>
       <c r="B12" s="17" t="s">
         <v>121</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>484</v>
+        <v>519</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>468</v>
+        <v>503</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>485</v>
+        <v>520</v>
       </c>
       <c r="F12" s="17" t="s">
-        <v>469</v>
+        <v>504</v>
       </c>
       <c r="G12" s="17" t="s">
-        <v>478</v>
+        <v>513</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A13" s="17" t="s">
-        <v>486</v>
+        <v>521</v>
       </c>
       <c r="B13" s="17" t="s">
-        <v>471</v>
+        <v>506</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>472</v>
+        <v>507</v>
       </c>
       <c r="D13" s="17" t="s">
-        <v>473</v>
+        <v>508</v>
       </c>
       <c r="E13" s="17" t="s">
-        <v>487</v>
+        <v>522</v>
       </c>
       <c r="F13" s="17" t="s">
-        <v>488</v>
+        <v>523</v>
       </c>
       <c r="G13" s="17" t="s">
-        <v>478</v>
+        <v>513</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="51" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
-        <v>489</v>
+        <v>524</v>
       </c>
       <c r="B14" s="17" t="s">
-        <v>438</v>
+        <v>473</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>490</v>
+        <v>525</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>440</v>
+        <v>475</v>
       </c>
       <c r="E14" s="17" t="s">
-        <v>491</v>
+        <v>526</v>
       </c>
       <c r="F14" s="17" t="s">
-        <v>492</v>
+        <v>527</v>
       </c>
       <c r="G14" s="17" t="s">
-        <v>478</v>
+        <v>513</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A15" s="17" t="s">
-        <v>493</v>
+        <v>528</v>
       </c>
       <c r="B15" s="17" t="s">
-        <v>445</v>
+        <v>480</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>494</v>
+        <v>529</v>
       </c>
       <c r="D15" s="17" t="s">
-        <v>440</v>
+        <v>475</v>
       </c>
       <c r="E15" s="17" t="s">
-        <v>495</v>
+        <v>530</v>
       </c>
       <c r="F15" s="17" t="s">
-        <v>496</v>
+        <v>531</v>
       </c>
       <c r="G15" s="17" t="s">
-        <v>478</v>
+        <v>513</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A16" s="17" t="s">
-        <v>497</v>
+        <v>532</v>
       </c>
       <c r="B16" s="17" t="s">
-        <v>450</v>
+        <v>485</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>498</v>
+        <v>533</v>
       </c>
       <c r="D16" s="17" t="s">
-        <v>440</v>
+        <v>475</v>
       </c>
       <c r="E16" s="17" t="s">
-        <v>499</v>
+        <v>534</v>
       </c>
       <c r="F16" s="17" t="s">
-        <v>500</v>
+        <v>535</v>
       </c>
       <c r="G16" s="17" t="s">
-        <v>478</v>
+        <v>513</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="51" x14ac:dyDescent="0.25">
       <c r="A17" s="17" t="s">
-        <v>501</v>
+        <v>536</v>
       </c>
       <c r="B17" s="17" t="s">
-        <v>502</v>
+        <v>537</v>
       </c>
       <c r="C17" s="17" t="s">
+        <v>538</v>
+      </c>
+      <c r="D17" s="17" t="s">
         <v>503</v>
       </c>
-      <c r="D17" s="17" t="s">
-        <v>468</v>
-      </c>
       <c r="E17" s="17" t="s">
-        <v>504</v>
+        <v>539</v>
       </c>
       <c r="F17" s="17" t="s">
-        <v>505</v>
+        <v>540</v>
       </c>
       <c r="G17" s="17" t="s">
-        <v>478</v>
+        <v>513</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A18" s="17" t="s">
-        <v>506</v>
+        <v>541</v>
       </c>
       <c r="B18" s="17" t="s">
-        <v>445</v>
+        <v>480</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>507</v>
+        <v>542</v>
       </c>
       <c r="D18" s="17" t="s">
-        <v>440</v>
+        <v>475</v>
       </c>
       <c r="E18" s="17" t="s">
-        <v>508</v>
+        <v>543</v>
       </c>
       <c r="F18" s="17" t="s">
-        <v>509</v>
+        <v>544</v>
       </c>
       <c r="G18" s="17" t="s">
-        <v>478</v>
+        <v>513</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="51" x14ac:dyDescent="0.25">
       <c r="A19" s="17" t="s">
-        <v>510</v>
+        <v>545</v>
       </c>
       <c r="B19" s="17" t="s">
-        <v>450</v>
+        <v>485</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>511</v>
+        <v>546</v>
       </c>
       <c r="D19" s="17" t="s">
-        <v>440</v>
+        <v>475</v>
       </c>
       <c r="E19" s="17" t="s">
-        <v>512</v>
+        <v>547</v>
       </c>
       <c r="F19" s="17" t="s">
-        <v>500</v>
+        <v>535</v>
       </c>
       <c r="G19" s="17" t="s">
-        <v>478</v>
+        <v>513</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A20" s="17" t="s">
+        <v>548</v>
+      </c>
+      <c r="B20" s="17" t="s">
+        <v>537</v>
+      </c>
+      <c r="C20" s="17" t="s">
+        <v>549</v>
+      </c>
+      <c r="D20" s="17" t="s">
+        <v>503</v>
+      </c>
+      <c r="E20" s="17" t="s">
+        <v>550</v>
+      </c>
+      <c r="F20" s="17" t="s">
+        <v>551</v>
+      </c>
+      <c r="G20" s="17" t="s">
         <v>513</v>
-      </c>
-      <c r="B20" s="17" t="s">
-        <v>502</v>
-      </c>
-      <c r="C20" s="17" t="s">
-        <v>514</v>
-      </c>
-      <c r="D20" s="17" t="s">
-        <v>468</v>
-      </c>
-      <c r="E20" s="17" t="s">
-        <v>515</v>
-      </c>
-      <c r="F20" s="17" t="s">
-        <v>516</v>
-      </c>
-      <c r="G20" s="17" t="s">
-        <v>478</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A21" s="17" t="s">
-        <v>517</v>
+        <v>552</v>
       </c>
       <c r="B21" s="17" t="s">
-        <v>445</v>
+        <v>480</v>
       </c>
       <c r="C21" s="17" t="s">
-        <v>518</v>
+        <v>553</v>
       </c>
       <c r="D21" s="17" t="s">
-        <v>440</v>
+        <v>475</v>
       </c>
       <c r="E21" s="17" t="s">
-        <v>519</v>
+        <v>554</v>
       </c>
       <c r="F21" s="17" t="s">
-        <v>509</v>
+        <v>544</v>
       </c>
       <c r="G21" s="17" t="s">
-        <v>478</v>
+        <v>513</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A22" s="17" t="s">
-        <v>520</v>
+        <v>555</v>
       </c>
       <c r="B22" s="17" t="s">
-        <v>450</v>
+        <v>485</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>521</v>
+        <v>556</v>
       </c>
       <c r="D22" s="17" t="s">
-        <v>440</v>
+        <v>475</v>
       </c>
       <c r="E22" s="17" t="s">
-        <v>499</v>
+        <v>534</v>
       </c>
       <c r="F22" s="17" t="s">
-        <v>500</v>
+        <v>535</v>
       </c>
       <c r="G22" s="17" t="s">
-        <v>478</v>
+        <v>513</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A23" s="17" t="s">
-        <v>522</v>
+        <v>557</v>
       </c>
       <c r="B23" s="17" t="s">
-        <v>502</v>
+        <v>537</v>
       </c>
       <c r="C23" s="17" t="s">
-        <v>523</v>
+        <v>558</v>
       </c>
       <c r="D23" s="17" t="s">
-        <v>468</v>
+        <v>503</v>
       </c>
       <c r="E23" s="17" t="s">
-        <v>524</v>
+        <v>559</v>
       </c>
       <c r="F23" s="17" t="s">
-        <v>525</v>
+        <v>560</v>
       </c>
       <c r="G23" s="17" t="s">
-        <v>478</v>
+        <v>513</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A24" s="17" t="s">
-        <v>526</v>
+        <v>561</v>
       </c>
       <c r="B24" s="17" t="s">
-        <v>438</v>
+        <v>473</v>
       </c>
       <c r="C24" s="17" t="s">
-        <v>527</v>
+        <v>562</v>
       </c>
       <c r="D24" s="17" t="s">
-        <v>440</v>
+        <v>475</v>
       </c>
       <c r="E24" s="17" t="s">
-        <v>528</v>
+        <v>563</v>
       </c>
       <c r="F24" s="17" t="s">
-        <v>529</v>
+        <v>564</v>
       </c>
       <c r="G24" s="17" t="s">
-        <v>478</v>
+        <v>513</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="17" t="s">
-        <v>530</v>
+        <v>565</v>
       </c>
       <c r="B25" s="17" t="s">
-        <v>445</v>
+        <v>480</v>
       </c>
       <c r="C25" s="17" t="s">
-        <v>531</v>
+        <v>566</v>
       </c>
       <c r="D25" s="17" t="s">
-        <v>440</v>
+        <v>475</v>
       </c>
       <c r="E25" s="17" t="s">
-        <v>532</v>
+        <v>567</v>
       </c>
       <c r="F25" s="17" t="s">
-        <v>509</v>
+        <v>544</v>
       </c>
       <c r="G25" s="17" t="s">
-        <v>478</v>
+        <v>513</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A26" s="17" t="s">
-        <v>533</v>
+        <v>568</v>
       </c>
       <c r="B26" s="17" t="s">
-        <v>450</v>
+        <v>485</v>
       </c>
       <c r="C26" s="17" t="s">
-        <v>534</v>
+        <v>569</v>
       </c>
       <c r="D26" s="17" t="s">
-        <v>440</v>
+        <v>475</v>
       </c>
       <c r="E26" s="17" t="s">
+        <v>570</v>
+      </c>
+      <c r="F26" s="17" t="s">
         <v>535</v>
       </c>
-      <c r="F26" s="17" t="s">
-        <v>500</v>
-      </c>
       <c r="G26" s="17" t="s">
-        <v>478</v>
+        <v>513</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A27" s="17" t="s">
-        <v>536</v>
+        <v>571</v>
       </c>
       <c r="B27" s="17" t="s">
-        <v>502</v>
+        <v>537</v>
       </c>
       <c r="C27" s="17" t="s">
-        <v>537</v>
+        <v>572</v>
       </c>
       <c r="D27" s="17" t="s">
-        <v>468</v>
+        <v>503</v>
       </c>
       <c r="E27" s="17" t="s">
-        <v>538</v>
+        <v>573</v>
       </c>
       <c r="F27" s="17" t="s">
-        <v>539</v>
+        <v>574</v>
       </c>
       <c r="G27" s="17" t="s">
-        <v>478</v>
+        <v>513</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A28" s="17" t="s">
-        <v>540</v>
+        <v>575</v>
       </c>
       <c r="B28" s="17" t="s">
-        <v>450</v>
+        <v>485</v>
       </c>
       <c r="C28" s="17" t="s">
-        <v>541</v>
+        <v>576</v>
       </c>
       <c r="D28" s="17" t="s">
-        <v>542</v>
+        <v>577</v>
       </c>
       <c r="E28" s="17" t="s">
-        <v>543</v>
+        <v>578</v>
       </c>
       <c r="F28" s="17" t="s">
-        <v>544</v>
+        <v>579</v>
       </c>
       <c r="G28" s="17" t="s">
         <v>86</v>
@@ -5949,45 +6383,45 @@
     </row>
     <row r="29" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A29" s="17" t="s">
-        <v>545</v>
+        <v>580</v>
       </c>
       <c r="B29" s="17" t="s">
-        <v>450</v>
+        <v>485</v>
       </c>
       <c r="C29" s="17" t="s">
-        <v>546</v>
+        <v>581</v>
       </c>
       <c r="D29" s="17" t="s">
-        <v>468</v>
+        <v>503</v>
       </c>
       <c r="E29" s="17" t="s">
-        <v>547</v>
+        <v>582</v>
       </c>
       <c r="F29" s="17" t="s">
-        <v>500</v>
+        <v>535</v>
       </c>
       <c r="G29" s="17" t="s">
-        <v>478</v>
+        <v>513</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A30" s="17" t="s">
-        <v>548</v>
+        <v>583</v>
       </c>
       <c r="B30" s="17" t="s">
-        <v>549</v>
+        <v>584</v>
       </c>
       <c r="C30" s="17" t="s">
-        <v>550</v>
+        <v>585</v>
       </c>
       <c r="D30" s="17" t="s">
-        <v>440</v>
+        <v>475</v>
       </c>
       <c r="E30" s="17" t="s">
-        <v>551</v>
+        <v>586</v>
       </c>
       <c r="F30" s="17" t="s">
-        <v>509</v>
+        <v>544</v>
       </c>
       <c r="G30" s="17" t="s">
         <v>86</v>
@@ -5995,59 +6429,174 @@
     </row>
     <row r="31" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A31" s="17" t="s">
-        <v>552</v>
+        <v>587</v>
       </c>
       <c r="B31" s="17" t="s">
-        <v>438</v>
+        <v>473</v>
       </c>
       <c r="C31" s="17" t="s">
-        <v>553</v>
+        <v>588</v>
       </c>
       <c r="D31" s="17" t="s">
-        <v>554</v>
+        <v>589</v>
       </c>
       <c r="E31" s="17" t="s">
-        <v>555</v>
+        <v>590</v>
       </c>
       <c r="F31" s="17" t="s">
-        <v>556</v>
+        <v>591</v>
       </c>
       <c r="G31" s="17" t="s">
-        <v>478</v>
+        <v>513</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A32" s="17" t="s">
-        <v>557</v>
+        <v>592</v>
       </c>
       <c r="B32" s="17" t="s">
-        <v>502</v>
+        <v>537</v>
       </c>
       <c r="C32" s="17" t="s">
-        <v>558</v>
+        <v>593</v>
       </c>
       <c r="D32" s="17" t="s">
-        <v>559</v>
+        <v>594</v>
       </c>
       <c r="E32" s="17" t="s">
-        <v>560</v>
+        <v>595</v>
       </c>
       <c r="F32" s="17" t="s">
-        <v>561</v>
+        <v>596</v>
       </c>
       <c r="G32" s="17" t="s">
         <v>86</v>
       </c>
     </row>
+    <row r="33" spans="1:7" ht="51" x14ac:dyDescent="0.25">
+      <c r="A33" s="17" t="s">
+        <v>597</v>
+      </c>
+      <c r="B33" s="17" t="s">
+        <v>598</v>
+      </c>
+      <c r="C33" s="17" t="s">
+        <v>599</v>
+      </c>
+      <c r="D33" s="17" t="s">
+        <v>600</v>
+      </c>
+      <c r="E33" s="17" t="s">
+        <v>493</v>
+      </c>
+      <c r="F33" s="17" t="s">
+        <v>601</v>
+      </c>
+      <c r="G33" s="17" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A34" s="17" t="s">
+        <v>602</v>
+      </c>
+      <c r="B34" s="17" t="s">
+        <v>473</v>
+      </c>
+      <c r="C34" s="17" t="s">
+        <v>603</v>
+      </c>
+      <c r="D34" s="17" t="s">
+        <v>475</v>
+      </c>
+      <c r="E34" s="17" t="s">
+        <v>604</v>
+      </c>
+      <c r="F34" s="17" t="s">
+        <v>605</v>
+      </c>
+      <c r="G34" s="17" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A35" s="17" t="s">
+        <v>606</v>
+      </c>
+      <c r="B35" s="17" t="s">
+        <v>473</v>
+      </c>
+      <c r="C35" s="17" t="s">
+        <v>607</v>
+      </c>
+      <c r="D35" s="17" t="s">
+        <v>475</v>
+      </c>
+      <c r="E35" s="17" t="s">
+        <v>608</v>
+      </c>
+      <c r="F35" s="17" t="s">
+        <v>609</v>
+      </c>
+      <c r="G35" s="17" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A36" s="17" t="s">
+        <v>610</v>
+      </c>
+      <c r="B36" s="17" t="s">
+        <v>485</v>
+      </c>
+      <c r="C36" s="17" t="s">
+        <v>611</v>
+      </c>
+      <c r="D36" s="17" t="s">
+        <v>503</v>
+      </c>
+      <c r="E36" s="17" t="s">
+        <v>612</v>
+      </c>
+      <c r="F36" s="17" t="s">
+        <v>613</v>
+      </c>
+      <c r="G36" s="17" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" ht="51" x14ac:dyDescent="0.25">
+      <c r="A37" s="17" t="s">
+        <v>614</v>
+      </c>
+      <c r="B37" s="17" t="s">
+        <v>615</v>
+      </c>
+      <c r="C37" s="17" t="s">
+        <v>616</v>
+      </c>
+      <c r="D37" s="17" t="s">
+        <v>617</v>
+      </c>
+      <c r="E37" s="17" t="s">
+        <v>618</v>
+      </c>
+      <c r="F37" s="17" t="s">
+        <v>619</v>
+      </c>
+      <c r="G37" s="17" t="s">
+        <v>86</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G32" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
+  <autoFilter ref="A1:G37" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -6059,39 +6608,39 @@
   <sheetData>
     <row r="1" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>562</v>
+        <v>620</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>563</v>
+        <v>621</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>564</v>
+        <v>622</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>436</v>
+        <v>471</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>565</v>
+        <v>623</v>
       </c>
       <c r="F1" s="16" t="s">
-        <v>566</v>
+        <v>624</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
-        <v>567</v>
+        <v>625</v>
       </c>
       <c r="B2" s="17" t="s">
         <v>72</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>568</v>
+        <v>626</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>443</v>
+        <v>478</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>569</v>
+        <v>627</v>
       </c>
       <c r="F2" s="17" t="s">
         <v>88</v>
@@ -6099,19 +6648,19 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
-        <v>570</v>
+        <v>628</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>571</v>
+        <v>629</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>572</v>
+        <v>630</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>443</v>
+        <v>478</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>573</v>
+        <v>631</v>
       </c>
       <c r="F3" s="17" t="s">
         <v>88</v>
@@ -6119,39 +6668,39 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>574</v>
+        <v>632</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>575</v>
+        <v>633</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>576</v>
+        <v>634</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>443</v>
+        <v>478</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>577</v>
+        <v>635</v>
       </c>
       <c r="F4" s="17" t="s">
-        <v>578</v>
+        <v>636</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>579</v>
+        <v>637</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>580</v>
+        <v>638</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>581</v>
+        <v>639</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>443</v>
+        <v>478</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>582</v>
+        <v>640</v>
       </c>
       <c r="F5" s="17" t="s">
         <v>166</v>
@@ -6159,16 +6708,16 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
-        <v>583</v>
+        <v>641</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>584</v>
+        <v>642</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>585</v>
+        <v>643</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>443</v>
+        <v>478</v>
       </c>
       <c r="E6" s="17" t="s">
         <v>26</v>
@@ -6179,19 +6728,19 @@
     </row>
     <row r="7" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
-        <v>586</v>
+        <v>644</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>587</v>
+        <v>645</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>588</v>
+        <v>646</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>443</v>
+        <v>478</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>589</v>
+        <v>647</v>
       </c>
       <c r="F7" s="17" t="s">
         <v>166</v>
@@ -6199,22 +6748,22 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
-        <v>590</v>
+        <v>648</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>591</v>
+        <v>649</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>592</v>
+        <v>650</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>443</v>
+        <v>478</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>593</v>
+        <v>651</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>594</v>
+        <v>652</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -6222,16 +6771,16 @@
         <v>178</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>595</v>
+        <v>653</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>596</v>
+        <v>654</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>443</v>
+        <v>478</v>
       </c>
       <c r="E9" s="17" t="s">
-        <v>593</v>
+        <v>651</v>
       </c>
       <c r="F9" s="17" t="s">
         <v>173</v>
@@ -6239,16 +6788,16 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="17" t="s">
-        <v>597</v>
+        <v>655</v>
       </c>
       <c r="B10" s="17" t="s">
         <v>52</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>598</v>
+        <v>656</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>443</v>
+        <v>478</v>
       </c>
       <c r="E10" s="17" t="s">
         <v>51</v>
@@ -6259,39 +6808,39 @@
     </row>
     <row r="11" spans="1:6" ht="51" x14ac:dyDescent="0.25">
       <c r="A11" s="17" t="s">
-        <v>599</v>
+        <v>657</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>600</v>
+        <v>658</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>601</v>
+        <v>659</v>
       </c>
       <c r="D11" s="17" t="s">
-        <v>478</v>
+        <v>513</v>
       </c>
       <c r="E11" s="17" t="s">
-        <v>602</v>
+        <v>660</v>
       </c>
       <c r="F11" s="17" t="s">
-        <v>603</v>
+        <v>661</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
-        <v>604</v>
+        <v>662</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>605</v>
+        <v>663</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>606</v>
+        <v>664</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>443</v>
+        <v>478</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>607</v>
+        <v>665</v>
       </c>
       <c r="F12" s="17" t="s">
         <v>101</v>
@@ -6299,46 +6848,66 @@
     </row>
     <row r="13" spans="1:6" ht="51" x14ac:dyDescent="0.25">
       <c r="A13" s="17" t="s">
-        <v>608</v>
+        <v>666</v>
       </c>
       <c r="B13" s="17" t="s">
-        <v>609</v>
+        <v>667</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>610</v>
+        <v>668</v>
       </c>
       <c r="D13" s="17" t="s">
-        <v>478</v>
+        <v>513</v>
       </c>
       <c r="E13" s="17" t="s">
-        <v>611</v>
+        <v>669</v>
       </c>
       <c r="F13" s="17" t="s">
-        <v>612</v>
+        <v>670</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="51" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B14" s="17" t="s">
-        <v>613</v>
+        <v>671</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>614</v>
+        <v>672</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>478</v>
+        <v>513</v>
       </c>
       <c r="E14" s="17" t="s">
-        <v>615</v>
+        <v>673</v>
       </c>
       <c r="F14" s="17" t="s">
-        <v>616</v>
+        <v>674</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="51" x14ac:dyDescent="0.25">
+      <c r="A15" s="17" t="s">
+        <v>675</v>
+      </c>
+      <c r="B15" s="17" t="s">
+        <v>676</v>
+      </c>
+      <c r="C15" s="17" t="s">
+        <v>677</v>
+      </c>
+      <c r="D15" s="17" t="s">
+        <v>86</v>
+      </c>
+      <c r="E15" s="17" t="s">
+        <v>60</v>
+      </c>
+      <c r="F15" s="17" t="s">
+        <v>678</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F14" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
+  <autoFilter ref="A1:F15" xr:uid="{00000000-0009-0000-0000-000005000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6357,121 +6926,121 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>617</v>
+        <v>679</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>618</v>
+        <v>680</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>619</v>
+        <v>681</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>620</v>
+        <v>682</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>621</v>
+        <v>683</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
-        <v>622</v>
+        <v>684</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>623</v>
+        <v>685</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>624</v>
+        <v>686</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>625</v>
+        <v>687</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>626</v>
+        <v>688</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
-        <v>627</v>
+        <v>689</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>628</v>
+        <v>690</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>629</v>
+        <v>691</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>630</v>
+        <v>692</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>631</v>
+        <v>693</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>632</v>
+        <v>694</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>633</v>
+        <v>695</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>633</v>
+        <v>695</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>634</v>
+        <v>696</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>635</v>
+        <v>697</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>636</v>
+        <v>698</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>637</v>
+        <v>699</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>638</v>
+        <v>700</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>639</v>
+        <v>701</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>631</v>
+        <v>693</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
-        <v>640</v>
+        <v>702</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>641</v>
+        <v>703</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>641</v>
+        <v>703</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>642</v>
+        <v>704</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>626</v>
+        <v>688</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
-        <v>643</v>
+        <v>705</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>644</v>
+        <v>706</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>645</v>
+        <v>707</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>646</v>
+        <v>708</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>626</v>
+        <v>688</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Checkpoint: D-012 S6 PASS, S7 switched and verified technically (user test pending); tracker updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/SMARTDOC_2_0_MASTER_TRACKER.xlsx
+++ b/docs/SMARTDOC_2_0_MASTER_TRACKER.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\speed\Desktop\Claude - ПРОЕКТ\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79E22CCE-591B-49A0-BBB5-9EE59E662F39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E99D4B0B-1904-4C89-AEBB-86EB69694DFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,12 +22,12 @@
     <sheet name="Release Readiness" sheetId="7" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Bugs!$A$1:$H$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Bugs!$A$1:$H$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Decisions!$A$1:$F$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Release Readiness'!$A$1:$E$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Roadmap!$A$1:$F$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Tasks!$A$1:$P$38</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Tests!$A$1:$G$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Tests!$A$1:$G$39</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1219" uniqueCount="709">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1250" uniqueCount="732">
   <si>
     <t>SmartDoc 2.0 -- master tracker</t>
   </si>
@@ -226,7 +226,7 @@
     <t>P2-P7</t>
   </si>
   <si>
-    <t>An approvable release candidate</t>
+    <t>2.0 Preview on its own Supabase project and Storage (D-012 S7 verified technically; user test pending)</t>
   </si>
   <si>
     <t>P9</t>
@@ -841,13 +841,16 @@
     <t>Owner + Claude</t>
   </si>
   <si>
-    <t>f48e84a</t>
-  </si>
-  <si>
-    <t>Isolated GitHub Actions workflow on a throwaway PostgreSQL (no secrets, read-only token): https://github.com/Drajeto07/claude/actions/runs/38701081333 -- empty database, migrations up / check / down / up, isolation tests 49 passed (owner's negative cases incl. wrong/missing bucket through the real S3 code, missing configuration, production resources, no start-up writes or worker while unproven, wrong database id and second marker row on PostgreSQL), every PostgreSQL-marked test 14 passed.</t>
-  </si>
-  <si>
-    <t>S1 project smartdoc-preview (ksmwhnnupkrtzrupcitc, free, $0 checked); S4 schema on the new empty project only (head d41f7a60c9e2, 16 tables, RLS on all, same as production -- production only read); S5 database marker written, private bucket created, bucket marker file docs/d012-preview/identity.json waits for the owner's upload; S2 (password) and S3 key pair: owner, in Supabase. NOT done (owner): S6 Vercel variables, S7 switching redeploy, S8 Free Design writes, S9 old test accounts.</t>
+    <t>3489a6a (S7) + diagnostics</t>
+  </si>
+  <si>
+    <t>dpl_3262fjM25cveZESWDNfkoBZF6csr READY; https://smartdoc-git-feature-smartdoc-20-drajeto.vercel.app</t>
+  </si>
+  <si>
+    <t>S6 PASS (Vercel API: 12/12 branch rows Preview + feature/smartdoc-2.0, 3 Sensitive, 20 existing rows unchanged, nothing inheritable). S7: CI green (run 38718605753: isolation 75, PostgreSQL 14). First health: refused (pooler: password authentication failed -- wrong password in the branch DATABASE_URL; guard refused correctly). After the owner's fix, health verified; independent proof in the new project's logs: 10:38:17 Supavisor 'Connection authenticated', marker read once by postgres (pg_stat_statements), Storage GET 200 _smartdoc/identity.json by Boto3/1.43.101; production: no connections or storage access after 10:12:17, data unchanged (2 users / 11 documents / 4 files).</t>
+  </si>
+  <si>
+    <t>D-012 NOT yet VERIFIED: waits for the owner's user test (synthetic account, DOCX with a picture, edit, reload, DOCX/PDF export) and the read-only check that the records exist only in smartdoc-preview. S8/S9 not done.</t>
   </si>
   <si>
     <t>S2-023</t>
@@ -1444,6 +1447,42 @@
     <t>scratchpad investigation; docs analysis section 13</t>
   </si>
   <si>
+    <t>B-024</t>
+  </si>
+  <si>
+    <t>A preview's settings refused at start</t>
+  </si>
+  <si>
+    <t>No secret in logs</t>
+  </si>
+  <si>
+    <t>pydantic copied the settings (DATABASE_URL with its password) into the error text</t>
+  </si>
+  <si>
+    <t>hide_input_in_errors=True (ea50bd6)</t>
+  </si>
+  <si>
+    <t>tests/test_preview_isolation.py leak tests; CI run 38713707649</t>
+  </si>
+  <si>
+    <t>B-025</t>
+  </si>
+  <si>
+    <t>S7 health showed 'the identity marker can't be read'</t>
+  </si>
+  <si>
+    <t>The reason, safely</t>
+  </si>
+  <si>
+    <t>A sign-in failure was reported like a missing marker</t>
+  </si>
+  <si>
+    <t>Refusal codes from SQLSTATE / S3 codes / exception class names only; health status not_serving until proven</t>
+  </si>
+  <si>
+    <t>tests/test_preview_isolation.py 89; backend 2806 passed</t>
+  </si>
+  <si>
     <t>Test ID</t>
   </si>
   <si>
@@ -1909,6 +1948,36 @@
     <t>docs/SMARTDOC_DOCUMENT_DOCTOR_SAFEEDIT_ANALYSIS.md section 13</t>
   </si>
   <si>
+    <t>T-037</t>
+  </si>
+  <si>
+    <t>Release</t>
+  </si>
+  <si>
+    <t>D-012 S6 check (Vercel API names/scope/type/timestamps, no values)</t>
+  </si>
+  <si>
+    <t>Vercel project smartdoc</t>
+  </si>
+  <si>
+    <t>scratchpad/s6_check.py</t>
+  </si>
+  <si>
+    <t>T-038</t>
+  </si>
+  <si>
+    <t>D-012 S7: switch + independent proof (Supabase logs, statement statistics, storage logs; production unchanged)</t>
+  </si>
+  <si>
+    <t>Vercel Preview dpl_3262fjM25cveZESWDNfkoBZF6csr</t>
+  </si>
+  <si>
+    <t>PASS technically; user test pending</t>
+  </si>
+  <si>
+    <t>docs/d012-preview/S6_PROCEDURE.md; this tracker row S2-050</t>
+  </si>
+  <si>
     <t>Decision ID</t>
   </si>
   <si>
@@ -2053,7 +2122,7 @@
     <t>Canvas documents and the shared database</t>
   </si>
   <si>
-    <t>Option (a). Rev 2 approved in part (2026-10-15): S1-S5 done (separate free project, schema, markers, private bucket; production only read); S6-S9 refused for now (no Vercel variables, no switching redeploy, no Free Design writes, old test accounts untouched).</t>
+    <t>Option (a). S1-S6 done; S7 switched (2026-10-15) and technically verified; VERIFIED only after the owner's user test. S8 (Free Design writes) and S9 (old test accounts) not approved.</t>
   </si>
   <si>
     <t>S2-050, P5 persistence</t>
@@ -2808,7 +2877,7 @@
       </c>
       <c r="C5" s="5">
         <f>COUNTIF(Roadmap!$D$2:$D$11,A5)</f>
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -2830,11 +2899,11 @@
       </c>
       <c r="B7" s="5">
         <f>COUNTIF(Tasks!$G$2:$G$38,A7)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C7" s="5">
         <f>COUNTIF(Roadmap!$D$2:$D$11,A7)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -2856,7 +2925,7 @@
       </c>
       <c r="B9" s="5">
         <f>COUNTIF(Tasks!$G$2:$G$38,A9)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C9" s="5">
         <f>COUNTIF(Roadmap!$D$2:$D$11,A9)</f>
@@ -2925,7 +2994,7 @@
         <v>15</v>
       </c>
       <c r="B15">
-        <f>COUNTA(Bugs!$A$2:$A$24)-COUNTIF(Bugs!$F$2:$F$24,"DONE")-COUNTIF(Bugs!$F$2:$F$24,"VERIFIED")</f>
+        <f>COUNTA(Bugs!$A$2:$A$26)-COUNTIF(Bugs!$F$2:$F$26,"DONE")-COUNTIF(Bugs!$F$2:$F$26,"VERIFIED")</f>
         <v>4</v>
       </c>
     </row>
@@ -3140,7 +3209,7 @@
         <v>57</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E10" s="17" t="s">
         <v>58</v>
@@ -4538,7 +4607,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="28" spans="1:16" ht="280.5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:16" ht="382.5" x14ac:dyDescent="0.25">
       <c r="A28" s="17" t="s">
         <v>258</v>
       </c>
@@ -4558,7 +4627,7 @@
         <v>22</v>
       </c>
       <c r="G28" s="17" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H28" s="17"/>
       <c r="I28" s="17" t="s">
@@ -4573,20 +4642,22 @@
       <c r="L28" s="17" t="s">
         <v>264</v>
       </c>
-      <c r="M28" s="17"/>
+      <c r="M28" s="17" t="s">
+        <v>265</v>
+      </c>
       <c r="N28" s="17" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="O28" s="17" t="s">
         <v>86</v>
       </c>
       <c r="P28" s="17" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
     <row r="29" spans="1:16" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A29" s="17" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B29" s="17" t="s">
         <v>34</v>
@@ -4595,10 +4666,10 @@
         <v>121</v>
       </c>
       <c r="D29" s="17" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="E29" s="17" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="F29" s="17" t="s">
         <v>30</v>
@@ -4610,7 +4681,7 @@
         <v>251</v>
       </c>
       <c r="I29" s="17" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="J29" s="17" t="s">
         <v>83</v>
@@ -4625,12 +4696,12 @@
         <v>86</v>
       </c>
       <c r="P29" s="17" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="30" spans="1:16" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A30" s="17" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B30" s="17" t="s">
         <v>34</v>
@@ -4639,10 +4710,10 @@
         <v>121</v>
       </c>
       <c r="D30" s="17" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="E30" s="17" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F30" s="17" t="s">
         <v>30</v>
@@ -4654,7 +4725,7 @@
         <v>149</v>
       </c>
       <c r="I30" s="17" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="J30" s="17" t="s">
         <v>83</v>
@@ -4669,12 +4740,12 @@
         <v>86</v>
       </c>
       <c r="P30" s="17" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="31" spans="1:16" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A31" s="17" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B31" s="17" t="s">
         <v>30</v>
@@ -4683,10 +4754,10 @@
         <v>121</v>
       </c>
       <c r="D31" s="17" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="E31" s="17" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="F31" s="17" t="s">
         <v>30</v>
@@ -4698,7 +4769,7 @@
         <v>200</v>
       </c>
       <c r="I31" s="17" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="J31" s="17" t="s">
         <v>83</v>
@@ -4713,12 +4784,12 @@
         <v>86</v>
       </c>
       <c r="P31" s="17" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="32" spans="1:16" ht="255" x14ac:dyDescent="0.25">
       <c r="A32" s="17" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B32" s="17" t="s">
         <v>38</v>
@@ -4727,10 +4798,10 @@
         <v>158</v>
       </c>
       <c r="D32" s="17" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E32" s="17" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="F32" s="17" t="s">
         <v>26</v>
@@ -4742,7 +4813,7 @@
         <v>157</v>
       </c>
       <c r="I32" s="17" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="J32" s="17" t="s">
         <v>83</v>
@@ -4751,36 +4822,36 @@
         <v>84</v>
       </c>
       <c r="L32" s="17" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="M32" s="17" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="N32" s="17" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="O32" s="17" t="s">
         <v>86</v>
       </c>
       <c r="P32" s="17" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
     </row>
     <row r="33" spans="1:16" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A33" s="17" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B33" s="17" t="s">
         <v>60</v>
       </c>
       <c r="C33" s="17" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D33" s="17" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="E33" s="17" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="F33" s="17" t="s">
         <v>30</v>
@@ -4789,10 +4860,10 @@
         <v>11</v>
       </c>
       <c r="H33" s="17" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="I33" s="17" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="J33" s="17" t="s">
         <v>83</v>
@@ -4801,34 +4872,34 @@
         <v>84</v>
       </c>
       <c r="L33" s="17" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="M33" s="17"/>
       <c r="N33" s="17" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="O33" s="17" t="s">
         <v>86</v>
       </c>
       <c r="P33" s="17" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
     <row r="34" spans="1:16" ht="280.5" x14ac:dyDescent="0.25">
       <c r="A34" s="17" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B34" s="17" t="s">
         <v>60</v>
       </c>
       <c r="C34" s="17" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D34" s="17" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="E34" s="17" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="F34" s="17" t="s">
         <v>30</v>
@@ -4837,10 +4908,10 @@
         <v>9</v>
       </c>
       <c r="H34" s="17" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="I34" s="17" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="J34" s="17" t="s">
         <v>83</v>
@@ -4849,22 +4920,22 @@
         <v>84</v>
       </c>
       <c r="L34" s="17" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="M34" s="17"/>
       <c r="N34" s="17" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="O34" s="17" t="s">
         <v>86</v>
       </c>
       <c r="P34" s="17" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
     </row>
     <row r="35" spans="1:16" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A35" s="17" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B35" s="17" t="s">
         <v>38</v>
@@ -4873,10 +4944,10 @@
         <v>121</v>
       </c>
       <c r="D35" s="17" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E35" s="17" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="F35" s="17" t="s">
         <v>30</v>
@@ -4885,7 +4956,7 @@
         <v>5</v>
       </c>
       <c r="H35" s="17" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="I35" s="17"/>
       <c r="J35" s="17" t="s">
@@ -4901,12 +4972,12 @@
         <v>86</v>
       </c>
       <c r="P35" s="17" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
     </row>
     <row r="36" spans="1:16" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A36" s="17" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B36" s="17" t="s">
         <v>38</v>
@@ -4915,10 +4986,10 @@
         <v>121</v>
       </c>
       <c r="D36" s="17" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E36" s="17" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="F36" s="17" t="s">
         <v>30</v>
@@ -4927,7 +4998,7 @@
         <v>5</v>
       </c>
       <c r="H36" s="17" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="I36" s="17"/>
       <c r="J36" s="17" t="s">
@@ -4943,12 +5014,12 @@
         <v>86</v>
       </c>
       <c r="P36" s="17" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
     </row>
     <row r="37" spans="1:16" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A37" s="17" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B37" s="17" t="s">
         <v>38</v>
@@ -4957,10 +5028,10 @@
         <v>186</v>
       </c>
       <c r="D37" s="17" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E37" s="17" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="F37" s="17" t="s">
         <v>30</v>
@@ -4969,7 +5040,7 @@
         <v>5</v>
       </c>
       <c r="H37" s="17" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="I37" s="17"/>
       <c r="J37" s="17" t="s">
@@ -4985,24 +5056,24 @@
         <v>86</v>
       </c>
       <c r="P37" s="17" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
     </row>
     <row r="38" spans="1:16" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A38" s="17" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B38" s="17" t="s">
         <v>60</v>
       </c>
       <c r="C38" s="17" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="D38" s="17" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E38" s="17" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="F38" s="17" t="s">
         <v>30</v>
@@ -5011,7 +5082,7 @@
         <v>5</v>
       </c>
       <c r="H38" s="17" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="I38" s="17"/>
       <c r="J38" s="17" t="s">
@@ -5059,7 +5130,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -5074,629 +5145,681 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="F1" s="16" t="s">
         <v>2</v>
       </c>
       <c r="G1" s="16" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="H1" s="16" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="F2" s="17" t="s">
         <v>8</v>
       </c>
       <c r="G2" s="17" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="H2" s="17" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="F3" s="17" t="s">
         <v>5</v>
       </c>
       <c r="G3" s="17"/>
       <c r="H3" s="17" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="F4" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G4" s="17" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="H4" s="17" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="F5" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G5" s="17" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="H5" s="17" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="51" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="F6" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G6" s="17" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="H6" s="17" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="F7" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G7" s="17" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="H7" s="17" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="F8" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G8" s="17" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="H8" s="17" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="51" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="E9" s="17" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="F9" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G9" s="17" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="H9" s="17" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="51" x14ac:dyDescent="0.25">
       <c r="A10" s="17" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="E10" s="17" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="F10" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G10" s="17" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="H10" s="17" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A11" s="17" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="D11" s="17" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="E11" s="17" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="F11" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G11" s="17" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="H11" s="17" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="63.75" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="F12" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G12" s="17" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="H12" s="17" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="51" x14ac:dyDescent="0.25">
       <c r="A13" s="17" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="B13" s="17" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="D13" s="17" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="E13" s="17" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="F13" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G13" s="17" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="H13" s="17" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="51" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="B14" s="17" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="E14" s="17" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="F14" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G14" s="17" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="H14" s="17" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="102" x14ac:dyDescent="0.25">
       <c r="A15" s="17" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="B15" s="17" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="D15" s="17" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="E15" s="17" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="F15" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G15" s="17" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="H15" s="17" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A16" s="17" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="B16" s="17" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="D16" s="17" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="E16" s="17" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="F16" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G16" s="17" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="H16" s="17" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A17" s="17" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="B17" s="17" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C17" s="17" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="D17" s="17" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="E17" s="17" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="F17" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G17" s="17" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="H17" s="17" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A18" s="17" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="B18" s="17" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="D18" s="17" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="E18" s="17" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="F18" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G18" s="17" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="H18" s="17" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
     </row>
     <row r="19" spans="1:8" ht="51" x14ac:dyDescent="0.25">
       <c r="A19" s="17" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="B19" s="17" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="D19" s="17" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E19" s="17" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="F19" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G19" s="17" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="H19" s="17" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="102" x14ac:dyDescent="0.25">
       <c r="A20" s="17" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="B20" s="17" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="C20" s="17" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="D20" s="17" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="E20" s="17" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="F20" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G20" s="17" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="H20" s="17" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="76.5" x14ac:dyDescent="0.25">
       <c r="A21" s="17" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="B21" s="17" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C21" s="17" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="D21" s="17" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="E21" s="17" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="F21" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G21" s="17" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="H21" s="17" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="51" x14ac:dyDescent="0.25">
       <c r="A22" s="17" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="B22" s="17" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="D22" s="17" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="E22" s="17" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="F22" s="17" t="s">
         <v>10</v>
       </c>
       <c r="G22" s="17" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="H22" s="17" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
     </row>
     <row r="23" spans="1:8" ht="89.25" x14ac:dyDescent="0.25">
       <c r="A23" s="17" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="B23" s="17" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C23" s="17" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="D23" s="17" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="E23" s="17" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="F23" s="17" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="G23" s="17" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="H23" s="17" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="51" x14ac:dyDescent="0.25">
       <c r="A24" s="17" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="B24" s="17" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="C24" s="17" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="D24" s="17" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="E24" s="17" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="F24" s="17" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="G24" s="17" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="H24" s="17" t="s">
-        <v>464</v>
+        <v>465</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A25" s="17" t="s">
+        <v>466</v>
+      </c>
+      <c r="B25" s="17" t="s">
+        <v>326</v>
+      </c>
+      <c r="C25" s="17" t="s">
+        <v>467</v>
+      </c>
+      <c r="D25" s="17" t="s">
+        <v>468</v>
+      </c>
+      <c r="E25" s="17" t="s">
+        <v>469</v>
+      </c>
+      <c r="F25" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="G25" s="17" t="s">
+        <v>470</v>
+      </c>
+      <c r="H25" s="17" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="89.25" x14ac:dyDescent="0.25">
+      <c r="A26" s="17" t="s">
+        <v>472</v>
+      </c>
+      <c r="B26" s="17" t="s">
+        <v>345</v>
+      </c>
+      <c r="C26" s="17" t="s">
+        <v>473</v>
+      </c>
+      <c r="D26" s="17" t="s">
+        <v>474</v>
+      </c>
+      <c r="E26" s="17" t="s">
+        <v>475</v>
+      </c>
+      <c r="F26" s="17" t="s">
+        <v>10</v>
+      </c>
+      <c r="G26" s="17" t="s">
+        <v>476</v>
+      </c>
+      <c r="H26" s="17" t="s">
+        <v>477</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H24" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
-  <conditionalFormatting sqref="F2:F24">
+  <autoFilter ref="A1:H26" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
+  <conditionalFormatting sqref="F2:F26">
     <cfRule type="expression" dxfId="6" priority="1">
       <formula>$F2="BACKLOG"</formula>
     </cfRule>
@@ -5725,7 +5848,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -5739,643 +5862,643 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>465</v>
+        <v>478</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>466</v>
+        <v>479</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>467</v>
+        <v>480</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>468</v>
+        <v>481</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>469</v>
+        <v>482</v>
       </c>
       <c r="F1" s="16" t="s">
-        <v>470</v>
+        <v>483</v>
       </c>
       <c r="G1" s="16" t="s">
-        <v>471</v>
+        <v>484</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
-        <v>472</v>
+        <v>485</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>473</v>
+        <v>486</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>474</v>
+        <v>487</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>475</v>
+        <v>488</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>476</v>
+        <v>489</v>
       </c>
       <c r="F2" s="17" t="s">
-        <v>477</v>
+        <v>490</v>
       </c>
       <c r="G2" s="17" t="s">
-        <v>478</v>
+        <v>491</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
-        <v>479</v>
+        <v>492</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>480</v>
+        <v>493</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>481</v>
+        <v>494</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>475</v>
+        <v>488</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>482</v>
+        <v>495</v>
       </c>
       <c r="F3" s="17" t="s">
-        <v>483</v>
+        <v>496</v>
       </c>
       <c r="G3" s="17" t="s">
-        <v>478</v>
+        <v>491</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>484</v>
+        <v>497</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>485</v>
+        <v>498</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>486</v>
+        <v>499</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>475</v>
+        <v>488</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>487</v>
+        <v>500</v>
       </c>
       <c r="F4" s="17" t="s">
-        <v>488</v>
+        <v>501</v>
       </c>
       <c r="G4" s="17" t="s">
-        <v>478</v>
+        <v>491</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>489</v>
+        <v>502</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>490</v>
+        <v>503</v>
       </c>
       <c r="C5" s="17" t="s">
+        <v>504</v>
+      </c>
+      <c r="D5" s="17" t="s">
+        <v>505</v>
+      </c>
+      <c r="E5" s="17" t="s">
+        <v>506</v>
+      </c>
+      <c r="F5" s="17" t="s">
+        <v>507</v>
+      </c>
+      <c r="G5" s="17" t="s">
         <v>491</v>
-      </c>
-      <c r="D5" s="17" t="s">
-        <v>492</v>
-      </c>
-      <c r="E5" s="17" t="s">
-        <v>493</v>
-      </c>
-      <c r="F5" s="17" t="s">
-        <v>494</v>
-      </c>
-      <c r="G5" s="17" t="s">
-        <v>478</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
-        <v>495</v>
+        <v>508</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>480</v>
+        <v>493</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>496</v>
+        <v>509</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>475</v>
+        <v>488</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>497</v>
+        <v>510</v>
       </c>
       <c r="F6" s="17" t="s">
         <v>131</v>
       </c>
       <c r="G6" s="17" t="s">
-        <v>478</v>
+        <v>491</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
+        <v>511</v>
+      </c>
+      <c r="B7" s="17" t="s">
         <v>498</v>
       </c>
-      <c r="B7" s="17" t="s">
-        <v>485</v>
-      </c>
       <c r="C7" s="17" t="s">
-        <v>499</v>
+        <v>512</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>475</v>
+        <v>488</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>500</v>
+        <v>513</v>
       </c>
       <c r="F7" s="17" t="s">
         <v>131</v>
       </c>
       <c r="G7" s="17" t="s">
-        <v>478</v>
+        <v>491</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
-        <v>501</v>
+        <v>514</v>
       </c>
       <c r="B8" s="17" t="s">
         <v>121</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>502</v>
+        <v>515</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>503</v>
+        <v>516</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>493</v>
+        <v>506</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>504</v>
+        <v>517</v>
       </c>
       <c r="G8" s="17" t="s">
-        <v>478</v>
+        <v>491</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A9" s="17" t="s">
-        <v>505</v>
+        <v>518</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>506</v>
+        <v>519</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>507</v>
+        <v>520</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>508</v>
+        <v>521</v>
       </c>
       <c r="E9" s="17" t="s">
-        <v>509</v>
+        <v>522</v>
       </c>
       <c r="F9" s="17" t="s">
-        <v>510</v>
+        <v>523</v>
       </c>
       <c r="G9" s="17" t="s">
-        <v>478</v>
+        <v>491</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="17" t="s">
-        <v>511</v>
+        <v>524</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>480</v>
+        <v>493</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>496</v>
+        <v>509</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>475</v>
+        <v>488</v>
       </c>
       <c r="E10" s="17" t="s">
-        <v>512</v>
+        <v>525</v>
       </c>
       <c r="F10" s="17" t="s">
         <v>139</v>
       </c>
       <c r="G10" s="17" t="s">
-        <v>513</v>
+        <v>526</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A11" s="17" t="s">
-        <v>514</v>
+        <v>527</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>485</v>
+        <v>498</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>515</v>
+        <v>528</v>
       </c>
       <c r="D11" s="17" t="s">
-        <v>516</v>
+        <v>529</v>
       </c>
       <c r="E11" s="17" t="s">
-        <v>517</v>
+        <v>530</v>
       </c>
       <c r="F11" s="17" t="s">
         <v>139</v>
       </c>
       <c r="G11" s="17" t="s">
-        <v>513</v>
+        <v>526</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
-        <v>518</v>
+        <v>531</v>
       </c>
       <c r="B12" s="17" t="s">
         <v>121</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>519</v>
+        <v>532</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>503</v>
+        <v>516</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>520</v>
+        <v>533</v>
       </c>
       <c r="F12" s="17" t="s">
-        <v>504</v>
+        <v>517</v>
       </c>
       <c r="G12" s="17" t="s">
-        <v>513</v>
+        <v>526</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A13" s="17" t="s">
+        <v>534</v>
+      </c>
+      <c r="B13" s="17" t="s">
+        <v>519</v>
+      </c>
+      <c r="C13" s="17" t="s">
+        <v>520</v>
+      </c>
+      <c r="D13" s="17" t="s">
         <v>521</v>
       </c>
-      <c r="B13" s="17" t="s">
-        <v>506</v>
-      </c>
-      <c r="C13" s="17" t="s">
-        <v>507</v>
-      </c>
-      <c r="D13" s="17" t="s">
-        <v>508</v>
-      </c>
       <c r="E13" s="17" t="s">
-        <v>522</v>
+        <v>535</v>
       </c>
       <c r="F13" s="17" t="s">
-        <v>523</v>
+        <v>536</v>
       </c>
       <c r="G13" s="17" t="s">
-        <v>513</v>
+        <v>526</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="51" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
-        <v>524</v>
+        <v>537</v>
       </c>
       <c r="B14" s="17" t="s">
-        <v>473</v>
+        <v>486</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>525</v>
+        <v>538</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>475</v>
+        <v>488</v>
       </c>
       <c r="E14" s="17" t="s">
+        <v>539</v>
+      </c>
+      <c r="F14" s="17" t="s">
+        <v>540</v>
+      </c>
+      <c r="G14" s="17" t="s">
         <v>526</v>
-      </c>
-      <c r="F14" s="17" t="s">
-        <v>527</v>
-      </c>
-      <c r="G14" s="17" t="s">
-        <v>513</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A15" s="17" t="s">
-        <v>528</v>
+        <v>541</v>
       </c>
       <c r="B15" s="17" t="s">
-        <v>480</v>
+        <v>493</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>529</v>
+        <v>542</v>
       </c>
       <c r="D15" s="17" t="s">
-        <v>475</v>
+        <v>488</v>
       </c>
       <c r="E15" s="17" t="s">
-        <v>530</v>
+        <v>543</v>
       </c>
       <c r="F15" s="17" t="s">
-        <v>531</v>
+        <v>544</v>
       </c>
       <c r="G15" s="17" t="s">
-        <v>513</v>
+        <v>526</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A16" s="17" t="s">
-        <v>532</v>
+        <v>545</v>
       </c>
       <c r="B16" s="17" t="s">
-        <v>485</v>
+        <v>498</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>533</v>
+        <v>546</v>
       </c>
       <c r="D16" s="17" t="s">
-        <v>475</v>
+        <v>488</v>
       </c>
       <c r="E16" s="17" t="s">
-        <v>534</v>
+        <v>547</v>
       </c>
       <c r="F16" s="17" t="s">
-        <v>535</v>
+        <v>548</v>
       </c>
       <c r="G16" s="17" t="s">
-        <v>513</v>
+        <v>526</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="51" x14ac:dyDescent="0.25">
       <c r="A17" s="17" t="s">
-        <v>536</v>
+        <v>549</v>
       </c>
       <c r="B17" s="17" t="s">
-        <v>537</v>
+        <v>550</v>
       </c>
       <c r="C17" s="17" t="s">
-        <v>538</v>
+        <v>551</v>
       </c>
       <c r="D17" s="17" t="s">
-        <v>503</v>
+        <v>516</v>
       </c>
       <c r="E17" s="17" t="s">
-        <v>539</v>
+        <v>552</v>
       </c>
       <c r="F17" s="17" t="s">
-        <v>540</v>
+        <v>553</v>
       </c>
       <c r="G17" s="17" t="s">
-        <v>513</v>
+        <v>526</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A18" s="17" t="s">
-        <v>541</v>
+        <v>554</v>
       </c>
       <c r="B18" s="17" t="s">
-        <v>480</v>
+        <v>493</v>
       </c>
       <c r="C18" s="17" t="s">
-        <v>542</v>
+        <v>555</v>
       </c>
       <c r="D18" s="17" t="s">
-        <v>475</v>
+        <v>488</v>
       </c>
       <c r="E18" s="17" t="s">
-        <v>543</v>
+        <v>556</v>
       </c>
       <c r="F18" s="17" t="s">
-        <v>544</v>
+        <v>557</v>
       </c>
       <c r="G18" s="17" t="s">
-        <v>513</v>
+        <v>526</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="51" x14ac:dyDescent="0.25">
       <c r="A19" s="17" t="s">
-        <v>545</v>
+        <v>558</v>
       </c>
       <c r="B19" s="17" t="s">
-        <v>485</v>
+        <v>498</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>546</v>
+        <v>559</v>
       </c>
       <c r="D19" s="17" t="s">
-        <v>475</v>
+        <v>488</v>
       </c>
       <c r="E19" s="17" t="s">
-        <v>547</v>
+        <v>560</v>
       </c>
       <c r="F19" s="17" t="s">
-        <v>535</v>
+        <v>548</v>
       </c>
       <c r="G19" s="17" t="s">
-        <v>513</v>
+        <v>526</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A20" s="17" t="s">
-        <v>548</v>
+        <v>561</v>
       </c>
       <c r="B20" s="17" t="s">
-        <v>537</v>
+        <v>550</v>
       </c>
       <c r="C20" s="17" t="s">
-        <v>549</v>
+        <v>562</v>
       </c>
       <c r="D20" s="17" t="s">
-        <v>503</v>
+        <v>516</v>
       </c>
       <c r="E20" s="17" t="s">
-        <v>550</v>
+        <v>563</v>
       </c>
       <c r="F20" s="17" t="s">
-        <v>551</v>
+        <v>564</v>
       </c>
       <c r="G20" s="17" t="s">
-        <v>513</v>
+        <v>526</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A21" s="17" t="s">
-        <v>552</v>
+        <v>565</v>
       </c>
       <c r="B21" s="17" t="s">
-        <v>480</v>
+        <v>493</v>
       </c>
       <c r="C21" s="17" t="s">
-        <v>553</v>
+        <v>566</v>
       </c>
       <c r="D21" s="17" t="s">
-        <v>475</v>
+        <v>488</v>
       </c>
       <c r="E21" s="17" t="s">
-        <v>554</v>
+        <v>567</v>
       </c>
       <c r="F21" s="17" t="s">
-        <v>544</v>
+        <v>557</v>
       </c>
       <c r="G21" s="17" t="s">
-        <v>513</v>
+        <v>526</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A22" s="17" t="s">
-        <v>555</v>
+        <v>568</v>
       </c>
       <c r="B22" s="17" t="s">
-        <v>485</v>
+        <v>498</v>
       </c>
       <c r="C22" s="17" t="s">
-        <v>556</v>
+        <v>569</v>
       </c>
       <c r="D22" s="17" t="s">
-        <v>475</v>
+        <v>488</v>
       </c>
       <c r="E22" s="17" t="s">
-        <v>534</v>
+        <v>547</v>
       </c>
       <c r="F22" s="17" t="s">
-        <v>535</v>
+        <v>548</v>
       </c>
       <c r="G22" s="17" t="s">
-        <v>513</v>
+        <v>526</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A23" s="17" t="s">
-        <v>557</v>
+        <v>570</v>
       </c>
       <c r="B23" s="17" t="s">
-        <v>537</v>
+        <v>550</v>
       </c>
       <c r="C23" s="17" t="s">
-        <v>558</v>
+        <v>571</v>
       </c>
       <c r="D23" s="17" t="s">
-        <v>503</v>
+        <v>516</v>
       </c>
       <c r="E23" s="17" t="s">
-        <v>559</v>
+        <v>572</v>
       </c>
       <c r="F23" s="17" t="s">
-        <v>560</v>
+        <v>573</v>
       </c>
       <c r="G23" s="17" t="s">
-        <v>513</v>
+        <v>526</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A24" s="17" t="s">
-        <v>561</v>
+        <v>574</v>
       </c>
       <c r="B24" s="17" t="s">
-        <v>473</v>
+        <v>486</v>
       </c>
       <c r="C24" s="17" t="s">
-        <v>562</v>
+        <v>575</v>
       </c>
       <c r="D24" s="17" t="s">
-        <v>475</v>
+        <v>488</v>
       </c>
       <c r="E24" s="17" t="s">
-        <v>563</v>
+        <v>576</v>
       </c>
       <c r="F24" s="17" t="s">
-        <v>564</v>
+        <v>577</v>
       </c>
       <c r="G24" s="17" t="s">
-        <v>513</v>
+        <v>526</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="17" t="s">
-        <v>565</v>
+        <v>578</v>
       </c>
       <c r="B25" s="17" t="s">
-        <v>480</v>
+        <v>493</v>
       </c>
       <c r="C25" s="17" t="s">
-        <v>566</v>
+        <v>579</v>
       </c>
       <c r="D25" s="17" t="s">
-        <v>475</v>
+        <v>488</v>
       </c>
       <c r="E25" s="17" t="s">
-        <v>567</v>
+        <v>580</v>
       </c>
       <c r="F25" s="17" t="s">
-        <v>544</v>
+        <v>557</v>
       </c>
       <c r="G25" s="17" t="s">
-        <v>513</v>
+        <v>526</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A26" s="17" t="s">
-        <v>568</v>
+        <v>581</v>
       </c>
       <c r="B26" s="17" t="s">
-        <v>485</v>
+        <v>498</v>
       </c>
       <c r="C26" s="17" t="s">
-        <v>569</v>
+        <v>582</v>
       </c>
       <c r="D26" s="17" t="s">
-        <v>475</v>
+        <v>488</v>
       </c>
       <c r="E26" s="17" t="s">
-        <v>570</v>
+        <v>583</v>
       </c>
       <c r="F26" s="17" t="s">
-        <v>535</v>
+        <v>548</v>
       </c>
       <c r="G26" s="17" t="s">
-        <v>513</v>
+        <v>526</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A27" s="17" t="s">
-        <v>571</v>
+        <v>584</v>
       </c>
       <c r="B27" s="17" t="s">
-        <v>537</v>
+        <v>550</v>
       </c>
       <c r="C27" s="17" t="s">
-        <v>572</v>
+        <v>585</v>
       </c>
       <c r="D27" s="17" t="s">
-        <v>503</v>
+        <v>516</v>
       </c>
       <c r="E27" s="17" t="s">
-        <v>573</v>
+        <v>586</v>
       </c>
       <c r="F27" s="17" t="s">
-        <v>574</v>
+        <v>587</v>
       </c>
       <c r="G27" s="17" t="s">
-        <v>513</v>
+        <v>526</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A28" s="17" t="s">
-        <v>575</v>
+        <v>588</v>
       </c>
       <c r="B28" s="17" t="s">
-        <v>485</v>
+        <v>498</v>
       </c>
       <c r="C28" s="17" t="s">
-        <v>576</v>
+        <v>589</v>
       </c>
       <c r="D28" s="17" t="s">
-        <v>577</v>
+        <v>590</v>
       </c>
       <c r="E28" s="17" t="s">
-        <v>578</v>
+        <v>591</v>
       </c>
       <c r="F28" s="17" t="s">
-        <v>579</v>
+        <v>592</v>
       </c>
       <c r="G28" s="17" t="s">
         <v>86</v>
@@ -6383,45 +6506,45 @@
     </row>
     <row r="29" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A29" s="17" t="s">
-        <v>580</v>
+        <v>593</v>
       </c>
       <c r="B29" s="17" t="s">
-        <v>485</v>
+        <v>498</v>
       </c>
       <c r="C29" s="17" t="s">
-        <v>581</v>
+        <v>594</v>
       </c>
       <c r="D29" s="17" t="s">
-        <v>503</v>
+        <v>516</v>
       </c>
       <c r="E29" s="17" t="s">
-        <v>582</v>
+        <v>595</v>
       </c>
       <c r="F29" s="17" t="s">
-        <v>535</v>
+        <v>548</v>
       </c>
       <c r="G29" s="17" t="s">
-        <v>513</v>
+        <v>526</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A30" s="17" t="s">
-        <v>583</v>
+        <v>596</v>
       </c>
       <c r="B30" s="17" t="s">
-        <v>584</v>
+        <v>597</v>
       </c>
       <c r="C30" s="17" t="s">
-        <v>585</v>
+        <v>598</v>
       </c>
       <c r="D30" s="17" t="s">
-        <v>475</v>
+        <v>488</v>
       </c>
       <c r="E30" s="17" t="s">
-        <v>586</v>
+        <v>599</v>
       </c>
       <c r="F30" s="17" t="s">
-        <v>544</v>
+        <v>557</v>
       </c>
       <c r="G30" s="17" t="s">
         <v>86</v>
@@ -6429,45 +6552,45 @@
     </row>
     <row r="31" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A31" s="17" t="s">
-        <v>587</v>
+        <v>600</v>
       </c>
       <c r="B31" s="17" t="s">
-        <v>473</v>
+        <v>486</v>
       </c>
       <c r="C31" s="17" t="s">
-        <v>588</v>
+        <v>601</v>
       </c>
       <c r="D31" s="17" t="s">
-        <v>589</v>
+        <v>602</v>
       </c>
       <c r="E31" s="17" t="s">
-        <v>590</v>
+        <v>603</v>
       </c>
       <c r="F31" s="17" t="s">
-        <v>591</v>
+        <v>604</v>
       </c>
       <c r="G31" s="17" t="s">
-        <v>513</v>
+        <v>526</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A32" s="17" t="s">
-        <v>592</v>
+        <v>605</v>
       </c>
       <c r="B32" s="17" t="s">
-        <v>537</v>
+        <v>550</v>
       </c>
       <c r="C32" s="17" t="s">
-        <v>593</v>
+        <v>606</v>
       </c>
       <c r="D32" s="17" t="s">
-        <v>594</v>
+        <v>607</v>
       </c>
       <c r="E32" s="17" t="s">
-        <v>595</v>
+        <v>608</v>
       </c>
       <c r="F32" s="17" t="s">
-        <v>596</v>
+        <v>609</v>
       </c>
       <c r="G32" s="17" t="s">
         <v>86</v>
@@ -6475,22 +6598,22 @@
     </row>
     <row r="33" spans="1:7" ht="51" x14ac:dyDescent="0.25">
       <c r="A33" s="17" t="s">
-        <v>597</v>
+        <v>610</v>
       </c>
       <c r="B33" s="17" t="s">
-        <v>598</v>
+        <v>611</v>
       </c>
       <c r="C33" s="17" t="s">
-        <v>599</v>
+        <v>612</v>
       </c>
       <c r="D33" s="17" t="s">
-        <v>600</v>
+        <v>613</v>
       </c>
       <c r="E33" s="17" t="s">
-        <v>493</v>
+        <v>506</v>
       </c>
       <c r="F33" s="17" t="s">
-        <v>601</v>
+        <v>614</v>
       </c>
       <c r="G33" s="17" t="s">
         <v>86</v>
@@ -6498,22 +6621,22 @@
     </row>
     <row r="34" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A34" s="17" t="s">
-        <v>602</v>
+        <v>615</v>
       </c>
       <c r="B34" s="17" t="s">
-        <v>473</v>
+        <v>486</v>
       </c>
       <c r="C34" s="17" t="s">
-        <v>603</v>
+        <v>616</v>
       </c>
       <c r="D34" s="17" t="s">
-        <v>475</v>
+        <v>488</v>
       </c>
       <c r="E34" s="17" t="s">
-        <v>604</v>
+        <v>617</v>
       </c>
       <c r="F34" s="17" t="s">
-        <v>605</v>
+        <v>618</v>
       </c>
       <c r="G34" s="17" t="s">
         <v>86</v>
@@ -6521,22 +6644,22 @@
     </row>
     <row r="35" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A35" s="17" t="s">
-        <v>606</v>
+        <v>619</v>
       </c>
       <c r="B35" s="17" t="s">
-        <v>473</v>
+        <v>486</v>
       </c>
       <c r="C35" s="17" t="s">
-        <v>607</v>
+        <v>620</v>
       </c>
       <c r="D35" s="17" t="s">
-        <v>475</v>
+        <v>488</v>
       </c>
       <c r="E35" s="17" t="s">
-        <v>608</v>
+        <v>621</v>
       </c>
       <c r="F35" s="17" t="s">
-        <v>609</v>
+        <v>622</v>
       </c>
       <c r="G35" s="17" t="s">
         <v>86</v>
@@ -6544,22 +6667,22 @@
     </row>
     <row r="36" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A36" s="17" t="s">
-        <v>610</v>
+        <v>623</v>
       </c>
       <c r="B36" s="17" t="s">
-        <v>485</v>
+        <v>498</v>
       </c>
       <c r="C36" s="17" t="s">
-        <v>611</v>
+        <v>624</v>
       </c>
       <c r="D36" s="17" t="s">
-        <v>503</v>
+        <v>516</v>
       </c>
       <c r="E36" s="17" t="s">
-        <v>612</v>
+        <v>625</v>
       </c>
       <c r="F36" s="17" t="s">
-        <v>613</v>
+        <v>626</v>
       </c>
       <c r="G36" s="17" t="s">
         <v>86</v>
@@ -6567,29 +6690,75 @@
     </row>
     <row r="37" spans="1:7" ht="51" x14ac:dyDescent="0.25">
       <c r="A37" s="17" t="s">
-        <v>614</v>
+        <v>627</v>
       </c>
       <c r="B37" s="17" t="s">
-        <v>615</v>
+        <v>628</v>
       </c>
       <c r="C37" s="17" t="s">
-        <v>616</v>
+        <v>629</v>
       </c>
       <c r="D37" s="17" t="s">
-        <v>617</v>
+        <v>630</v>
       </c>
       <c r="E37" s="17" t="s">
-        <v>618</v>
+        <v>631</v>
       </c>
       <c r="F37" s="17" t="s">
-        <v>619</v>
+        <v>632</v>
       </c>
       <c r="G37" s="17" t="s">
         <v>86</v>
       </c>
     </row>
+    <row r="38" spans="1:7" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A38" s="17" t="s">
+        <v>633</v>
+      </c>
+      <c r="B38" s="17" t="s">
+        <v>634</v>
+      </c>
+      <c r="C38" s="17" t="s">
+        <v>635</v>
+      </c>
+      <c r="D38" s="17" t="s">
+        <v>636</v>
+      </c>
+      <c r="E38" s="17" t="s">
+        <v>506</v>
+      </c>
+      <c r="F38" s="17" t="s">
+        <v>637</v>
+      </c>
+      <c r="G38" s="17" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A39" s="17" t="s">
+        <v>638</v>
+      </c>
+      <c r="B39" s="17" t="s">
+        <v>634</v>
+      </c>
+      <c r="C39" s="17" t="s">
+        <v>639</v>
+      </c>
+      <c r="D39" s="17" t="s">
+        <v>640</v>
+      </c>
+      <c r="E39" s="17" t="s">
+        <v>641</v>
+      </c>
+      <c r="F39" s="17" t="s">
+        <v>642</v>
+      </c>
+      <c r="G39" s="17" t="s">
+        <v>86</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G37" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
+  <autoFilter ref="A1:G39" xr:uid="{00000000-0009-0000-0000-000004000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6608,39 +6777,39 @@
   <sheetData>
     <row r="1" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>620</v>
+        <v>643</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>621</v>
+        <v>644</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>622</v>
+        <v>645</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>471</v>
+        <v>484</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>623</v>
+        <v>646</v>
       </c>
       <c r="F1" s="16" t="s">
-        <v>624</v>
+        <v>647</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
-        <v>625</v>
+        <v>648</v>
       </c>
       <c r="B2" s="17" t="s">
         <v>72</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>626</v>
+        <v>649</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>478</v>
+        <v>491</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>627</v>
+        <v>650</v>
       </c>
       <c r="F2" s="17" t="s">
         <v>88</v>
@@ -6648,19 +6817,19 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
-        <v>628</v>
+        <v>651</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>629</v>
+        <v>652</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>630</v>
+        <v>653</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>478</v>
+        <v>491</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>631</v>
+        <v>654</v>
       </c>
       <c r="F3" s="17" t="s">
         <v>88</v>
@@ -6668,39 +6837,39 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>632</v>
+        <v>655</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>633</v>
+        <v>656</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>634</v>
+        <v>657</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>478</v>
+        <v>491</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>635</v>
+        <v>658</v>
       </c>
       <c r="F4" s="17" t="s">
-        <v>636</v>
+        <v>659</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>637</v>
+        <v>660</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>638</v>
+        <v>661</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>639</v>
+        <v>662</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>478</v>
+        <v>491</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>640</v>
+        <v>663</v>
       </c>
       <c r="F5" s="17" t="s">
         <v>166</v>
@@ -6708,16 +6877,16 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
-        <v>641</v>
+        <v>664</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>642</v>
+        <v>665</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>643</v>
+        <v>666</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>478</v>
+        <v>491</v>
       </c>
       <c r="E6" s="17" t="s">
         <v>26</v>
@@ -6728,19 +6897,19 @@
     </row>
     <row r="7" spans="1:6" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
-        <v>644</v>
+        <v>667</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>645</v>
+        <v>668</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>646</v>
+        <v>669</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>478</v>
+        <v>491</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>647</v>
+        <v>670</v>
       </c>
       <c r="F7" s="17" t="s">
         <v>166</v>
@@ -6748,22 +6917,22 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="17" t="s">
-        <v>648</v>
+        <v>671</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>649</v>
+        <v>672</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>650</v>
+        <v>673</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>478</v>
+        <v>491</v>
       </c>
       <c r="E8" s="17" t="s">
-        <v>651</v>
+        <v>674</v>
       </c>
       <c r="F8" s="17" t="s">
-        <v>652</v>
+        <v>675</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -6771,16 +6940,16 @@
         <v>178</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>653</v>
+        <v>676</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>654</v>
+        <v>677</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>478</v>
+        <v>491</v>
       </c>
       <c r="E9" s="17" t="s">
-        <v>651</v>
+        <v>674</v>
       </c>
       <c r="F9" s="17" t="s">
         <v>173</v>
@@ -6788,16 +6957,16 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="17" t="s">
-        <v>655</v>
+        <v>678</v>
       </c>
       <c r="B10" s="17" t="s">
         <v>52</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>656</v>
+        <v>679</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>478</v>
+        <v>491</v>
       </c>
       <c r="E10" s="17" t="s">
         <v>51</v>
@@ -6808,93 +6977,93 @@
     </row>
     <row r="11" spans="1:6" ht="51" x14ac:dyDescent="0.25">
       <c r="A11" s="17" t="s">
-        <v>657</v>
+        <v>680</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>658</v>
+        <v>681</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>659</v>
+        <v>682</v>
       </c>
       <c r="D11" s="17" t="s">
-        <v>513</v>
+        <v>526</v>
       </c>
       <c r="E11" s="17" t="s">
-        <v>660</v>
+        <v>683</v>
       </c>
       <c r="F11" s="17" t="s">
-        <v>661</v>
+        <v>684</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="17" t="s">
-        <v>662</v>
+        <v>685</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>663</v>
+        <v>686</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>664</v>
+        <v>687</v>
       </c>
       <c r="D12" s="17" t="s">
-        <v>478</v>
+        <v>491</v>
       </c>
       <c r="E12" s="17" t="s">
-        <v>665</v>
+        <v>688</v>
       </c>
       <c r="F12" s="17" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="51" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A13" s="17" t="s">
-        <v>666</v>
+        <v>689</v>
       </c>
       <c r="B13" s="17" t="s">
-        <v>667</v>
+        <v>690</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>668</v>
+        <v>691</v>
       </c>
       <c r="D13" s="17" t="s">
-        <v>513</v>
+        <v>526</v>
       </c>
       <c r="E13" s="17" t="s">
-        <v>669</v>
+        <v>692</v>
       </c>
       <c r="F13" s="17" t="s">
-        <v>670</v>
+        <v>693</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="51" x14ac:dyDescent="0.25">
       <c r="A14" s="17" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B14" s="17" t="s">
-        <v>671</v>
+        <v>694</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>672</v>
+        <v>695</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>513</v>
+        <v>526</v>
       </c>
       <c r="E14" s="17" t="s">
-        <v>673</v>
+        <v>696</v>
       </c>
       <c r="F14" s="17" t="s">
-        <v>674</v>
+        <v>697</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="51" x14ac:dyDescent="0.25">
       <c r="A15" s="17" t="s">
-        <v>675</v>
+        <v>698</v>
       </c>
       <c r="B15" s="17" t="s">
-        <v>676</v>
+        <v>699</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>677</v>
+        <v>700</v>
       </c>
       <c r="D15" s="17" t="s">
         <v>86</v>
@@ -6903,7 +7072,7 @@
         <v>60</v>
       </c>
       <c r="F15" s="17" t="s">
-        <v>678</v>
+        <v>701</v>
       </c>
     </row>
   </sheetData>
@@ -6926,121 +7095,121 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>679</v>
+        <v>702</v>
       </c>
       <c r="B1" s="16" t="s">
-        <v>680</v>
+        <v>703</v>
       </c>
       <c r="C1" s="16" t="s">
-        <v>681</v>
+        <v>704</v>
       </c>
       <c r="D1" s="16" t="s">
-        <v>682</v>
+        <v>705</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>683</v>
+        <v>706</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
-        <v>684</v>
+        <v>707</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>685</v>
+        <v>708</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>686</v>
+        <v>709</v>
       </c>
       <c r="D2" s="17" t="s">
-        <v>687</v>
+        <v>710</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>688</v>
+        <v>711</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
-        <v>689</v>
+        <v>712</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>690</v>
+        <v>713</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>691</v>
+        <v>714</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>692</v>
+        <v>715</v>
       </c>
       <c r="E3" s="17" t="s">
-        <v>693</v>
+        <v>716</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>694</v>
+        <v>717</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>695</v>
+        <v>718</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>695</v>
+        <v>718</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>696</v>
+        <v>719</v>
       </c>
       <c r="E4" s="17" t="s">
-        <v>697</v>
+        <v>720</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>698</v>
+        <v>721</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>699</v>
+        <v>722</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>700</v>
+        <v>723</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>701</v>
+        <v>724</v>
       </c>
       <c r="E5" s="17" t="s">
-        <v>693</v>
+        <v>716</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="17" t="s">
-        <v>702</v>
+        <v>725</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>703</v>
+        <v>726</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>703</v>
+        <v>726</v>
       </c>
       <c r="D6" s="17" t="s">
-        <v>704</v>
+        <v>727</v>
       </c>
       <c r="E6" s="17" t="s">
-        <v>688</v>
+        <v>711</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A7" s="17" t="s">
-        <v>705</v>
+        <v>728</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>706</v>
+        <v>729</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>707</v>
+        <v>730</v>
       </c>
       <c r="D7" s="17" t="s">
-        <v>708</v>
+        <v>731</v>
       </c>
       <c r="E7" s="17" t="s">
-        <v>688</v>
+        <v>711</v>
       </c>
     </row>
   </sheetData>

</xml_diff>